<commit_message>
Sync catalogue v4: 168 main entries, 11 related works and review history
</commit_message>
<xml_diff>
--- a/downloads/catalogue.xlsx
+++ b/downloads/catalogue.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="目录总览" sheetId="1" r:id="R8139e326e26b4576"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="论文目录" sheetId="2" r:id="R3136048753d54ac4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="边界相关" sheetId="3" r:id="R20a57cace0334d30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="目录总览" sheetId="1" r:id="R211faeb502164b50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="论文目录" sheetId="2" r:id="R8dbbff83562b4659"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="边界相关" sheetId="3" r:id="Re6d7832b0cbb4e02"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -73,12 +73,32 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF243D59"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEDF2F7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF243D59"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEDF2F7"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -151,7 +171,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="59">
+  <x:cellXfs count="79">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -325,11 +345,93 @@
     <x:xf numFmtId="200" fontId="4" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="5" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="5" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="5" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="3">
+  <x:dxfs count="6">
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF795400"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF795400"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
@@ -363,13 +465,24 @@
         </x:patternFill>
       </x:fill>
     </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF795400"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
   </x:dxfs>
 </x:styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MainBibliography" displayName="MainBibliography" ref="A5:Q171" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:Q171"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MainBibliography" displayName="MainBibliography" ref="A5:Q173" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:Q173"/>
   <x:tableColumns count="17">
     <x:tableColumn id="1" name="编号"/>
     <x:tableColumn id="2" name="研究主题"/>
@@ -394,8 +507,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="AdjacentBibliography" displayName="AdjacentBibliography" ref="A5:Q12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:Q12"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="AdjacentBibliography" displayName="AdjacentBibliography" ref="A5:Q16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:Q16"/>
   <x:tableColumns count="17">
     <x:tableColumn id="1" name="编号"/>
     <x:tableColumn id="2" name="研究主题"/>
@@ -676,26 +789,26 @@
       <x:c r="H4" s="2"/>
     </x:row>
     <x:row r="5" ht="29" customHeight="1">
-      <x:c r="A5" s="51" t="str">
+      <x:c r="A5" s="72" t="str">
         <x:v>简称</x:v>
       </x:c>
-      <x:c r="B5" s="52" t="str">
+      <x:c r="B5" s="73" t="str">
         <x:v>期刊</x:v>
       </x:c>
-      <x:c r="C5" s="52" t="str">
+      <x:c r="C5" s="73" t="str">
         <x:v>主目录</x:v>
       </x:c>
-      <x:c r="D5" s="52" t="str">
+      <x:c r="D5" s="73" t="str">
         <x:v>边界相关</x:v>
       </x:c>
-      <x:c r="E5" s="53" t="str">
+      <x:c r="E5" s="74" t="str">
         <x:v>学科</x:v>
       </x:c>
       <x:c r="F5" s="2"/>
-      <x:c r="G5" s="51" t="str">
+      <x:c r="G5" s="72" t="str">
         <x:v>主主题</x:v>
       </x:c>
-      <x:c r="H5" s="53" t="str">
+      <x:c r="H5" s="74" t="str">
         <x:v>篇数</x:v>
       </x:c>
     </x:row>
@@ -707,11 +820,11 @@
         <x:v>American Economic Review</x:v>
       </x:c>
       <x:c r="C6" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$171,A6)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A6)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D6" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$12,A6)</x:f>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A6)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="E6" s="14" t="str">
@@ -722,7 +835,7 @@
         <x:v>货币竞争、加密资产估值与收益</x:v>
       </x:c>
       <x:c r="H6" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$B$6:$B$171,G6)</x:f>
+        <x:f>COUNTIFS('论文目录'!$B$6:$B$173,G6)</x:f>
         <x:v>14</x:v>
       </x:c>
     </x:row>
@@ -734,11 +847,11 @@
         <x:v>Econometrica</x:v>
       </x:c>
       <x:c r="C7" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$171,A7)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A7)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D7" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$12,A7)</x:f>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A7)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E7" s="14" t="str">
@@ -749,7 +862,7 @@
         <x:v>ICO、代币融资与平台经济</x:v>
       </x:c>
       <x:c r="H7" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$B$6:$B$171,G7)</x:f>
+        <x:f>COUNTIFS('论文目录'!$B$6:$B$173,G7)</x:f>
         <x:v>23</x:v>
       </x:c>
     </x:row>
@@ -761,11 +874,11 @@
         <x:v>The Quarterly Journal of Economics</x:v>
       </x:c>
       <x:c r="C8" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$171,A8)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A8)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D8" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$12,A8)</x:f>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A8)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E8" s="14" t="str">
@@ -776,7 +889,7 @@
         <x:v>共识机制、挖矿与去中心化安全</x:v>
       </x:c>
       <x:c r="H8" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$B$6:$B$171,G8)</x:f>
+        <x:f>COUNTIFS('论文目录'!$B$6:$B$173,G8)</x:f>
         <x:v>19</x:v>
       </x:c>
     </x:row>
@@ -788,12 +901,12 @@
         <x:v>Journal of Political Economy</x:v>
       </x:c>
       <x:c r="C9" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$171,A9)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A9)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D9" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$12,A9)</x:f>
-        <x:v>0</x:v>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A9)</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E9" s="14" t="str">
         <x:v>经济学</x:v>
@@ -803,7 +916,7 @@
         <x:v>交易费用、支付与区块链扩容</x:v>
       </x:c>
       <x:c r="H9" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$B$6:$B$171,G9)</x:f>
+        <x:f>COUNTIFS('论文目录'!$B$6:$B$173,G9)</x:f>
         <x:v>11</x:v>
       </x:c>
     </x:row>
@@ -815,11 +928,11 @@
         <x:v>The Review of Economic Studies</x:v>
       </x:c>
       <x:c r="C10" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$171,A10)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A10)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D10" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$12,A10)</x:f>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A10)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E10" s="14" t="str">
@@ -830,7 +943,7 @@
         <x:v>交易市场、衍生品与投资者行为</x:v>
       </x:c>
       <x:c r="H10" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$B$6:$B$171,G10)</x:f>
+        <x:f>COUNTIFS('论文目录'!$B$6:$B$173,G10)</x:f>
         <x:v>19</x:v>
       </x:c>
     </x:row>
@@ -842,12 +955,12 @@
         <x:v>Journal of Monetary Economics</x:v>
       </x:c>
       <x:c r="C11" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$171,A11)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A11)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="D11" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$12,A11)</x:f>
-        <x:v>1</x:v>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A11)</x:f>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E11" s="14" t="str">
         <x:v>经济学</x:v>
@@ -857,7 +970,7 @@
         <x:v>去中心化交易所、自动做市与流动性</x:v>
       </x:c>
       <x:c r="H11" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$B$6:$B$171,G11)</x:f>
+        <x:f>COUNTIFS('论文目录'!$B$6:$B$173,G11)</x:f>
         <x:v>13</x:v>
       </x:c>
     </x:row>
@@ -869,11 +982,11 @@
         <x:v>The Review of Financial Studies</x:v>
       </x:c>
       <x:c r="C12" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$171,A12)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A12)</x:f>
         <x:v>19</x:v>
       </x:c>
       <x:c r="D12" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$12,A12)</x:f>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A12)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E12" s="14" t="str">
@@ -884,7 +997,7 @@
         <x:v>稳定币、DeFi 借贷与预测市场</x:v>
       </x:c>
       <x:c r="H12" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$B$6:$B$171,G12)</x:f>
+        <x:f>COUNTIFS('论文目录'!$B$6:$B$173,G12)</x:f>
         <x:v>8</x:v>
       </x:c>
     </x:row>
@@ -896,12 +1009,12 @@
         <x:v>Journal of Financial Economics</x:v>
       </x:c>
       <x:c r="C13" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$171,A13)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A13)</x:f>
         <x:v>13</x:v>
       </x:c>
       <x:c r="D13" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$12,A13)</x:f>
-        <x:v>0</x:v>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A13)</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E13" s="14" t="str">
         <x:v>金融学</x:v>
@@ -911,8 +1024,8 @@
         <x:v>智能合约、DAO、社区与制度治理</x:v>
       </x:c>
       <x:c r="H13" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$B$6:$B$171,G13)</x:f>
-        <x:v>18</x:v>
+        <x:f>COUNTIFS('论文目录'!$B$6:$B$173,G13)</x:f>
+        <x:v>20</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="26" customHeight="1">
@@ -923,11 +1036,11 @@
         <x:v>The Journal of Finance</x:v>
       </x:c>
       <x:c r="C14" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$171,A14)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A14)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="D14" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$12,A14)</x:f>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A14)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E14" s="14" t="str">
@@ -938,7 +1051,7 @@
         <x:v>企业披露、财务会计与审计</x:v>
       </x:c>
       <x:c r="H14" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$B$6:$B$171,G14)</x:f>
+        <x:f>COUNTIFS('论文目录'!$B$6:$B$173,G14)</x:f>
         <x:v>11</x:v>
       </x:c>
     </x:row>
@@ -950,11 +1063,11 @@
         <x:v>Mathematical Finance</x:v>
       </x:c>
       <x:c r="C15" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$171,A15)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A15)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="D15" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$12,A15)</x:f>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A15)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E15" s="14" t="str">
@@ -965,7 +1078,7 @@
         <x:v>市场操纵、非法活动、网络犯罪与税收</x:v>
       </x:c>
       <x:c r="H15" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$B$6:$B$171,G15)</x:f>
+        <x:f>COUNTIFS('论文目录'!$B$6:$B$173,G15)</x:f>
         <x:v>11</x:v>
       </x:c>
     </x:row>
@@ -977,11 +1090,11 @@
         <x:v>Finance and Stochastics</x:v>
       </x:c>
       <x:c r="C16" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$171,A16)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A16)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D16" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$12,A16)</x:f>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A16)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E16" s="14" t="str">
@@ -992,7 +1105,7 @@
         <x:v>供应链、企业应用与金融包容</x:v>
       </x:c>
       <x:c r="H16" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$B$6:$B$171,G16)</x:f>
+        <x:f>COUNTIFS('论文目录'!$B$6:$B$173,G16)</x:f>
         <x:v>11</x:v>
       </x:c>
     </x:row>
@@ -1004,11 +1117,11 @@
         <x:v>SIAM Journal on Financial Mathematics</x:v>
       </x:c>
       <x:c r="C17" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$171,A17)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A17)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="D17" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$12,A17)</x:f>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A17)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E17" s="14" t="str">
@@ -1019,7 +1132,7 @@
         <x:v>NFT、艺术品与创作者经济</x:v>
       </x:c>
       <x:c r="H17" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$B$6:$B$171,G17)</x:f>
+        <x:f>COUNTIFS('论文目录'!$B$6:$B$173,G17)</x:f>
         <x:v>7</x:v>
       </x:c>
     </x:row>
@@ -1031,12 +1144,12 @@
         <x:v>Management Science</x:v>
       </x:c>
       <x:c r="C18" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$171,A18)</x:f>
-        <x:v>67</x:v>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A18)</x:f>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="D18" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$12,A18)</x:f>
-        <x:v>2</x:v>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A18)</x:f>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E18" s="14" t="str">
         <x:v>管理科学</x:v>
@@ -1046,7 +1159,7 @@
         <x:v>综述与研究议程</x:v>
       </x:c>
       <x:c r="H18" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$B$6:$B$171,G18)</x:f>
+        <x:f>COUNTIFS('论文目录'!$B$6:$B$173,G18)</x:f>
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -1058,23 +1171,23 @@
         <x:v>Operations Research</x:v>
       </x:c>
       <x:c r="C19" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$171,A19)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A19)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="D19" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$12,A19)</x:f>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A19)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E19" s="14" t="str">
         <x:v>管理科学</x:v>
       </x:c>
       <x:c r="F19" s="2"/>
-      <x:c r="G19" s="55" t="str">
+      <x:c r="G19" s="75" t="str">
         <x:v>主题合计</x:v>
       </x:c>
-      <x:c r="H19" s="56" t="n">
+      <x:c r="H19" s="76" t="n">
         <x:f>SUM(H6:H18)</x:f>
-        <x:v>166</x:v>
+        <x:v>168</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="26" customHeight="1">
@@ -1085,11 +1198,11 @@
         <x:v>Information Systems Research</x:v>
       </x:c>
       <x:c r="C20" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$171,A20)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A20)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="D20" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$12,A20)</x:f>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A20)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="E20" s="14" t="str">
@@ -1107,21 +1220,21 @@
         <x:v>MIS Quarterly</x:v>
       </x:c>
       <x:c r="C21" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$171,A21)</x:f>
-        <x:v>9</x:v>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A21)</x:f>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D21" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$12,A21)</x:f>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A21)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E21" s="14" t="str">
         <x:v>信息系统</x:v>
       </x:c>
       <x:c r="F21" s="2"/>
-      <x:c r="G21" s="51" t="str">
+      <x:c r="G21" s="72" t="str">
         <x:v>主目录发表状态</x:v>
       </x:c>
-      <x:c r="H21" s="58" t="str">
+      <x:c r="H21" s="78" t="str">
         <x:v>篇数</x:v>
       </x:c>
     </x:row>
@@ -1133,11 +1246,11 @@
         <x:v>Journal of Accounting and Economics</x:v>
       </x:c>
       <x:c r="C22" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$171,A22)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A22)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="D22" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$12,A22)</x:f>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A22)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E22" s="14" t="str">
@@ -1148,8 +1261,8 @@
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="H22" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$H$6:$H$171,G22)</x:f>
-        <x:v>142</x:v>
+        <x:f>COUNTIFS('论文目录'!$H$6:$H$173,G22)</x:f>
+        <x:v>144</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="26" customHeight="1">
@@ -1160,11 +1273,11 @@
         <x:v>Journal of Accounting Research</x:v>
       </x:c>
       <x:c r="C23" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$171,A23)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A23)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="D23" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$12,A23)</x:f>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A23)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E23" s="14" t="str">
@@ -1175,7 +1288,7 @@
         <x:v>在线发表</x:v>
       </x:c>
       <x:c r="H23" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$H$6:$H$171,G23)</x:f>
+        <x:f>COUNTIFS('论文目录'!$H$6:$H$173,G23)</x:f>
         <x:v>22</x:v>
       </x:c>
     </x:row>
@@ -1187,11 +1300,11 @@
         <x:v>The Accounting Review</x:v>
       </x:c>
       <x:c r="C24" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$171,A24)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A24)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D24" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$12,A24)</x:f>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A24)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="E24" s="14" t="str">
@@ -1202,31 +1315,31 @@
         <x:v>已接收</x:v>
       </x:c>
       <x:c r="H24" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$H$6:$H$171,G24)</x:f>
+        <x:f>COUNTIFS('论文目录'!$H$6:$H$173,G24)</x:f>
         <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="26" customHeight="1">
-      <x:c r="A25" s="55" t="str">
+      <x:c r="A25" s="75" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B25" s="55"/>
-      <x:c r="C25" s="56" t="n">
+      <x:c r="B25" s="75"/>
+      <x:c r="C25" s="76" t="n">
         <x:f>SUM(C6:C24)</x:f>
-        <x:v>166</x:v>
-      </x:c>
-      <x:c r="D25" s="56" t="n">
+        <x:v>168</x:v>
+      </x:c>
+      <x:c r="D25" s="76" t="n">
         <x:f>SUM(D6:D24)</x:f>
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="E25" s="55"/>
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E25" s="75"/>
       <x:c r="F25" s="2"/>
-      <x:c r="G25" s="55" t="str">
+      <x:c r="G25" s="75" t="str">
         <x:v>状态合计</x:v>
       </x:c>
-      <x:c r="H25" s="56" t="n">
+      <x:c r="H25" s="76" t="n">
         <x:f>SUM(H22:H24)</x:f>
-        <x:v>166</x:v>
+        <x:v>168</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="20" customHeight="1">
@@ -1374,7 +1487,7 @@
         <x:v>题录覆盖</x:v>
       </x:c>
       <x:c r="B37" s="20" t="str">
-        <x:v>筛查 2008 年以来 35,916 条题录，另查 55 条未来日期记录。v2 新增 P162–P166，原有编号保留。</x:v>
+        <x:v>v4 逐行对照用户表格 167 条。补入主目录 P167–P168、边界相关 R11。旧记录及编号保留。</x:v>
       </x:c>
       <x:c r="C37" s="2"/>
       <x:c r="D37" s="2"/>
@@ -1388,7 +1501,7 @@
         <x:v>类型与数量</x:v>
       </x:c>
       <x:c r="B38" s="20" t="str">
-        <x:v>主目录含 3 篇评论、1 篇区块链专辑导论和 4 篇加密数据场景研究。另列 7 篇边界相关文献。</x:v>
+        <x:v>主目录含 3 篇评论、1 篇专辑导论、1 篇社论和 4 篇加密数据场景研究。另列 11 篇边界相关文献。</x:v>
       </x:c>
       <x:c r="C38" s="2"/>
       <x:c r="D38" s="2"/>
@@ -1519,55 +1632,55 @@
       <x:c r="Q4" s="2"/>
     </x:row>
     <x:row r="5" ht="29" customHeight="1">
-      <x:c r="A5" s="51" t="str">
+      <x:c r="A5" s="72" t="str">
         <x:v>编号</x:v>
       </x:c>
-      <x:c r="B5" s="52" t="str">
+      <x:c r="B5" s="73" t="str">
         <x:v>研究主题</x:v>
       </x:c>
-      <x:c r="C5" s="52" t="str">
+      <x:c r="C5" s="73" t="str">
         <x:v>年份</x:v>
       </x:c>
-      <x:c r="D5" s="52" t="str">
+      <x:c r="D5" s="73" t="str">
         <x:v>年月或日期</x:v>
       </x:c>
-      <x:c r="E5" s="52" t="str">
+      <x:c r="E5" s="73" t="str">
         <x:v>期刊</x:v>
       </x:c>
-      <x:c r="F5" s="52" t="str">
+      <x:c r="F5" s="73" t="str">
         <x:v>英文题名</x:v>
       </x:c>
-      <x:c r="G5" s="52" t="str">
+      <x:c r="G5" s="73" t="str">
         <x:v>完整作者</x:v>
       </x:c>
-      <x:c r="H5" s="52" t="str">
+      <x:c r="H5" s="73" t="str">
         <x:v>发表状态</x:v>
       </x:c>
-      <x:c r="I5" s="52" t="str">
+      <x:c r="I5" s="73" t="str">
         <x:v>研究焦点</x:v>
       </x:c>
-      <x:c r="J5" s="52" t="str">
+      <x:c r="J5" s="73" t="str">
         <x:v>文献类型</x:v>
       </x:c>
-      <x:c r="K5" s="52" t="str">
+      <x:c r="K5" s="73" t="str">
         <x:v>卷期与页码</x:v>
       </x:c>
-      <x:c r="L5" s="52" t="str">
+      <x:c r="L5" s="73" t="str">
         <x:v>首次在线日期</x:v>
       </x:c>
-      <x:c r="M5" s="52" t="str">
+      <x:c r="M5" s="73" t="str">
         <x:v>DOI</x:v>
       </x:c>
-      <x:c r="N5" s="52" t="str">
+      <x:c r="N5" s="73" t="str">
         <x:v>来源网址</x:v>
       </x:c>
-      <x:c r="O5" s="52" t="str">
-        <x:v>打开来源</x:v>
-      </x:c>
-      <x:c r="P5" s="52" t="str">
+      <x:c r="O5" s="73" t="str">
+        <x:v>打开来源</x:v>
+      </x:c>
+      <x:c r="P5" s="73" t="str">
         <x:v>补充核验来源</x:v>
       </x:c>
-      <x:c r="Q5" s="53" t="str">
+      <x:c r="Q5" s="74" t="str">
         <x:v>核验说明</x:v>
       </x:c>
     </x:row>
@@ -7104,9 +7217,9 @@
       <x:c r="P120" s="20" t="str"/>
       <x:c r="Q120" s="20" t="str"/>
     </x:row>
-    <x:row r="121" ht="46" customHeight="1">
+    <x:row r="121" ht="90" customHeight="1">
       <x:c r="A121" s="12" t="str">
-        <x:v>P111</x:v>
+        <x:v>P167</x:v>
       </x:c>
       <x:c r="B121" s="18" t="str">
         <x:v>智能合约、DAO、社区与制度治理</x:v>
@@ -7118,42 +7231,48 @@
         <x:v>2024-12-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E121" s="14" t="str">
-        <x:v>JFE</x:v>
+        <x:v>MISQ</x:v>
       </x:c>
       <x:c r="F121" s="20" t="str">
-        <x:v>Token-based platform governance</x:v>
+        <x:v>Time for a Decentralization Journey of Digital Infrastructures? Reflections on the 2023 Impact Award</x:v>
       </x:c>
       <x:c r="G121" s="20" t="str">
-        <x:v>Joseph Abadi; Markus Brunnermeier</x:v>
+        <x:v>Ola Henfridsson; Bendik Bygstad</x:v>
       </x:c>
       <x:c r="H121" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I121" s="20" t="str">
-        <x:v>代币化平台的治理与利益分配</x:v>
+        <x:v>Web3 与 DAO 数字基础设施；以 MakerDAO、DAI 讨论采用、创新及扩展机制</x:v>
       </x:c>
       <x:c r="J121" s="20" t="str">
-        <x:v>直接相关</x:v>
+        <x:v>社论</x:v>
       </x:c>
       <x:c r="K121" s="20" t="str">
-        <x:v>162: 103951</x:v>
-      </x:c>
-      <x:c r="L121" s="22"/>
+        <x:v>48(4): ix-xiv</x:v>
+      </x:c>
+      <x:c r="L121" s="22" t="d">
+        <x:v>2024-12-01T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="M121" s="20" t="str">
-        <x:v>10.1016/j.jfineco.2024.103951</x:v>
+        <x:v>10.25300/misq/2024/788</x:v>
       </x:c>
       <x:c r="N121" s="20" t="str">
-        <x:v>https://doi.org/10.1016/j.jfineco.2024.103951</x:v>
+        <x:v>https://doi.org/10.25300/MISQ/2024/788</x:v>
       </x:c>
       <x:c r="O121" s="23" t="str">
         <x:v>打开来源</x:v>
       </x:c>
-      <x:c r="P121" s="20" t="str"/>
-      <x:c r="Q121" s="20" t="str"/>
+      <x:c r="P121" s="20" t="str">
+        <x:v>https://aisel.aisnet.org/misq/vol48/iss4/5/</x:v>
+      </x:c>
+      <x:c r="Q121" s="20" t="str">
+        <x:v>v4 根据用户表格第 137 行确认遗漏。MISQ/AIS 正式目录确认 2024 年 48(4):ix-xiv，作者为 Ola Henfridsson 与 Bendik Bygstad；用户表与 Crossref 均漏列第二作者，按期刊正式署名补齐。作者公开上传稿明确讨论 Web3、区块链、智能合约、DAO 及 MakerDAO/DAI。此文为 Guest Editorial，单独标为社论，不当作原创实证或理论研究。</x:v>
+      </x:c>
     </x:row>
     <x:row r="122" ht="46" customHeight="1">
       <x:c r="A122" s="12" t="str">
-        <x:v>P112</x:v>
+        <x:v>P111</x:v>
       </x:c>
       <x:c r="B122" s="18" t="str">
         <x:v>智能合约、DAO、社区与制度治理</x:v>
@@ -7165,32 +7284,32 @@
         <x:v>2024-12-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E122" s="14" t="str">
-        <x:v>Management Science</x:v>
+        <x:v>JFE</x:v>
       </x:c>
       <x:c r="F122" s="20" t="str">
-        <x:v>Voting with Time Commitment for Decentralized Governance: Bond Voting as a Sybil-Resistant Mechanism</x:v>
+        <x:v>Token-based platform governance</x:v>
       </x:c>
       <x:c r="G122" s="20" t="str">
-        <x:v>Vijay Mohan; Peyman Khezr; Chris Berg</x:v>
+        <x:v>Joseph Abadi; Markus Brunnermeier</x:v>
       </x:c>
       <x:c r="H122" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I122" s="20" t="str">
-        <x:v>去中心化治理中的锁定承诺与抗女巫投票</x:v>
+        <x:v>代币化平台的治理与利益分配</x:v>
       </x:c>
       <x:c r="J122" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K122" s="20" t="str">
-        <x:v>70(12): 8709-8734</x:v>
+        <x:v>162: 103951</x:v>
       </x:c>
       <x:c r="L122" s="22"/>
       <x:c r="M122" s="20" t="str">
-        <x:v>10.1287/mnsc.2023.01536</x:v>
+        <x:v>10.1016/j.jfineco.2024.103951</x:v>
       </x:c>
       <x:c r="N122" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2023.01536</x:v>
+        <x:v>https://doi.org/10.1016/j.jfineco.2024.103951</x:v>
       </x:c>
       <x:c r="O122" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -7200,46 +7319,44 @@
     </x:row>
     <x:row r="123" ht="46" customHeight="1">
       <x:c r="A123" s="12" t="str">
-        <x:v>P113</x:v>
+        <x:v>P112</x:v>
       </x:c>
       <x:c r="B123" s="18" t="str">
         <x:v>智能合约、DAO、社区与制度治理</x:v>
       </x:c>
       <x:c r="C123" s="15" t="n">
-        <x:v>2025</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="D123" s="24" t="d">
-        <x:v>2025-03-01T00:00:00.000Z</x:v>
+        <x:v>2024-12-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E123" s="14" t="str">
-        <x:v>MISQ</x:v>
+        <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F123" s="20" t="str">
-        <x:v>Regulating Emerging Technologies: Prospective Sensemaking Through Abstraction And Elaboration</x:v>
+        <x:v>Voting with Time Commitment for Decentralized Governance: Bond Voting as a Sybil-Resistant Mechanism</x:v>
       </x:c>
       <x:c r="G123" s="20" t="str">
-        <x:v>Stefan Seidel; Christoph J. Frick; Jan vom Brocke</x:v>
+        <x:v>Vijay Mohan; Peyman Khezr; Chris Berg</x:v>
       </x:c>
       <x:c r="H123" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I123" s="20" t="str">
-        <x:v>围绕区块链与代币经济的监管制度建构</x:v>
+        <x:v>去中心化治理中的锁定承诺与抗女巫投票</x:v>
       </x:c>
       <x:c r="J123" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K123" s="20" t="str">
-        <x:v>49(1): 179-204</x:v>
-      </x:c>
-      <x:c r="L123" s="22" t="d">
-        <x:v>2025-03-01T00:00:00.000Z</x:v>
-      </x:c>
+        <x:v>70(12): 8709-8734</x:v>
+      </x:c>
+      <x:c r="L123" s="22"/>
       <x:c r="M123" s="20" t="str">
-        <x:v>10.25300/misq/2024/18039</x:v>
+        <x:v>10.1287/mnsc.2023.01536</x:v>
       </x:c>
       <x:c r="N123" s="20" t="str">
-        <x:v>https://doi.org/10.25300/MISQ/2024/18039</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2023.01536</x:v>
       </x:c>
       <x:c r="O123" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -7249,7 +7366,7 @@
     </x:row>
     <x:row r="124" ht="46" customHeight="1">
       <x:c r="A124" s="12" t="str">
-        <x:v>P114</x:v>
+        <x:v>P113</x:v>
       </x:c>
       <x:c r="B124" s="18" t="str">
         <x:v>智能合约、DAO、社区与制度治理</x:v>
@@ -7258,35 +7375,37 @@
         <x:v>2025</x:v>
       </x:c>
       <x:c r="D124" s="24" t="d">
-        <x:v>2025-05-01T00:00:00.000Z</x:v>
+        <x:v>2025-03-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E124" s="14" t="str">
-        <x:v>JFE</x:v>
+        <x:v>MISQ</x:v>
       </x:c>
       <x:c r="F124" s="20" t="str">
-        <x:v>Distributed ledgers and the governance of money</x:v>
+        <x:v>Regulating Emerging Technologies: Prospective Sensemaking Through Abstraction And Elaboration</x:v>
       </x:c>
       <x:c r="G124" s="20" t="str">
-        <x:v>Raphael Auer; Cyril Monnet; Hyun Song Shin</x:v>
+        <x:v>Stefan Seidel; Christoph J. Frick; Jan vom Brocke</x:v>
       </x:c>
       <x:c r="H124" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I124" s="20" t="str">
-        <x:v>分布式账本与货币体系治理</x:v>
+        <x:v>围绕区块链与代币经济的监管制度建构</x:v>
       </x:c>
       <x:c r="J124" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K124" s="20" t="str">
-        <x:v>167: 104026</x:v>
-      </x:c>
-      <x:c r="L124" s="22"/>
+        <x:v>49(1): 179-204</x:v>
+      </x:c>
+      <x:c r="L124" s="22" t="d">
+        <x:v>2025-03-01T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="M124" s="20" t="str">
-        <x:v>10.1016/j.jfineco.2025.104026</x:v>
+        <x:v>10.25300/misq/2024/18039</x:v>
       </x:c>
       <x:c r="N124" s="20" t="str">
-        <x:v>https://doi.org/10.1016/j.jfineco.2025.104026</x:v>
+        <x:v>https://doi.org/10.25300/MISQ/2024/18039</x:v>
       </x:c>
       <x:c r="O124" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -7296,7 +7415,7 @@
     </x:row>
     <x:row r="125" ht="46" customHeight="1">
       <x:c r="A125" s="12" t="str">
-        <x:v>P115</x:v>
+        <x:v>P114</x:v>
       </x:c>
       <x:c r="B125" s="18" t="str">
         <x:v>智能合约、DAO、社区与制度治理</x:v>
@@ -7305,35 +7424,35 @@
         <x:v>2025</x:v>
       </x:c>
       <x:c r="D125" s="24" t="d">
-        <x:v>2025-08-01T00:00:00.000Z</x:v>
+        <x:v>2025-05-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E125" s="14" t="str">
-        <x:v>Management Science</x:v>
+        <x:v>JFE</x:v>
       </x:c>
       <x:c r="F125" s="20" t="str">
-        <x:v>Demand-Side Effects of Open Innovation: The Case of Cryptocurrency Forking</x:v>
+        <x:v>Distributed ledgers and the governance of money</x:v>
       </x:c>
       <x:c r="G125" s="20" t="str">
-        <x:v>Vasundhara Sharma; Ashish Agarwal; Anitesh Barua</x:v>
+        <x:v>Raphael Auer; Cyril Monnet; Hyun Song Shin</x:v>
       </x:c>
       <x:c r="H125" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I125" s="20" t="str">
-        <x:v>加密货币分叉与开放创新的需求侧效应</x:v>
+        <x:v>分布式账本与货币体系治理</x:v>
       </x:c>
       <x:c r="J125" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K125" s="20" t="str">
-        <x:v>71(8): 7136-7160</x:v>
+        <x:v>167: 104026</x:v>
       </x:c>
       <x:c r="L125" s="22"/>
       <x:c r="M125" s="20" t="str">
-        <x:v>10.1287/mnsc.2021.03132</x:v>
+        <x:v>10.1016/j.jfineco.2025.104026</x:v>
       </x:c>
       <x:c r="N125" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2021.03132</x:v>
+        <x:v>https://doi.org/10.1016/j.jfineco.2025.104026</x:v>
       </x:c>
       <x:c r="O125" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -7343,7 +7462,7 @@
     </x:row>
     <x:row r="126" ht="46" customHeight="1">
       <x:c r="A126" s="12" t="str">
-        <x:v>P116</x:v>
+        <x:v>P115</x:v>
       </x:c>
       <x:c r="B126" s="18" t="str">
         <x:v>智能合约、DAO、社区与制度治理</x:v>
@@ -7352,37 +7471,35 @@
         <x:v>2025</x:v>
       </x:c>
       <x:c r="D126" s="24" t="d">
-        <x:v>2025-12-01T00:00:00.000Z</x:v>
+        <x:v>2025-08-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E126" s="14" t="str">
-        <x:v>MISQ</x:v>
+        <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F126" s="20" t="str">
-        <x:v>Deductive Certainty? Exploring the Boundaries of Trust Formation in Smart Contracts on Blockchains</x:v>
+        <x:v>Demand-Side Effects of Open Innovation: The Case of Cryptocurrency Forking</x:v>
       </x:c>
       <x:c r="G126" s="20" t="str">
-        <x:v>Daniel Obermeier; Joachim Henkel</x:v>
+        <x:v>Vasundhara Sharma; Ashish Agarwal; Anitesh Barua</x:v>
       </x:c>
       <x:c r="H126" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I126" s="20" t="str">
-        <x:v>区块链智能合约的信任形成及边界</x:v>
+        <x:v>加密货币分叉与开放创新的需求侧效应</x:v>
       </x:c>
       <x:c r="J126" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K126" s="20" t="str">
-        <x:v>49(4): 1513-1538</x:v>
-      </x:c>
-      <x:c r="L126" s="22" t="d">
-        <x:v>2025-12-01T00:00:00.000Z</x:v>
-      </x:c>
+        <x:v>71(8): 7136-7160</x:v>
+      </x:c>
+      <x:c r="L126" s="22"/>
       <x:c r="M126" s="20" t="str">
-        <x:v>10.25300/misq/2025/18501</x:v>
+        <x:v>10.1287/mnsc.2021.03132</x:v>
       </x:c>
       <x:c r="N126" s="20" t="str">
-        <x:v>https://doi.org/10.25300/MISQ/2025/18501</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2021.03132</x:v>
       </x:c>
       <x:c r="O126" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -7392,46 +7509,46 @@
     </x:row>
     <x:row r="127" ht="46" customHeight="1">
       <x:c r="A127" s="12" t="str">
-        <x:v>P117</x:v>
+        <x:v>P116</x:v>
       </x:c>
       <x:c r="B127" s="18" t="str">
         <x:v>智能合约、DAO、社区与制度治理</x:v>
       </x:c>
       <x:c r="C127" s="15" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="D127" s="16" t="d">
-        <x:v>2026-04-06T00:00:00.000Z</x:v>
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="D127" s="24" t="d">
+        <x:v>2025-12-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E127" s="14" t="str">
-        <x:v>ISR</x:v>
+        <x:v>MISQ</x:v>
       </x:c>
       <x:c r="F127" s="20" t="str">
-        <x:v>Token Incentive and Blockchain Developer Contribution</x:v>
+        <x:v>Deductive Certainty? Exploring the Boundaries of Trust Formation in Smart Contracts on Blockchains</x:v>
       </x:c>
       <x:c r="G127" s="20" t="str">
-        <x:v>Ning Luo; Zhiqiang (Eric) Zheng</x:v>
+        <x:v>Daniel Obermeier; Joachim Henkel</x:v>
       </x:c>
       <x:c r="H127" s="21" t="str">
-        <x:v>在线发表</x:v>
+        <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I127" s="20" t="str">
-        <x:v>代币激励与区块链开发者贡献</x:v>
+        <x:v>区块链智能合约的信任形成及边界</x:v>
       </x:c>
       <x:c r="J127" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K127" s="20" t="str">
-        <x:v>未编入卷期</x:v>
+        <x:v>49(4): 1513-1538</x:v>
       </x:c>
       <x:c r="L127" s="22" t="d">
-        <x:v>2026-04-06T00:00:00.000Z</x:v>
+        <x:v>2025-12-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="M127" s="20" t="str">
-        <x:v>10.1287/isre.2023.0480</x:v>
+        <x:v>10.25300/misq/2025/18501</x:v>
       </x:c>
       <x:c r="N127" s="20" t="str">
-        <x:v>https://doi.org/10.1287/isre.2023.0480</x:v>
+        <x:v>https://doi.org/10.25300/MISQ/2025/18501</x:v>
       </x:c>
       <x:c r="O127" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -7441,7 +7558,7 @@
     </x:row>
     <x:row r="128" ht="46" customHeight="1">
       <x:c r="A128" s="12" t="str">
-        <x:v>P118</x:v>
+        <x:v>P117</x:v>
       </x:c>
       <x:c r="B128" s="18" t="str">
         <x:v>智能合约、DAO、社区与制度治理</x:v>
@@ -7450,37 +7567,37 @@
         <x:v>2026</x:v>
       </x:c>
       <x:c r="D128" s="16" t="d">
-        <x:v>2026-04-30T00:00:00.000Z</x:v>
+        <x:v>2026-04-06T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E128" s="14" t="str">
-        <x:v>Management Science</x:v>
+        <x:v>ISR</x:v>
       </x:c>
       <x:c r="F128" s="20" t="str">
-        <x:v>Continuity of Fixed-Fraction Rules: Comment on “Sharing Sequentially Triggered Losses: Automated Conflict Resolution Through Smart Contracts”</x:v>
+        <x:v>Token Incentive and Blockchain Developer Contribution</x:v>
       </x:c>
       <x:c r="G128" s="20" t="str">
-        <x:v>René van den Brink; Elena Gavilán; Conrado Manuel; Takayuki Oishi</x:v>
+        <x:v>Ning Luo; Zhiqiang (Eric) Zheng</x:v>
       </x:c>
       <x:c r="H128" s="21" t="str">
         <x:v>在线发表</x:v>
       </x:c>
       <x:c r="I128" s="20" t="str">
-        <x:v>智能合约损失分配规则论文的后续评论</x:v>
+        <x:v>代币激励与区块链开发者贡献</x:v>
       </x:c>
       <x:c r="J128" s="20" t="str">
-        <x:v>评论</x:v>
+        <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K128" s="20" t="str">
         <x:v>未编入卷期</x:v>
       </x:c>
       <x:c r="L128" s="22" t="d">
-        <x:v>2026-04-30T00:00:00.000Z</x:v>
+        <x:v>2026-04-06T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="M128" s="20" t="str">
-        <x:v>10.1287/mnsc.2025.03401</x:v>
+        <x:v>10.1287/isre.2023.0480</x:v>
       </x:c>
       <x:c r="N128" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2025.03401</x:v>
+        <x:v>https://doi.org/10.1287/isre.2023.0480</x:v>
       </x:c>
       <x:c r="O128" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -7490,7 +7607,7 @@
     </x:row>
     <x:row r="129" ht="46" customHeight="1">
       <x:c r="A129" s="12" t="str">
-        <x:v>P119</x:v>
+        <x:v>P118</x:v>
       </x:c>
       <x:c r="B129" s="18" t="str">
         <x:v>智能合约、DAO、社区与制度治理</x:v>
@@ -7499,37 +7616,37 @@
         <x:v>2026</x:v>
       </x:c>
       <x:c r="D129" s="16" t="d">
-        <x:v>2026-06-12T00:00:00.000Z</x:v>
+        <x:v>2026-04-30T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E129" s="14" t="str">
         <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F129" s="20" t="str">
-        <x:v>Decentralized Autonomous Organization Governance</x:v>
+        <x:v>Continuity of Fixed-Fraction Rules: Comment on “Sharing Sequentially Triggered Losses: Automated Conflict Resolution Through Smart Contracts”</x:v>
       </x:c>
       <x:c r="G129" s="20" t="str">
-        <x:v>Jungsuk Han; Jongsub Lee; Tao Li</x:v>
+        <x:v>René van den Brink; Elena Gavilán; Conrado Manuel; Takayuki Oishi</x:v>
       </x:c>
       <x:c r="H129" s="21" t="str">
         <x:v>在线发表</x:v>
       </x:c>
       <x:c r="I129" s="20" t="str">
-        <x:v>去中心化自治组织的治理</x:v>
+        <x:v>智能合约损失分配规则论文的后续评论</x:v>
       </x:c>
       <x:c r="J129" s="20" t="str">
-        <x:v>直接相关</x:v>
+        <x:v>评论</x:v>
       </x:c>
       <x:c r="K129" s="20" t="str">
         <x:v>未编入卷期</x:v>
       </x:c>
       <x:c r="L129" s="22" t="d">
-        <x:v>2026-06-12T00:00:00.000Z</x:v>
+        <x:v>2026-04-30T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="M129" s="20" t="str">
-        <x:v>10.1287/mnsc.2024.07033</x:v>
+        <x:v>10.1287/mnsc.2025.03401</x:v>
       </x:c>
       <x:c r="N129" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2024.07033</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2025.03401</x:v>
       </x:c>
       <x:c r="O129" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -7537,9 +7654,9 @@
       <x:c r="P129" s="20" t="str"/>
       <x:c r="Q129" s="20" t="str"/>
     </x:row>
-    <x:row r="130" ht="46" customHeight="1">
+    <x:row r="130" ht="64" customHeight="1">
       <x:c r="A130" s="12" t="str">
-        <x:v>P120</x:v>
+        <x:v>P168</x:v>
       </x:c>
       <x:c r="B130" s="18" t="str">
         <x:v>智能合约、DAO、社区与制度治理</x:v>
@@ -7547,134 +7664,140 @@
       <x:c r="C130" s="15" t="n">
         <x:v>2026</x:v>
       </x:c>
-      <x:c r="D130" s="16" t="d">
-        <x:v>2026-09-17T00:00:00.000Z</x:v>
+      <x:c r="D130" s="24" t="d">
+        <x:v>2026-06-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E130" s="14" t="str">
-        <x:v>ISR</x:v>
+        <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F130" s="20" t="str">
-        <x:v>Unveiling the Impact of Delegated Voting on Decentralized Autonomous Organizations</x:v>
+        <x:v>Balancing Power in Decentralized Governance: Quadratic Voting and Information Aggregation</x:v>
       </x:c>
       <x:c r="G130" s="20" t="str">
-        <x:v>Zhecheng Wang; Xinyu Zang; Xiang (Shawn) Wan; Hsing Kenneth Cheng; Xi Zhao; Gengzhong Feng</x:v>
+        <x:v>Alon Benhaim; Brett Hemenway Falk; Gerry Tsoukalas</x:v>
       </x:c>
       <x:c r="H130" s="21" t="str">
+        <x:v>卷期发表</x:v>
+      </x:c>
+      <x:c r="I130" s="20" t="str">
+        <x:v>DAO 与去中心化治理中的二次投票、偏好聚合与信息聚合的权衡</x:v>
+      </x:c>
+      <x:c r="J130" s="20" t="str">
+        <x:v>直接相关</x:v>
+      </x:c>
+      <x:c r="K130" s="20" t="str">
+        <x:v>72(6): 4597-4609</x:v>
+      </x:c>
+      <x:c r="L130" s="22" t="d">
+        <x:v>2025-11-03T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="M130" s="20" t="str">
+        <x:v>10.1287/mnsc.2024.08469</x:v>
+      </x:c>
+      <x:c r="N130" s="20" t="str">
+        <x:v>https://doi.org/10.1287/mnsc.2024.08469</x:v>
+      </x:c>
+      <x:c r="O130" s="23" t="str">
+        <x:v>打开来源</x:v>
+      </x:c>
+      <x:c r="P130" s="20" t="str">
+        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=4416748</x:v>
+      </x:c>
+      <x:c r="Q130" s="20" t="str">
+        <x:v>v4 根据用户表格第 103 行确认此前遗漏。出版方确认 72(6):4597-4609，正式卷期 2026-06，首次在线 2025-11-03，接收 2025-06-08。作者公开稿将 blockchain、dApps 列为关键词；属于去中心化治理的投票机制研究。原题名及摘要的通用表述未触发首轮关键词筛选。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131" ht="46" customHeight="1">
+      <x:c r="A131" s="12" t="str">
+        <x:v>P119</x:v>
+      </x:c>
+      <x:c r="B131" s="18" t="str">
+        <x:v>智能合约、DAO、社区与制度治理</x:v>
+      </x:c>
+      <x:c r="C131" s="15" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="D131" s="16" t="d">
+        <x:v>2026-06-12T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E131" s="14" t="str">
+        <x:v>Management Science</x:v>
+      </x:c>
+      <x:c r="F131" s="20" t="str">
+        <x:v>Decentralized Autonomous Organization Governance</x:v>
+      </x:c>
+      <x:c r="G131" s="20" t="str">
+        <x:v>Jungsuk Han; Jongsub Lee; Tao Li</x:v>
+      </x:c>
+      <x:c r="H131" s="21" t="str">
         <x:v>在线发表</x:v>
       </x:c>
-      <x:c r="I130" s="20" t="str">
-        <x:v>委托投票对 DAO 治理的影响</x:v>
-      </x:c>
-      <x:c r="J130" s="20" t="str">
-        <x:v>直接相关</x:v>
-      </x:c>
-      <x:c r="K130" s="20" t="str">
+      <x:c r="I131" s="20" t="str">
+        <x:v>去中心化自治组织的治理</x:v>
+      </x:c>
+      <x:c r="J131" s="20" t="str">
+        <x:v>直接相关</x:v>
+      </x:c>
+      <x:c r="K131" s="20" t="str">
         <x:v>未编入卷期</x:v>
       </x:c>
-      <x:c r="L130" s="22" t="d">
-        <x:v>2026-09-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="M130" s="20" t="str">
-        <x:v>10.1287/isre.2024.1718</x:v>
-      </x:c>
-      <x:c r="N130" s="20" t="str">
-        <x:v>https://doi.org/10.1287/isre.2024.1718</x:v>
-      </x:c>
-      <x:c r="O130" s="23" t="str">
-        <x:v>打开来源</x:v>
-      </x:c>
-      <x:c r="P130" s="20" t="str"/>
-      <x:c r="Q130" s="20" t="str"/>
-    </x:row>
-    <x:row r="131" ht="46" customHeight="1">
-      <x:c r="A131" s="25" t="str">
-        <x:v>P121</x:v>
-      </x:c>
-      <x:c r="B131" s="34" t="str">
-        <x:v>企业披露、财务会计与审计</x:v>
-      </x:c>
-      <x:c r="C131" s="27" t="n">
-        <x:v>2019</x:v>
-      </x:c>
-      <x:c r="D131" s="28" t="d">
-        <x:v>2019-12-01T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="E131" s="29" t="str">
-        <x:v>Management Science</x:v>
-      </x:c>
-      <x:c r="F131" s="30" t="str">
-        <x:v>Riding the Blockchain Mania: Public Firms’ Speculative 8-K Disclosures</x:v>
-      </x:c>
-      <x:c r="G131" s="30" t="str">
-        <x:v>Stephanie F. Cheng; Gus De Franco; Haibo Jiang; Pengkai Lin</x:v>
-      </x:c>
-      <x:c r="H131" s="31" t="str">
-        <x:v>卷期发表</x:v>
-      </x:c>
-      <x:c r="I131" s="30" t="str">
-        <x:v>上市公司投机性区块链 8-K 披露</x:v>
-      </x:c>
-      <x:c r="J131" s="30" t="str">
-        <x:v>直接相关</x:v>
-      </x:c>
-      <x:c r="K131" s="30" t="str">
-        <x:v>65(12): 5901-5913</x:v>
-      </x:c>
-      <x:c r="L131" s="32"/>
-      <x:c r="M131" s="30" t="str">
-        <x:v>10.1287/mnsc.2019.3357</x:v>
-      </x:c>
-      <x:c r="N131" s="30" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2019.3357</x:v>
-      </x:c>
-      <x:c r="O131" s="33" t="str">
-        <x:v>打开来源</x:v>
-      </x:c>
-      <x:c r="P131" s="30" t="str"/>
-      <x:c r="Q131" s="30" t="str"/>
+      <x:c r="L131" s="22" t="d">
+        <x:v>2026-06-12T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="M131" s="20" t="str">
+        <x:v>10.1287/mnsc.2024.07033</x:v>
+      </x:c>
+      <x:c r="N131" s="20" t="str">
+        <x:v>https://doi.org/10.1287/mnsc.2024.07033</x:v>
+      </x:c>
+      <x:c r="O131" s="23" t="str">
+        <x:v>打开来源</x:v>
+      </x:c>
+      <x:c r="P131" s="20" t="str"/>
+      <x:c r="Q131" s="20" t="str"/>
     </x:row>
     <x:row r="132" ht="46" customHeight="1">
       <x:c r="A132" s="12" t="str">
-        <x:v>P122</x:v>
+        <x:v>P120</x:v>
       </x:c>
       <x:c r="B132" s="18" t="str">
-        <x:v>企业披露、财务会计与审计</x:v>
+        <x:v>智能合约、DAO、社区与制度治理</x:v>
       </x:c>
       <x:c r="C132" s="15" t="n">
-        <x:v>2022</x:v>
-      </x:c>
-      <x:c r="D132" s="24" t="d">
-        <x:v>2022-03-01T00:00:00.000Z</x:v>
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="D132" s="16" t="d">
+        <x:v>2026-09-17T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E132" s="14" t="str">
-        <x:v>JAR</x:v>
+        <x:v>ISR</x:v>
       </x:c>
       <x:c r="F132" s="20" t="str">
-        <x:v>The Role of Disclosure and Information Intermediaries in an Unregulated Capital Market: Evidence from Initial Coin Offerings</x:v>
+        <x:v>Unveiling the Impact of Delegated Voting on Decentralized Autonomous Organizations</x:v>
       </x:c>
       <x:c r="G132" s="20" t="str">
-        <x:v>Thomas Bourveau; Emmanuel T. De George; Atif Ellahie; Daniele Macciocchi</x:v>
+        <x:v>Zhecheng Wang; Xinyu Zang; Xiang (Shawn) Wan; Hsing Kenneth Cheng; Xi Zhao; Gengzhong Feng</x:v>
       </x:c>
       <x:c r="H132" s="21" t="str">
-        <x:v>卷期发表</x:v>
+        <x:v>在线发表</x:v>
       </x:c>
       <x:c r="I132" s="20" t="str">
-        <x:v>ICO 自愿披露与信息中介</x:v>
+        <x:v>委托投票对 DAO 治理的影响</x:v>
       </x:c>
       <x:c r="J132" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K132" s="20" t="str">
-        <x:v>60(1): 129-167</x:v>
-      </x:c>
-      <x:c r="L132" s="35" t="d">
-        <x:v>2021-11-01T00:00:00.000Z</x:v>
+        <x:v>未编入卷期</x:v>
+      </x:c>
+      <x:c r="L132" s="22" t="d">
+        <x:v>2026-09-17T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="M132" s="20" t="str">
-        <x:v>10.1111/1475-679x.12404</x:v>
+        <x:v>10.1287/isre.2024.1718</x:v>
       </x:c>
       <x:c r="N132" s="20" t="str">
-        <x:v>https://doi.org/10.1111/1475-679x.12404</x:v>
+        <x:v>https://doi.org/10.1287/isre.2024.1718</x:v>
       </x:c>
       <x:c r="O132" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -7683,92 +7806,94 @@
       <x:c r="Q132" s="20" t="str"/>
     </x:row>
     <x:row r="133" ht="46" customHeight="1">
-      <x:c r="A133" s="12" t="str">
-        <x:v>P123</x:v>
-      </x:c>
-      <x:c r="B133" s="18" t="str">
+      <x:c r="A133" s="25" t="str">
+        <x:v>P121</x:v>
+      </x:c>
+      <x:c r="B133" s="34" t="str">
         <x:v>企业披露、财务会计与审计</x:v>
       </x:c>
-      <x:c r="C133" s="15" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="D133" s="24" t="d">
-        <x:v>2023-11-01T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="E133" s="14" t="str">
+      <x:c r="C133" s="27" t="n">
+        <x:v>2019</x:v>
+      </x:c>
+      <x:c r="D133" s="28" t="d">
+        <x:v>2019-12-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E133" s="29" t="str">
         <x:v>Management Science</x:v>
       </x:c>
-      <x:c r="F133" s="20" t="str">
-        <x:v>Conflicted Analysts and Initial Coin Offerings</x:v>
-      </x:c>
-      <x:c r="G133" s="20" t="str">
-        <x:v>Andreas Barth; Valerie Laturnus; Sasan Mansouri; Alexander F. Wagner</x:v>
-      </x:c>
-      <x:c r="H133" s="21" t="str">
-        <x:v>卷期发表</x:v>
-      </x:c>
-      <x:c r="I133" s="20" t="str">
-        <x:v>ICO 分析师利益冲突与评级</x:v>
-      </x:c>
-      <x:c r="J133" s="20" t="str">
-        <x:v>直接相关</x:v>
-      </x:c>
-      <x:c r="K133" s="20" t="str">
-        <x:v>69(11): 6641-6666</x:v>
-      </x:c>
-      <x:c r="L133" s="22"/>
-      <x:c r="M133" s="20" t="str">
-        <x:v>10.1287/mnsc.2021.02928</x:v>
-      </x:c>
-      <x:c r="N133" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2021.02928</x:v>
-      </x:c>
-      <x:c r="O133" s="23" t="str">
-        <x:v>打开来源</x:v>
-      </x:c>
-      <x:c r="P133" s="20" t="str"/>
-      <x:c r="Q133" s="20" t="str"/>
+      <x:c r="F133" s="30" t="str">
+        <x:v>Riding the Blockchain Mania: Public Firms’ Speculative 8-K Disclosures</x:v>
+      </x:c>
+      <x:c r="G133" s="30" t="str">
+        <x:v>Stephanie F. Cheng; Gus De Franco; Haibo Jiang; Pengkai Lin</x:v>
+      </x:c>
+      <x:c r="H133" s="31" t="str">
+        <x:v>卷期发表</x:v>
+      </x:c>
+      <x:c r="I133" s="30" t="str">
+        <x:v>上市公司投机性区块链 8-K 披露</x:v>
+      </x:c>
+      <x:c r="J133" s="30" t="str">
+        <x:v>直接相关</x:v>
+      </x:c>
+      <x:c r="K133" s="30" t="str">
+        <x:v>65(12): 5901-5913</x:v>
+      </x:c>
+      <x:c r="L133" s="32"/>
+      <x:c r="M133" s="30" t="str">
+        <x:v>10.1287/mnsc.2019.3357</x:v>
+      </x:c>
+      <x:c r="N133" s="30" t="str">
+        <x:v>https://doi.org/10.1287/mnsc.2019.3357</x:v>
+      </x:c>
+      <x:c r="O133" s="33" t="str">
+        <x:v>打开来源</x:v>
+      </x:c>
+      <x:c r="P133" s="30" t="str"/>
+      <x:c r="Q133" s="30" t="str"/>
     </x:row>
     <x:row r="134" ht="46" customHeight="1">
       <x:c r="A134" s="12" t="str">
-        <x:v>P124</x:v>
+        <x:v>P122</x:v>
       </x:c>
       <x:c r="B134" s="18" t="str">
         <x:v>企业披露、财务会计与审计</x:v>
       </x:c>
       <x:c r="C134" s="15" t="n">
-        <x:v>2024</x:v>
+        <x:v>2022</x:v>
       </x:c>
       <x:c r="D134" s="24" t="d">
-        <x:v>2024-02-01T00:00:00.000Z</x:v>
+        <x:v>2022-03-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E134" s="14" t="str">
-        <x:v>Management Science</x:v>
+        <x:v>JAR</x:v>
       </x:c>
       <x:c r="F134" s="20" t="str">
-        <x:v>The (Limited) Power of Blockchain Networks for Information Provision</x:v>
+        <x:v>The Role of Disclosure and Information Intermediaries in an Unregulated Capital Market: Evidence from Initial Coin Offerings</x:v>
       </x:c>
       <x:c r="G134" s="20" t="str">
-        <x:v>Benedikt Franke; Qi Gao Fritz; André Stenzel</x:v>
+        <x:v>Thomas Bourveau; Emmanuel T. De George; Atif Ellahie; Daniele Macciocchi</x:v>
       </x:c>
       <x:c r="H134" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I134" s="20" t="str">
-        <x:v>企业区块链的信息提供能力与边界</x:v>
+        <x:v>ICO 自愿披露与信息中介</x:v>
       </x:c>
       <x:c r="J134" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K134" s="20" t="str">
-        <x:v>70(2): 971-990</x:v>
-      </x:c>
-      <x:c r="L134" s="22"/>
+        <x:v>60(1): 129-167</x:v>
+      </x:c>
+      <x:c r="L134" s="35" t="d">
+        <x:v>2021-11-01T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="M134" s="20" t="str">
-        <x:v>10.1287/mnsc.2023.4718</x:v>
+        <x:v>10.1111/1475-679x.12404</x:v>
       </x:c>
       <x:c r="N134" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2023.4718</x:v>
+        <x:v>https://doi.org/10.1111/1475-679x.12404</x:v>
       </x:c>
       <x:c r="O134" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -7778,46 +7903,44 @@
     </x:row>
     <x:row r="135" ht="46" customHeight="1">
       <x:c r="A135" s="12" t="str">
-        <x:v>P125</x:v>
+        <x:v>P123</x:v>
       </x:c>
       <x:c r="B135" s="18" t="str">
         <x:v>企业披露、财务会计与审计</x:v>
       </x:c>
       <x:c r="C135" s="15" t="n">
-        <x:v>2025</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="D135" s="24" t="d">
-        <x:v>2025-05-01T00:00:00.000Z</x:v>
+        <x:v>2023-11-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E135" s="14" t="str">
-        <x:v>TAR</x:v>
+        <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F135" s="20" t="str">
-        <x:v>Using Blockchain, Non-Fungible Tokens, and Smart Contracts to Track and Report Greenhouse Gas Emissions</x:v>
+        <x:v>Conflicted Analysts and Initial Coin Offerings</x:v>
       </x:c>
       <x:c r="G135" s="20" t="str">
-        <x:v>J. Gregory Jenkins; Eric M. Negangard; Mark D. Sheldon</x:v>
+        <x:v>Andreas Barth; Valerie Laturnus; Sasan Mansouri; Alexander F. Wagner</x:v>
       </x:c>
       <x:c r="H135" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I135" s="20" t="str">
-        <x:v>区块链、NFT 与智能合约支持温室气体排放报告</x:v>
+        <x:v>ICO 分析师利益冲突与评级</x:v>
       </x:c>
       <x:c r="J135" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K135" s="20" t="str">
-        <x:v>100(3): 277-305</x:v>
-      </x:c>
-      <x:c r="L135" s="22" t="d">
-        <x:v>2025-04-08T00:00:00.000Z</x:v>
-      </x:c>
+        <x:v>69(11): 6641-6666</x:v>
+      </x:c>
+      <x:c r="L135" s="22"/>
       <x:c r="M135" s="20" t="str">
-        <x:v>10.2308/tar-2023-0222</x:v>
+        <x:v>10.1287/mnsc.2021.02928</x:v>
       </x:c>
       <x:c r="N135" s="20" t="str">
-        <x:v>https://doi.org/10.2308/tar-2023-0222</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2021.02928</x:v>
       </x:c>
       <x:c r="O135" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -7827,44 +7950,44 @@
     </x:row>
     <x:row r="136" ht="46" customHeight="1">
       <x:c r="A136" s="12" t="str">
-        <x:v>P126</x:v>
+        <x:v>P124</x:v>
       </x:c>
       <x:c r="B136" s="18" t="str">
         <x:v>企业披露、财务会计与审计</x:v>
       </x:c>
       <x:c r="C136" s="15" t="n">
-        <x:v>2025</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="D136" s="24" t="d">
-        <x:v>2025-05-01T00:00:00.000Z</x:v>
+        <x:v>2024-02-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E136" s="14" t="str">
         <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F136" s="20" t="str">
-        <x:v>Distributed Ledgers and Secure Multiparty Computation for Financial Reporting and Auditing</x:v>
+        <x:v>The (Limited) Power of Blockchain Networks for Information Provision</x:v>
       </x:c>
       <x:c r="G136" s="20" t="str">
-        <x:v>Sean Shun Cao; Lin William Cong; Baozhong Yang</x:v>
+        <x:v>Benedikt Franke; Qi Gao Fritz; André Stenzel</x:v>
       </x:c>
       <x:c r="H136" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I136" s="20" t="str">
-        <x:v>分布式账本、安全多方计算与报告审计</x:v>
+        <x:v>企业区块链的信息提供能力与边界</x:v>
       </x:c>
       <x:c r="J136" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K136" s="20" t="str">
-        <x:v>71(5): 3852-3872</x:v>
+        <x:v>70(2): 971-990</x:v>
       </x:c>
       <x:c r="L136" s="22"/>
       <x:c r="M136" s="20" t="str">
-        <x:v>10.1287/mnsc.2023.02577</x:v>
+        <x:v>10.1287/mnsc.2023.4718</x:v>
       </x:c>
       <x:c r="N136" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2023.02577</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2023.4718</x:v>
       </x:c>
       <x:c r="O136" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -7874,7 +7997,7 @@
     </x:row>
     <x:row r="137" ht="46" customHeight="1">
       <x:c r="A137" s="12" t="str">
-        <x:v>P127</x:v>
+        <x:v>P125</x:v>
       </x:c>
       <x:c r="B137" s="18" t="str">
         <x:v>企业披露、财务会计与审计</x:v>
@@ -7883,37 +8006,37 @@
         <x:v>2025</x:v>
       </x:c>
       <x:c r="D137" s="24" t="d">
-        <x:v>2025-06-01T00:00:00.000Z</x:v>
+        <x:v>2025-05-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E137" s="14" t="str">
-        <x:v>JAR</x:v>
+        <x:v>TAR</x:v>
       </x:c>
       <x:c r="F137" s="20" t="str">
-        <x:v>The Effect of Intangible Asset Classification on Professional Financial Statement Users’ Assessments</x:v>
+        <x:v>Using Blockchain, Non-Fungible Tokens, and Smart Contracts to Track and Report Greenhouse Gas Emissions</x:v>
       </x:c>
       <x:c r="G137" s="20" t="str">
-        <x:v>Spencer B. Anderson; Kim I. Mendoza; Cassie Mongold</x:v>
+        <x:v>J. Gregory Jenkins; Eric M. Negangard; Mark D. Sheldon</x:v>
       </x:c>
       <x:c r="H137" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I137" s="20" t="str">
-        <x:v>以加密资产分类为场景的财务报表使用者实验</x:v>
+        <x:v>区块链、NFT 与智能合约支持温室气体排放报告</x:v>
       </x:c>
       <x:c r="J137" s="20" t="str">
-        <x:v>加密场景</x:v>
+        <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K137" s="20" t="str">
-        <x:v>63(3): 1107-1143</x:v>
+        <x:v>100(3): 277-305</x:v>
       </x:c>
       <x:c r="L137" s="22" t="d">
-        <x:v>2025-03-04T00:00:00.000Z</x:v>
+        <x:v>2025-04-08T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="M137" s="20" t="str">
-        <x:v>10.1111/1475-679x.12604</x:v>
+        <x:v>10.2308/tar-2023-0222</x:v>
       </x:c>
       <x:c r="N137" s="20" t="str">
-        <x:v>https://doi.org/10.1111/1475-679x.12604</x:v>
+        <x:v>https://doi.org/10.2308/tar-2023-0222</x:v>
       </x:c>
       <x:c r="O137" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -7923,95 +8046,93 @@
     </x:row>
     <x:row r="138" ht="46" customHeight="1">
       <x:c r="A138" s="12" t="str">
-        <x:v>P128</x:v>
+        <x:v>P126</x:v>
       </x:c>
       <x:c r="B138" s="18" t="str">
         <x:v>企业披露、财务会计与审计</x:v>
       </x:c>
       <x:c r="C138" s="15" t="n">
-        <x:v>2026</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="D138" s="24" t="d">
-        <x:v>2026-03-01T00:00:00.000Z</x:v>
+        <x:v>2025-05-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E138" s="14" t="str">
-        <x:v>JAR</x:v>
+        <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F138" s="20" t="str">
-        <x:v>Accounting for Cryptocurrencies</x:v>
+        <x:v>Distributed Ledgers and Secure Multiparty Computation for Financial Reporting and Auditing</x:v>
       </x:c>
       <x:c r="G138" s="20" t="str">
-        <x:v>Chelsea M. Anderson; Vivian W. Fang; James R. Moon Jr.; Jonathan E. Shipman</x:v>
+        <x:v>Sean Shun Cao; Lin William Cong; Baozhong Yang</x:v>
       </x:c>
       <x:c r="H138" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I138" s="20" t="str">
-        <x:v>上市公司加密资产持有与会计处理</x:v>
+        <x:v>分布式账本、安全多方计算与报告审计</x:v>
       </x:c>
       <x:c r="J138" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K138" s="20" t="str">
-        <x:v>64(1): 45-79</x:v>
-      </x:c>
-      <x:c r="L138" s="22" t="d">
-        <x:v>2025-09-15T00:00:00.000Z</x:v>
-      </x:c>
+        <x:v>71(5): 3852-3872</x:v>
+      </x:c>
+      <x:c r="L138" s="22"/>
       <x:c r="M138" s="20" t="str">
-        <x:v>10.1111/1475-679x.70018</x:v>
+        <x:v>10.1287/mnsc.2023.02577</x:v>
       </x:c>
       <x:c r="N138" s="20" t="str">
-        <x:v>https://doi.org/10.1111/1475-679x.70018</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2023.02577</x:v>
       </x:c>
       <x:c r="O138" s="23" t="str">
         <x:v>打开来源</x:v>
       </x:c>
       <x:c r="P138" s="20" t="str"/>
-      <x:c r="Q138" s="20" t="str">
-        <x:v>正式卷期为 2026 年 64(1)，首次在线为 2025-09-15。</x:v>
-      </x:c>
+      <x:c r="Q138" s="20" t="str"/>
     </x:row>
     <x:row r="139" ht="46" customHeight="1">
       <x:c r="A139" s="12" t="str">
-        <x:v>P129</x:v>
+        <x:v>P127</x:v>
       </x:c>
       <x:c r="B139" s="18" t="str">
         <x:v>企业披露、财务会计与审计</x:v>
       </x:c>
       <x:c r="C139" s="15" t="n">
-        <x:v>2026</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="D139" s="24" t="d">
-        <x:v>2026-06-01T00:00:00.000Z</x:v>
+        <x:v>2025-06-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E139" s="14" t="str">
-        <x:v>Management Science</x:v>
+        <x:v>JAR</x:v>
       </x:c>
       <x:c r="F139" s="20" t="str">
-        <x:v>The Role of Auditor Reputation in an Emerging Audit Marketplace: Evidence from Decentralized Finance (DeFi)</x:v>
+        <x:v>The Effect of Intangible Asset Classification on Professional Financial Statement Users’ Assessments</x:v>
       </x:c>
       <x:c r="G139" s="20" t="str">
-        <x:v>W. Robert Knechel; Steven A. Maex; Hyun Jong Park</x:v>
+        <x:v>Spencer B. Anderson; Kim I. Mendoza; Cassie Mongold</x:v>
       </x:c>
       <x:c r="H139" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I139" s="20" t="str">
-        <x:v>DeFi 审计市场中的审计师声誉</x:v>
+        <x:v>以加密资产分类为场景的财务报表使用者实验</x:v>
       </x:c>
       <x:c r="J139" s="20" t="str">
-        <x:v>直接相关</x:v>
+        <x:v>加密场景</x:v>
       </x:c>
       <x:c r="K139" s="20" t="str">
-        <x:v>72(6): 5083-5105</x:v>
-      </x:c>
-      <x:c r="L139" s="22"/>
+        <x:v>63(3): 1107-1143</x:v>
+      </x:c>
+      <x:c r="L139" s="22" t="d">
+        <x:v>2025-03-04T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="M139" s="20" t="str">
-        <x:v>10.1287/mnsc.2023.02245</x:v>
+        <x:v>10.1111/1475-679x.12604</x:v>
       </x:c>
       <x:c r="N139" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2023.02245</x:v>
+        <x:v>https://doi.org/10.1111/1475-679x.12604</x:v>
       </x:c>
       <x:c r="O139" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -8021,7 +8142,7 @@
     </x:row>
     <x:row r="140" ht="46" customHeight="1">
       <x:c r="A140" s="12" t="str">
-        <x:v>P130</x:v>
+        <x:v>P128</x:v>
       </x:c>
       <x:c r="B140" s="18" t="str">
         <x:v>企业披露、财务会计与审计</x:v>
@@ -8030,45 +8151,49 @@
         <x:v>2026</x:v>
       </x:c>
       <x:c r="D140" s="24" t="d">
-        <x:v>2026-07-01T00:00:00.000Z</x:v>
+        <x:v>2026-03-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E140" s="14" t="str">
-        <x:v>JAE</x:v>
+        <x:v>JAR</x:v>
       </x:c>
       <x:c r="F140" s="20" t="str">
-        <x:v>Auditing smart contracts</x:v>
+        <x:v>Accounting for Cryptocurrencies</x:v>
       </x:c>
       <x:c r="G140" s="20" t="str">
-        <x:v>Wayne Landsman; Evgeny Lyandres; Edward Maydew; Daniel Rabetti; Che Zhang</x:v>
+        <x:v>Chelsea M. Anderson; Vivian W. Fang; James R. Moon Jr.; Jonathan E. Shipman</x:v>
       </x:c>
       <x:c r="H140" s="21" t="str">
-        <x:v>在线发表</x:v>
+        <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I140" s="20" t="str">
-        <x:v>DeFi 智能合约审计的决定因素与后果</x:v>
+        <x:v>上市公司加密资产持有与会计处理</x:v>
       </x:c>
       <x:c r="J140" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K140" s="20" t="str">
-        <x:v>未编入卷期</x:v>
-      </x:c>
-      <x:c r="L140" s="22"/>
+        <x:v>64(1): 45-79</x:v>
+      </x:c>
+      <x:c r="L140" s="22" t="d">
+        <x:v>2025-09-15T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="M140" s="20" t="str">
-        <x:v>10.1016/j.jacceco.2026.101911</x:v>
+        <x:v>10.1111/1475-679x.70018</x:v>
       </x:c>
       <x:c r="N140" s="20" t="str">
-        <x:v>https://doi.org/10.1016/j.jacceco.2026.101911</x:v>
+        <x:v>https://doi.org/10.1111/1475-679x.70018</x:v>
       </x:c>
       <x:c r="O140" s="23" t="str">
         <x:v>打开来源</x:v>
       </x:c>
       <x:c r="P140" s="20" t="str"/>
-      <x:c r="Q140" s="20" t="str"/>
+      <x:c r="Q140" s="20" t="str">
+        <x:v>正式卷期为 2026 年 64(1)，首次在线为 2025-09-15。</x:v>
+      </x:c>
     </x:row>
     <x:row r="141" ht="46" customHeight="1">
       <x:c r="A141" s="12" t="str">
-        <x:v>P131</x:v>
+        <x:v>P129</x:v>
       </x:c>
       <x:c r="B141" s="18" t="str">
         <x:v>企业披露、财务会计与审计</x:v>
@@ -8077,35 +8202,35 @@
         <x:v>2026</x:v>
       </x:c>
       <x:c r="D141" s="24" t="d">
-        <x:v>2026-07-01T00:00:00.000Z</x:v>
+        <x:v>2026-06-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E141" s="14" t="str">
-        <x:v>JAE</x:v>
+        <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F141" s="20" t="str">
-        <x:v>Discussion of “Auditing smart contracts”: Assurance in the world of decentralized finance</x:v>
+        <x:v>The Role of Auditor Reputation in an Emerging Audit Marketplace: Evidence from Decentralized Finance (DeFi)</x:v>
       </x:c>
       <x:c r="G141" s="20" t="str">
-        <x:v>Andreas Park</x:v>
+        <x:v>W. Robert Knechel; Steven A. Maex; Hyun Jong Park</x:v>
       </x:c>
       <x:c r="H141" s="21" t="str">
-        <x:v>在线发表</x:v>
+        <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I141" s="20" t="str">
-        <x:v>对智能合约审计与 DeFi 鉴证的讨论</x:v>
+        <x:v>DeFi 审计市场中的审计师声誉</x:v>
       </x:c>
       <x:c r="J141" s="20" t="str">
-        <x:v>评论</x:v>
+        <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K141" s="20" t="str">
-        <x:v>未编入卷期</x:v>
+        <x:v>72(6): 5083-5105</x:v>
       </x:c>
       <x:c r="L141" s="22"/>
       <x:c r="M141" s="20" t="str">
-        <x:v>10.1016/j.jacceco.2026.101925</x:v>
+        <x:v>10.1287/mnsc.2023.02245</x:v>
       </x:c>
       <x:c r="N141" s="20" t="str">
-        <x:v>https://doi.org/10.1016/j.jacceco.2026.101925</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2023.02245</x:v>
       </x:c>
       <x:c r="O141" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -8114,94 +8239,92 @@
       <x:c r="Q141" s="20" t="str"/>
     </x:row>
     <x:row r="142" ht="46" customHeight="1">
-      <x:c r="A142" s="25" t="str">
-        <x:v>P132</x:v>
-      </x:c>
-      <x:c r="B142" s="34" t="str">
-        <x:v>市场操纵、非法活动、网络犯罪与税收</x:v>
-      </x:c>
-      <x:c r="C142" s="27" t="n">
-        <x:v>2018</x:v>
-      </x:c>
-      <x:c r="D142" s="28" t="d">
-        <x:v>2018-05-01T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="E142" s="29" t="str">
-        <x:v>JME</x:v>
-      </x:c>
-      <x:c r="F142" s="30" t="str">
-        <x:v>Price manipulation in the Bitcoin ecosystem</x:v>
-      </x:c>
-      <x:c r="G142" s="30" t="str">
-        <x:v>Neil Gandal; JT Hamrick; Tyler Moore; Tali Oberman</x:v>
-      </x:c>
-      <x:c r="H142" s="31" t="str">
-        <x:v>卷期发表</x:v>
-      </x:c>
-      <x:c r="I142" s="30" t="str">
-        <x:v>比特币交易所价格操纵</x:v>
-      </x:c>
-      <x:c r="J142" s="30" t="str">
-        <x:v>直接相关</x:v>
-      </x:c>
-      <x:c r="K142" s="30" t="str">
-        <x:v>95: 86-96</x:v>
-      </x:c>
-      <x:c r="L142" s="32"/>
-      <x:c r="M142" s="30" t="str">
-        <x:v>10.1016/j.jmoneco.2017.12.004</x:v>
-      </x:c>
-      <x:c r="N142" s="30" t="str">
-        <x:v>https://doi.org/10.1016/j.jmoneco.2017.12.004</x:v>
-      </x:c>
-      <x:c r="O142" s="33" t="str">
-        <x:v>打开来源</x:v>
-      </x:c>
-      <x:c r="P142" s="30" t="str"/>
-      <x:c r="Q142" s="30" t="str"/>
+      <x:c r="A142" s="12" t="str">
+        <x:v>P130</x:v>
+      </x:c>
+      <x:c r="B142" s="18" t="str">
+        <x:v>企业披露、财务会计与审计</x:v>
+      </x:c>
+      <x:c r="C142" s="15" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="D142" s="24" t="d">
+        <x:v>2026-07-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E142" s="14" t="str">
+        <x:v>JAE</x:v>
+      </x:c>
+      <x:c r="F142" s="20" t="str">
+        <x:v>Auditing smart contracts</x:v>
+      </x:c>
+      <x:c r="G142" s="20" t="str">
+        <x:v>Wayne Landsman; Evgeny Lyandres; Edward Maydew; Daniel Rabetti; Che Zhang</x:v>
+      </x:c>
+      <x:c r="H142" s="21" t="str">
+        <x:v>在线发表</x:v>
+      </x:c>
+      <x:c r="I142" s="20" t="str">
+        <x:v>DeFi 智能合约审计的决定因素与后果</x:v>
+      </x:c>
+      <x:c r="J142" s="20" t="str">
+        <x:v>直接相关</x:v>
+      </x:c>
+      <x:c r="K142" s="20" t="str">
+        <x:v>未编入卷期</x:v>
+      </x:c>
+      <x:c r="L142" s="22"/>
+      <x:c r="M142" s="20" t="str">
+        <x:v>10.1016/j.jacceco.2026.101911</x:v>
+      </x:c>
+      <x:c r="N142" s="20" t="str">
+        <x:v>https://doi.org/10.1016/j.jacceco.2026.101911</x:v>
+      </x:c>
+      <x:c r="O142" s="23" t="str">
+        <x:v>打开来源</x:v>
+      </x:c>
+      <x:c r="P142" s="20" t="str"/>
+      <x:c r="Q142" s="20" t="str"/>
     </x:row>
     <x:row r="143" ht="46" customHeight="1">
       <x:c r="A143" s="12" t="str">
-        <x:v>P133</x:v>
+        <x:v>P131</x:v>
       </x:c>
       <x:c r="B143" s="18" t="str">
-        <x:v>市场操纵、非法活动、网络犯罪与税收</x:v>
+        <x:v>企业披露、财务会计与审计</x:v>
       </x:c>
       <x:c r="C143" s="15" t="n">
-        <x:v>2019</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="D143" s="24" t="d">
-        <x:v>2019-05-01T00:00:00.000Z</x:v>
+        <x:v>2026-07-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E143" s="14" t="str">
-        <x:v>RFS</x:v>
+        <x:v>JAE</x:v>
       </x:c>
       <x:c r="F143" s="20" t="str">
-        <x:v>Sex, Drugs, and Bitcoin: How Much Illegal Activity Is Financed through Cryptocurrencies?</x:v>
+        <x:v>Discussion of “Auditing smart contracts”: Assurance in the world of decentralized finance</x:v>
       </x:c>
       <x:c r="G143" s="20" t="str">
-        <x:v>Sean Foley; Jonathan R Karlsen; Tālis J Putniņš</x:v>
+        <x:v>Andreas Park</x:v>
       </x:c>
       <x:c r="H143" s="21" t="str">
-        <x:v>卷期发表</x:v>
+        <x:v>在线发表</x:v>
       </x:c>
       <x:c r="I143" s="20" t="str">
-        <x:v>比特币非法活动的规模与资金流</x:v>
+        <x:v>对智能合约审计与 DeFi 鉴证的讨论</x:v>
       </x:c>
       <x:c r="J143" s="20" t="str">
-        <x:v>直接相关</x:v>
+        <x:v>评论</x:v>
       </x:c>
       <x:c r="K143" s="20" t="str">
-        <x:v>32(5): 1798-1853</x:v>
-      </x:c>
-      <x:c r="L143" s="22" t="d">
-        <x:v>2019-04-04T00:00:00.000Z</x:v>
-      </x:c>
+        <x:v>未编入卷期</x:v>
+      </x:c>
+      <x:c r="L143" s="22"/>
       <x:c r="M143" s="20" t="str">
-        <x:v>10.1093/rfs/hhz015</x:v>
+        <x:v>10.1016/j.jacceco.2026.101925</x:v>
       </x:c>
       <x:c r="N143" s="20" t="str">
-        <x:v>https://doi.org/10.1093/rfs/hhz015</x:v>
+        <x:v>https://doi.org/10.1016/j.jacceco.2026.101925</x:v>
       </x:c>
       <x:c r="O143" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -8210,96 +8333,94 @@
       <x:c r="Q143" s="20" t="str"/>
     </x:row>
     <x:row r="144" ht="46" customHeight="1">
-      <x:c r="A144" s="12" t="str">
-        <x:v>P134</x:v>
-      </x:c>
-      <x:c r="B144" s="18" t="str">
+      <x:c r="A144" s="25" t="str">
+        <x:v>P132</x:v>
+      </x:c>
+      <x:c r="B144" s="34" t="str">
         <x:v>市场操纵、非法活动、网络犯罪与税收</x:v>
       </x:c>
-      <x:c r="C144" s="15" t="n">
-        <x:v>2020</x:v>
-      </x:c>
-      <x:c r="D144" s="24" t="d">
-        <x:v>2020-08-01T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="E144" s="14" t="str">
-        <x:v>JF</x:v>
-      </x:c>
-      <x:c r="F144" s="20" t="str">
-        <x:v>Is Bitcoin Really Untethered?</x:v>
-      </x:c>
-      <x:c r="G144" s="20" t="str">
-        <x:v>John M. Griffin; Amin Shams</x:v>
-      </x:c>
-      <x:c r="H144" s="21" t="str">
-        <x:v>卷期发表</x:v>
-      </x:c>
-      <x:c r="I144" s="20" t="str">
-        <x:v>Tether 交易与比特币价格操纵</x:v>
-      </x:c>
-      <x:c r="J144" s="20" t="str">
-        <x:v>直接相关</x:v>
-      </x:c>
-      <x:c r="K144" s="20" t="str">
-        <x:v>75(4): 1913-1964</x:v>
-      </x:c>
-      <x:c r="L144" s="22" t="d">
-        <x:v>2020-06-15T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="M144" s="20" t="str">
-        <x:v>10.1111/jofi.12903</x:v>
-      </x:c>
-      <x:c r="N144" s="20" t="str">
-        <x:v>https://doi.org/10.1111/jofi.12903</x:v>
-      </x:c>
-      <x:c r="O144" s="23" t="str">
-        <x:v>打开来源</x:v>
-      </x:c>
-      <x:c r="P144" s="20" t="str"/>
-      <x:c r="Q144" s="20" t="str"/>
+      <x:c r="C144" s="27" t="n">
+        <x:v>2018</x:v>
+      </x:c>
+      <x:c r="D144" s="28" t="d">
+        <x:v>2018-05-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E144" s="29" t="str">
+        <x:v>JME</x:v>
+      </x:c>
+      <x:c r="F144" s="30" t="str">
+        <x:v>Price manipulation in the Bitcoin ecosystem</x:v>
+      </x:c>
+      <x:c r="G144" s="30" t="str">
+        <x:v>Neil Gandal; JT Hamrick; Tyler Moore; Tali Oberman</x:v>
+      </x:c>
+      <x:c r="H144" s="31" t="str">
+        <x:v>卷期发表</x:v>
+      </x:c>
+      <x:c r="I144" s="30" t="str">
+        <x:v>比特币交易所价格操纵</x:v>
+      </x:c>
+      <x:c r="J144" s="30" t="str">
+        <x:v>直接相关</x:v>
+      </x:c>
+      <x:c r="K144" s="30" t="str">
+        <x:v>95: 86-96</x:v>
+      </x:c>
+      <x:c r="L144" s="32"/>
+      <x:c r="M144" s="30" t="str">
+        <x:v>10.1016/j.jmoneco.2017.12.004</x:v>
+      </x:c>
+      <x:c r="N144" s="30" t="str">
+        <x:v>https://doi.org/10.1016/j.jmoneco.2017.12.004</x:v>
+      </x:c>
+      <x:c r="O144" s="33" t="str">
+        <x:v>打开来源</x:v>
+      </x:c>
+      <x:c r="P144" s="30" t="str"/>
+      <x:c r="Q144" s="30" t="str"/>
     </x:row>
     <x:row r="145" ht="46" customHeight="1">
       <x:c r="A145" s="12" t="str">
-        <x:v>P135</x:v>
+        <x:v>P133</x:v>
       </x:c>
       <x:c r="B145" s="18" t="str">
         <x:v>市场操纵、非法活动、网络犯罪与税收</x:v>
       </x:c>
       <x:c r="C145" s="15" t="n">
-        <x:v>2022</x:v>
+        <x:v>2019</x:v>
       </x:c>
       <x:c r="D145" s="24" t="d">
-        <x:v>2022-05-01T00:00:00.000Z</x:v>
+        <x:v>2019-05-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E145" s="14" t="str">
-        <x:v>JAR</x:v>
+        <x:v>RFS</x:v>
       </x:c>
       <x:c r="F145" s="20" t="str">
-        <x:v>Coins for Bombs: The Predictive Ability of On‐Chain Transfers for Terrorist Attacks</x:v>
+        <x:v>Sex, Drugs, and Bitcoin: How Much Illegal Activity Is Financed through Cryptocurrencies?</x:v>
       </x:c>
       <x:c r="G145" s="20" t="str">
-        <x:v>Dan Amiram; Bjørn N. Jørgensen; Daniel Rabetti</x:v>
+        <x:v>Sean Foley; Jonathan R Karlsen; Tālis J Putniņš</x:v>
       </x:c>
       <x:c r="H145" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I145" s="20" t="str">
-        <x:v>链上资金转移与恐怖袭击的预测</x:v>
+        <x:v>比特币非法活动的规模与资金流</x:v>
       </x:c>
       <x:c r="J145" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K145" s="20" t="str">
-        <x:v>60(2): 427-466</x:v>
+        <x:v>32(5): 1798-1853</x:v>
       </x:c>
       <x:c r="L145" s="22" t="d">
-        <x:v>2022-04-13T00:00:00.000Z</x:v>
+        <x:v>2019-04-04T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="M145" s="20" t="str">
-        <x:v>10.1111/1475-679x.12430</x:v>
+        <x:v>10.1093/rfs/hhz015</x:v>
       </x:c>
       <x:c r="N145" s="20" t="str">
-        <x:v>https://doi.org/10.1111/1475-679x.12430</x:v>
+        <x:v>https://doi.org/10.1093/rfs/hhz015</x:v>
       </x:c>
       <x:c r="O145" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -8309,44 +8430,46 @@
     </x:row>
     <x:row r="146" ht="46" customHeight="1">
       <x:c r="A146" s="12" t="str">
-        <x:v>P136</x:v>
+        <x:v>P134</x:v>
       </x:c>
       <x:c r="B146" s="18" t="str">
         <x:v>市场操纵、非法活动、网络犯罪与税收</x:v>
       </x:c>
       <x:c r="C146" s="15" t="n">
-        <x:v>2023</x:v>
+        <x:v>2020</x:v>
       </x:c>
       <x:c r="D146" s="24" t="d">
-        <x:v>2023-11-01T00:00:00.000Z</x:v>
+        <x:v>2020-08-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E146" s="14" t="str">
-        <x:v>JAE</x:v>
+        <x:v>JF</x:v>
       </x:c>
       <x:c r="F146" s="20" t="str">
-        <x:v>Comment on Cong et al., “Tax loss harvesting with cryptocurrencies”</x:v>
+        <x:v>Is Bitcoin Really Untethered?</x:v>
       </x:c>
       <x:c r="G146" s="20" t="str">
-        <x:v>Reuven Avi-Yonah</x:v>
+        <x:v>John M. Griffin; Amin Shams</x:v>
       </x:c>
       <x:c r="H146" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I146" s="20" t="str">
-        <x:v>对加密资产税损收割研究的税务评论</x:v>
+        <x:v>Tether 交易与比特币价格操纵</x:v>
       </x:c>
       <x:c r="J146" s="20" t="str">
-        <x:v>评论</x:v>
+        <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K146" s="20" t="str">
-        <x:v>76(2-3): 101612</x:v>
-      </x:c>
-      <x:c r="L146" s="22"/>
+        <x:v>75(4): 1913-1964</x:v>
+      </x:c>
+      <x:c r="L146" s="22" t="d">
+        <x:v>2020-06-15T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="M146" s="20" t="str">
-        <x:v>10.1016/j.jacceco.2023.101612</x:v>
+        <x:v>10.1111/jofi.12903</x:v>
       </x:c>
       <x:c r="N146" s="20" t="str">
-        <x:v>https://doi.org/10.1016/j.jacceco.2023.101612</x:v>
+        <x:v>https://doi.org/10.1111/jofi.12903</x:v>
       </x:c>
       <x:c r="O146" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -8356,44 +8479,46 @@
     </x:row>
     <x:row r="147" ht="46" customHeight="1">
       <x:c r="A147" s="12" t="str">
-        <x:v>P137</x:v>
+        <x:v>P135</x:v>
       </x:c>
       <x:c r="B147" s="18" t="str">
         <x:v>市场操纵、非法活动、网络犯罪与税收</x:v>
       </x:c>
       <x:c r="C147" s="15" t="n">
-        <x:v>2023</x:v>
+        <x:v>2022</x:v>
       </x:c>
       <x:c r="D147" s="24" t="d">
-        <x:v>2023-11-01T00:00:00.000Z</x:v>
+        <x:v>2022-05-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E147" s="14" t="str">
-        <x:v>Management Science</x:v>
+        <x:v>JAR</x:v>
       </x:c>
       <x:c r="F147" s="20" t="str">
-        <x:v>Crypto Wash Trading</x:v>
+        <x:v>Coins for Bombs: The Predictive Ability of On‐Chain Transfers for Terrorist Attacks</x:v>
       </x:c>
       <x:c r="G147" s="20" t="str">
-        <x:v>Lin William Cong; Xi Li; Ke Tang; Yang Yang</x:v>
+        <x:v>Dan Amiram; Bjørn N. Jørgensen; Daniel Rabetti</x:v>
       </x:c>
       <x:c r="H147" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I147" s="20" t="str">
-        <x:v>加密交易所虚假交易量与对刷</x:v>
+        <x:v>链上资金转移与恐怖袭击的预测</x:v>
       </x:c>
       <x:c r="J147" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K147" s="20" t="str">
-        <x:v>69(11): 6427-6454</x:v>
-      </x:c>
-      <x:c r="L147" s="22"/>
+        <x:v>60(2): 427-466</x:v>
+      </x:c>
+      <x:c r="L147" s="22" t="d">
+        <x:v>2022-04-13T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="M147" s="20" t="str">
-        <x:v>10.1287/mnsc.2021.02709</x:v>
+        <x:v>10.1111/1475-679x.12430</x:v>
       </x:c>
       <x:c r="N147" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2021.02709</x:v>
+        <x:v>https://doi.org/10.1111/1475-679x.12430</x:v>
       </x:c>
       <x:c r="O147" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -8403,7 +8528,7 @@
     </x:row>
     <x:row r="148" ht="46" customHeight="1">
       <x:c r="A148" s="12" t="str">
-        <x:v>P138</x:v>
+        <x:v>P136</x:v>
       </x:c>
       <x:c r="B148" s="18" t="str">
         <x:v>市场操纵、非法活动、网络犯罪与税收</x:v>
@@ -8418,29 +8543,29 @@
         <x:v>JAE</x:v>
       </x:c>
       <x:c r="F148" s="20" t="str">
-        <x:v>Tax-loss harvesting with cryptocurrencies</x:v>
+        <x:v>Comment on Cong et al., “Tax loss harvesting with cryptocurrencies”</x:v>
       </x:c>
       <x:c r="G148" s="20" t="str">
-        <x:v>Lin William Cong; Wayne Landsman; Edward Maydew; Daniel Rabetti</x:v>
+        <x:v>Reuven Avi-Yonah</x:v>
       </x:c>
       <x:c r="H148" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I148" s="20" t="str">
-        <x:v>加密资产税损收割与投资者交易</x:v>
+        <x:v>对加密资产税损收割研究的税务评论</x:v>
       </x:c>
       <x:c r="J148" s="20" t="str">
-        <x:v>直接相关</x:v>
+        <x:v>评论</x:v>
       </x:c>
       <x:c r="K148" s="20" t="str">
-        <x:v>76(2-3): 101607</x:v>
+        <x:v>76(2-3): 101612</x:v>
       </x:c>
       <x:c r="L148" s="22"/>
       <x:c r="M148" s="20" t="str">
-        <x:v>10.1016/j.jacceco.2023.101607</x:v>
+        <x:v>10.1016/j.jacceco.2023.101612</x:v>
       </x:c>
       <x:c r="N148" s="20" t="str">
-        <x:v>https://doi.org/10.1016/j.jacceco.2023.101607</x:v>
+        <x:v>https://doi.org/10.1016/j.jacceco.2023.101612</x:v>
       </x:c>
       <x:c r="O148" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -8450,44 +8575,44 @@
     </x:row>
     <x:row r="149" ht="46" customHeight="1">
       <x:c r="A149" s="12" t="str">
-        <x:v>P139</x:v>
+        <x:v>P137</x:v>
       </x:c>
       <x:c r="B149" s="18" t="str">
         <x:v>市场操纵、非法活动、网络犯罪与税收</x:v>
       </x:c>
       <x:c r="C149" s="15" t="n">
-        <x:v>2024</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="D149" s="24" t="d">
-        <x:v>2024-12-01T00:00:00.000Z</x:v>
+        <x:v>2023-11-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E149" s="14" t="str">
         <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F149" s="20" t="str">
-        <x:v>Direct Evidence of Bitcoin Wash Trading</x:v>
+        <x:v>Crypto Wash Trading</x:v>
       </x:c>
       <x:c r="G149" s="20" t="str">
-        <x:v>Arash Aloosh; Jiasun Li</x:v>
+        <x:v>Lin William Cong; Xi Li; Ke Tang; Yang Yang</x:v>
       </x:c>
       <x:c r="H149" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I149" s="20" t="str">
-        <x:v>比特币对刷交易的直接证据</x:v>
+        <x:v>加密交易所虚假交易量与对刷</x:v>
       </x:c>
       <x:c r="J149" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K149" s="20" t="str">
-        <x:v>70(12): 8875-8921</x:v>
+        <x:v>69(11): 6427-6454</x:v>
       </x:c>
       <x:c r="L149" s="22"/>
       <x:c r="M149" s="20" t="str">
-        <x:v>10.1287/mnsc.2021.01448</x:v>
+        <x:v>10.1287/mnsc.2021.02709</x:v>
       </x:c>
       <x:c r="N149" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2021.01448</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2021.02709</x:v>
       </x:c>
       <x:c r="O149" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -8497,44 +8622,44 @@
     </x:row>
     <x:row r="150" ht="46" customHeight="1">
       <x:c r="A150" s="12" t="str">
-        <x:v>P140</x:v>
+        <x:v>P138</x:v>
       </x:c>
       <x:c r="B150" s="18" t="str">
         <x:v>市场操纵、非法活动、网络犯罪与税收</x:v>
       </x:c>
       <x:c r="C150" s="15" t="n">
-        <x:v>2025</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="D150" s="24" t="d">
-        <x:v>2025-04-01T00:00:00.000Z</x:v>
+        <x:v>2023-11-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E150" s="14" t="str">
-        <x:v>Management Science</x:v>
+        <x:v>JAE</x:v>
       </x:c>
       <x:c r="F150" s="20" t="str">
-        <x:v>An Anatomy of Crypto-Enabled Cybercrimes</x:v>
+        <x:v>Tax-loss harvesting with cryptocurrencies</x:v>
       </x:c>
       <x:c r="G150" s="20" t="str">
-        <x:v>Will Cong; Campbell Harvey; Daniel Rabetti; Zong-Yu Wu</x:v>
+        <x:v>Lin William Cong; Wayne Landsman; Edward Maydew; Daniel Rabetti</x:v>
       </x:c>
       <x:c r="H150" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I150" s="20" t="str">
-        <x:v>加密资产支持的网络犯罪及链上资金追踪</x:v>
+        <x:v>加密资产税损收割与投资者交易</x:v>
       </x:c>
       <x:c r="J150" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K150" s="20" t="str">
-        <x:v>71(4): 3622-3633</x:v>
+        <x:v>76(2-3): 101607</x:v>
       </x:c>
       <x:c r="L150" s="22"/>
       <x:c r="M150" s="20" t="str">
-        <x:v>10.1287/mnsc.2023.03691</x:v>
+        <x:v>10.1016/j.jacceco.2023.101607</x:v>
       </x:c>
       <x:c r="N150" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2023.03691</x:v>
+        <x:v>https://doi.org/10.1016/j.jacceco.2023.101607</x:v>
       </x:c>
       <x:c r="O150" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -8544,44 +8669,44 @@
     </x:row>
     <x:row r="151" ht="46" customHeight="1">
       <x:c r="A151" s="12" t="str">
-        <x:v>P141</x:v>
+        <x:v>P139</x:v>
       </x:c>
       <x:c r="B151" s="18" t="str">
         <x:v>市场操纵、非法活动、网络犯罪与税收</x:v>
       </x:c>
       <x:c r="C151" s="15" t="n">
-        <x:v>2025</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="D151" s="24" t="d">
-        <x:v>2025-10-01T00:00:00.000Z</x:v>
+        <x:v>2024-12-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E151" s="14" t="str">
         <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F151" s="20" t="str">
-        <x:v>Trading Volume Manipulation and Competition Among Centralized Crypto Exchanges</x:v>
+        <x:v>Direct Evidence of Bitcoin Wash Trading</x:v>
       </x:c>
       <x:c r="G151" s="20" t="str">
-        <x:v>Dan Amiram; Evgeny Lyandres; Daniel Rabetti</x:v>
+        <x:v>Arash Aloosh; Jiasun Li</x:v>
       </x:c>
       <x:c r="H151" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I151" s="20" t="str">
-        <x:v>中心化加密交易所竞争与成交量操纵</x:v>
+        <x:v>比特币对刷交易的直接证据</x:v>
       </x:c>
       <x:c r="J151" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K151" s="20" t="str">
-        <x:v>71(10): 8604-8622</x:v>
+        <x:v>70(12): 8875-8921</x:v>
       </x:c>
       <x:c r="L151" s="22"/>
       <x:c r="M151" s="20" t="str">
-        <x:v>10.1287/mnsc.2021.02903</x:v>
+        <x:v>10.1287/mnsc.2021.01448</x:v>
       </x:c>
       <x:c r="N151" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2021.02903</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2021.01448</x:v>
       </x:c>
       <x:c r="O151" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -8591,7 +8716,7 @@
     </x:row>
     <x:row r="152" ht="46" customHeight="1">
       <x:c r="A152" s="12" t="str">
-        <x:v>P142</x:v>
+        <x:v>P140</x:v>
       </x:c>
       <x:c r="B152" s="18" t="str">
         <x:v>市场操纵、非法活动、网络犯罪与税收</x:v>
@@ -8600,35 +8725,35 @@
         <x:v>2025</x:v>
       </x:c>
       <x:c r="D152" s="24" t="d">
-        <x:v>2025-11-01T00:00:00.000Z</x:v>
+        <x:v>2025-04-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E152" s="14" t="str">
         <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F152" s="20" t="str">
-        <x:v>The Impact of Cryptocurrency on Cybersecurity</x:v>
+        <x:v>An Anatomy of Crypto-Enabled Cybercrimes</x:v>
       </x:c>
       <x:c r="G152" s="20" t="str">
-        <x:v>Terrence August; Duy Dao; Kihoon Kim; Marius Florin Niculescu</x:v>
+        <x:v>Will Cong; Campbell Harvey; Daniel Rabetti; Zong-Yu Wu</x:v>
       </x:c>
       <x:c r="H152" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I152" s="20" t="str">
-        <x:v>加密货币发展对网络安全激励的影响</x:v>
+        <x:v>加密资产支持的网络犯罪及链上资金追踪</x:v>
       </x:c>
       <x:c r="J152" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K152" s="20" t="str">
-        <x:v>71(11): 9606-9627</x:v>
+        <x:v>71(4): 3622-3633</x:v>
       </x:c>
       <x:c r="L152" s="22"/>
       <x:c r="M152" s="20" t="str">
-        <x:v>10.1287/mnsc.2023.00969</x:v>
+        <x:v>10.1287/mnsc.2023.03691</x:v>
       </x:c>
       <x:c r="N152" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2023.00969</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2023.03691</x:v>
       </x:c>
       <x:c r="O152" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -8637,94 +8762,92 @@
       <x:c r="Q152" s="20" t="str"/>
     </x:row>
     <x:row r="153" ht="46" customHeight="1">
-      <x:c r="A153" s="25" t="str">
-        <x:v>P143</x:v>
-      </x:c>
-      <x:c r="B153" s="34" t="str">
-        <x:v>供应链、企业应用与金融包容</x:v>
-      </x:c>
-      <x:c r="C153" s="27" t="n">
-        <x:v>2019</x:v>
-      </x:c>
-      <x:c r="D153" s="28" t="d">
-        <x:v>2019-05-01T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="E153" s="29" t="str">
-        <x:v>RFS</x:v>
-      </x:c>
-      <x:c r="F153" s="30" t="str">
-        <x:v>Blockchain-Based Settlement for Asset Trading</x:v>
-      </x:c>
-      <x:c r="G153" s="30" t="str">
-        <x:v>Jonathan Chiu; Thorsten V Koeppl</x:v>
-      </x:c>
-      <x:c r="H153" s="31" t="str">
-        <x:v>卷期发表</x:v>
-      </x:c>
-      <x:c r="I153" s="30" t="str">
-        <x:v>区块链在资产交易结算中的应用</x:v>
-      </x:c>
-      <x:c r="J153" s="30" t="str">
-        <x:v>直接相关</x:v>
-      </x:c>
-      <x:c r="K153" s="30" t="str">
-        <x:v>32(5): 1716-1753</x:v>
-      </x:c>
-      <x:c r="L153" s="32" t="d">
-        <x:v>2019-04-04T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="M153" s="30" t="str">
-        <x:v>10.1093/rfs/hhy122</x:v>
-      </x:c>
-      <x:c r="N153" s="30" t="str">
-        <x:v>https://doi.org/10.1093/rfs/hhy122</x:v>
-      </x:c>
-      <x:c r="O153" s="33" t="str">
-        <x:v>打开来源</x:v>
-      </x:c>
-      <x:c r="P153" s="30" t="str"/>
-      <x:c r="Q153" s="30" t="str"/>
+      <x:c r="A153" s="12" t="str">
+        <x:v>P141</x:v>
+      </x:c>
+      <x:c r="B153" s="18" t="str">
+        <x:v>市场操纵、非法活动、网络犯罪与税收</x:v>
+      </x:c>
+      <x:c r="C153" s="15" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="D153" s="24" t="d">
+        <x:v>2025-10-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E153" s="14" t="str">
+        <x:v>Management Science</x:v>
+      </x:c>
+      <x:c r="F153" s="20" t="str">
+        <x:v>Trading Volume Manipulation and Competition Among Centralized Crypto Exchanges</x:v>
+      </x:c>
+      <x:c r="G153" s="20" t="str">
+        <x:v>Dan Amiram; Evgeny Lyandres; Daniel Rabetti</x:v>
+      </x:c>
+      <x:c r="H153" s="21" t="str">
+        <x:v>卷期发表</x:v>
+      </x:c>
+      <x:c r="I153" s="20" t="str">
+        <x:v>中心化加密交易所竞争与成交量操纵</x:v>
+      </x:c>
+      <x:c r="J153" s="20" t="str">
+        <x:v>直接相关</x:v>
+      </x:c>
+      <x:c r="K153" s="20" t="str">
+        <x:v>71(10): 8604-8622</x:v>
+      </x:c>
+      <x:c r="L153" s="22"/>
+      <x:c r="M153" s="20" t="str">
+        <x:v>10.1287/mnsc.2021.02903</x:v>
+      </x:c>
+      <x:c r="N153" s="20" t="str">
+        <x:v>https://doi.org/10.1287/mnsc.2021.02903</x:v>
+      </x:c>
+      <x:c r="O153" s="23" t="str">
+        <x:v>打开来源</x:v>
+      </x:c>
+      <x:c r="P153" s="20" t="str"/>
+      <x:c r="Q153" s="20" t="str"/>
     </x:row>
     <x:row r="154" ht="46" customHeight="1">
       <x:c r="A154" s="12" t="str">
-        <x:v>P144</x:v>
+        <x:v>P142</x:v>
       </x:c>
       <x:c r="B154" s="18" t="str">
-        <x:v>供应链、企业应用与金融包容</x:v>
+        <x:v>市场操纵、非法活动、网络犯罪与税收</x:v>
       </x:c>
       <x:c r="C154" s="15" t="n">
-        <x:v>2020</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="D154" s="24" t="d">
-        <x:v>2020-10-01T00:00:00.000Z</x:v>
+        <x:v>2025-11-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E154" s="14" t="str">
         <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F154" s="20" t="str">
-        <x:v>On the Financing Benefits of Supply Chain Transparency and Blockchain Adoption</x:v>
+        <x:v>The Impact of Cryptocurrency on Cybersecurity</x:v>
       </x:c>
       <x:c r="G154" s="20" t="str">
-        <x:v>Jiri Chod; Nikolaos Trichakis; Gerry Tsoukalas; Henry Aspegren; Mark Weber</x:v>
+        <x:v>Terrence August; Duy Dao; Kihoon Kim; Marius Florin Niculescu</x:v>
       </x:c>
       <x:c r="H154" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I154" s="20" t="str">
-        <x:v>供应链透明度、区块链采用与融资收益</x:v>
+        <x:v>加密货币发展对网络安全激励的影响</x:v>
       </x:c>
       <x:c r="J154" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K154" s="20" t="str">
-        <x:v>66(10): 4378-4396</x:v>
+        <x:v>71(11): 9606-9627</x:v>
       </x:c>
       <x:c r="L154" s="22"/>
       <x:c r="M154" s="20" t="str">
-        <x:v>10.1287/mnsc.2019.3434</x:v>
+        <x:v>10.1287/mnsc.2023.00969</x:v>
       </x:c>
       <x:c r="N154" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2019.3434</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2023.00969</x:v>
       </x:c>
       <x:c r="O154" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -8733,92 +8856,94 @@
       <x:c r="Q154" s="20" t="str"/>
     </x:row>
     <x:row r="155" ht="46" customHeight="1">
-      <x:c r="A155" s="12" t="str">
-        <x:v>P145</x:v>
-      </x:c>
-      <x:c r="B155" s="18" t="str">
+      <x:c r="A155" s="25" t="str">
+        <x:v>P143</x:v>
+      </x:c>
+      <x:c r="B155" s="34" t="str">
         <x:v>供应链、企业应用与金融包容</x:v>
       </x:c>
-      <x:c r="C155" s="15" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="D155" s="24" t="d">
-        <x:v>2023-03-01T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="E155" s="14" t="str">
-        <x:v>Management Science</x:v>
-      </x:c>
-      <x:c r="F155" s="20" t="str">
-        <x:v>Impact of Traceability Technology Adoption in Food Supply Chain Networks</x:v>
-      </x:c>
-      <x:c r="G155" s="20" t="str">
-        <x:v>Lingxiu Dong; Puping (Phil) Jiang; Fasheng Xu</x:v>
-      </x:c>
-      <x:c r="H155" s="21" t="str">
-        <x:v>卷期发表</x:v>
-      </x:c>
-      <x:c r="I155" s="20" t="str">
-        <x:v>食品供应链中区块链等追溯技术的采用</x:v>
-      </x:c>
-      <x:c r="J155" s="20" t="str">
-        <x:v>直接相关</x:v>
-      </x:c>
-      <x:c r="K155" s="20" t="str">
-        <x:v>69(3): 1518-1535</x:v>
-      </x:c>
-      <x:c r="L155" s="22"/>
-      <x:c r="M155" s="20" t="str">
-        <x:v>10.1287/mnsc.2022.4440</x:v>
-      </x:c>
-      <x:c r="N155" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2022.4440</x:v>
-      </x:c>
-      <x:c r="O155" s="23" t="str">
-        <x:v>打开来源</x:v>
-      </x:c>
-      <x:c r="P155" s="20" t="str"/>
-      <x:c r="Q155" s="20" t="str"/>
+      <x:c r="C155" s="27" t="n">
+        <x:v>2019</x:v>
+      </x:c>
+      <x:c r="D155" s="28" t="d">
+        <x:v>2019-05-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E155" s="29" t="str">
+        <x:v>RFS</x:v>
+      </x:c>
+      <x:c r="F155" s="30" t="str">
+        <x:v>Blockchain-Based Settlement for Asset Trading</x:v>
+      </x:c>
+      <x:c r="G155" s="30" t="str">
+        <x:v>Jonathan Chiu; Thorsten V Koeppl</x:v>
+      </x:c>
+      <x:c r="H155" s="31" t="str">
+        <x:v>卷期发表</x:v>
+      </x:c>
+      <x:c r="I155" s="30" t="str">
+        <x:v>区块链在资产交易结算中的应用</x:v>
+      </x:c>
+      <x:c r="J155" s="30" t="str">
+        <x:v>直接相关</x:v>
+      </x:c>
+      <x:c r="K155" s="30" t="str">
+        <x:v>32(5): 1716-1753</x:v>
+      </x:c>
+      <x:c r="L155" s="32" t="d">
+        <x:v>2019-04-04T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="M155" s="30" t="str">
+        <x:v>10.1093/rfs/hhy122</x:v>
+      </x:c>
+      <x:c r="N155" s="30" t="str">
+        <x:v>https://doi.org/10.1093/rfs/hhy122</x:v>
+      </x:c>
+      <x:c r="O155" s="33" t="str">
+        <x:v>打开来源</x:v>
+      </x:c>
+      <x:c r="P155" s="30" t="str"/>
+      <x:c r="Q155" s="30" t="str"/>
     </x:row>
     <x:row r="156" ht="46" customHeight="1">
       <x:c r="A156" s="12" t="str">
-        <x:v>P146</x:v>
+        <x:v>P144</x:v>
       </x:c>
       <x:c r="B156" s="18" t="str">
         <x:v>供应链、企业应用与金融包容</x:v>
       </x:c>
       <x:c r="C156" s="15" t="n">
-        <x:v>2023</x:v>
+        <x:v>2020</x:v>
       </x:c>
       <x:c r="D156" s="24" t="d">
-        <x:v>2023-06-01T00:00:00.000Z</x:v>
+        <x:v>2020-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E156" s="14" t="str">
         <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F156" s="20" t="str">
-        <x:v>Economics of Permissioned Blockchain Adoption</x:v>
+        <x:v>On the Financing Benefits of Supply Chain Transparency and Blockchain Adoption</x:v>
       </x:c>
       <x:c r="G156" s="20" t="str">
-        <x:v>Garud Iyengar; Fahad Saleh; Jay Sethuraman; Wenjun Wang</x:v>
+        <x:v>Jiri Chod; Nikolaos Trichakis; Gerry Tsoukalas; Henry Aspegren; Mark Weber</x:v>
       </x:c>
       <x:c r="H156" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I156" s="20" t="str">
-        <x:v>许可链采用的经济条件与激励</x:v>
+        <x:v>供应链透明度、区块链采用与融资收益</x:v>
       </x:c>
       <x:c r="J156" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K156" s="20" t="str">
-        <x:v>69(6): 3415-3436</x:v>
+        <x:v>66(10): 4378-4396</x:v>
       </x:c>
       <x:c r="L156" s="22"/>
       <x:c r="M156" s="20" t="str">
-        <x:v>10.1287/mnsc.2022.4532</x:v>
+        <x:v>10.1287/mnsc.2019.3434</x:v>
       </x:c>
       <x:c r="N156" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2022.4532</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2019.3434</x:v>
       </x:c>
       <x:c r="O156" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -8828,44 +8953,44 @@
     </x:row>
     <x:row r="157" ht="46" customHeight="1">
       <x:c r="A157" s="12" t="str">
-        <x:v>P147</x:v>
+        <x:v>P145</x:v>
       </x:c>
       <x:c r="B157" s="18" t="str">
         <x:v>供应链、企业应用与金融包容</x:v>
       </x:c>
       <x:c r="C157" s="15" t="n">
-        <x:v>2024</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="D157" s="24" t="d">
-        <x:v>2024-01-01T00:00:00.000Z</x:v>
+        <x:v>2023-03-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E157" s="14" t="str">
         <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F157" s="20" t="str">
-        <x:v>The Economic Value of Blockchain Applications: Early Evidence from Asset-Backed Securities</x:v>
+        <x:v>Impact of Traceability Technology Adoption in Food Supply Chain Networks</x:v>
       </x:c>
       <x:c r="G157" s="20" t="str">
-        <x:v>Xia Chen; Qiang Cheng; Ting Luo</x:v>
+        <x:v>Lingxiu Dong; Puping (Phil) Jiang; Fasheng Xu</x:v>
       </x:c>
       <x:c r="H157" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I157" s="20" t="str">
-        <x:v>资产支持证券中的区块链应用价值</x:v>
+        <x:v>食品供应链中区块链等追溯技术的采用</x:v>
       </x:c>
       <x:c r="J157" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K157" s="20" t="str">
-        <x:v>70(1): 439-463</x:v>
+        <x:v>69(3): 1518-1535</x:v>
       </x:c>
       <x:c r="L157" s="22"/>
       <x:c r="M157" s="20" t="str">
-        <x:v>10.1287/mnsc.2023.4671</x:v>
+        <x:v>10.1287/mnsc.2022.4440</x:v>
       </x:c>
       <x:c r="N157" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2023.4671</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2022.4440</x:v>
       </x:c>
       <x:c r="O157" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -8875,44 +9000,44 @@
     </x:row>
     <x:row r="158" ht="46" customHeight="1">
       <x:c r="A158" s="12" t="str">
-        <x:v>P148</x:v>
+        <x:v>P146</x:v>
       </x:c>
       <x:c r="B158" s="18" t="str">
         <x:v>供应链、企业应用与金融包容</x:v>
       </x:c>
       <x:c r="C158" s="15" t="n">
-        <x:v>2024</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="D158" s="24" t="d">
-        <x:v>2024-05-01T00:00:00.000Z</x:v>
+        <x:v>2023-06-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E158" s="14" t="str">
         <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F158" s="20" t="str">
-        <x:v>Supply Chain Transparency and Blockchain Design</x:v>
+        <x:v>Economics of Permissioned Blockchain Adoption</x:v>
       </x:c>
       <x:c r="G158" s="20" t="str">
-        <x:v>Yao Cui; Vishal Gaur; Jingchen Liu</x:v>
+        <x:v>Garud Iyengar; Fahad Saleh; Jay Sethuraman; Wenjun Wang</x:v>
       </x:c>
       <x:c r="H158" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I158" s="20" t="str">
-        <x:v>供应链透明度与区块链设计选择</x:v>
+        <x:v>许可链采用的经济条件与激励</x:v>
       </x:c>
       <x:c r="J158" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K158" s="20" t="str">
-        <x:v>70(5): 3245-3263</x:v>
+        <x:v>69(6): 3415-3436</x:v>
       </x:c>
       <x:c r="L158" s="22"/>
       <x:c r="M158" s="20" t="str">
-        <x:v>10.1287/mnsc.2023.4851</x:v>
+        <x:v>10.1287/mnsc.2022.4532</x:v>
       </x:c>
       <x:c r="N158" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2023.4851</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2022.4532</x:v>
       </x:c>
       <x:c r="O158" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -8922,7 +9047,7 @@
     </x:row>
     <x:row r="159" ht="46" customHeight="1">
       <x:c r="A159" s="12" t="str">
-        <x:v>P149</x:v>
+        <x:v>P147</x:v>
       </x:c>
       <x:c r="B159" s="18" t="str">
         <x:v>供应链、企业应用与金融包容</x:v>
@@ -8931,88 +9056,82 @@
         <x:v>2024</x:v>
       </x:c>
       <x:c r="D159" s="24" t="d">
-        <x:v>2024-09-01T00:00:00.000Z</x:v>
+        <x:v>2024-01-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E159" s="14" t="str">
         <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F159" s="20" t="str">
-        <x:v>Blockchain Adoption in a Supply Chain with Manufacturer Market Power</x:v>
+        <x:v>The Economic Value of Blockchain Applications: Early Evidence from Asset-Backed Securities</x:v>
       </x:c>
       <x:c r="G159" s="20" t="str">
-        <x:v>Garud Iyengar; Fahad Saleh; Jay Sethuraman; Wenjun Wang</x:v>
+        <x:v>Xia Chen; Qiang Cheng; Ting Luo</x:v>
       </x:c>
       <x:c r="H159" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I159" s="20" t="str">
-        <x:v>制造商市场势力与供应链区块链采用</x:v>
+        <x:v>资产支持证券中的区块链应用价值</x:v>
       </x:c>
       <x:c r="J159" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K159" s="20" t="str">
-        <x:v>70(9): 6158-6178</x:v>
-      </x:c>
-      <x:c r="L159" s="22" t="d">
-        <x:v>2023-10-27T00:00:00.000Z</x:v>
-      </x:c>
+        <x:v>70(1): 439-463</x:v>
+      </x:c>
+      <x:c r="L159" s="22"/>
       <x:c r="M159" s="20" t="str">
-        <x:v>10.1287/mnsc.2022.02505</x:v>
+        <x:v>10.1287/mnsc.2023.4671</x:v>
       </x:c>
       <x:c r="N159" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2022.02505</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2023.4671</x:v>
       </x:c>
       <x:c r="O159" s="23" t="str">
         <x:v>打开来源</x:v>
       </x:c>
-      <x:c r="P159" s="20" t="str">
-        <x:v>https://pubsonline.informs.org/doi/abs/10.1287/mnsc.2022.02505</x:v>
-      </x:c>
-      <x:c r="Q159" s="20" t="str">
-        <x:v>Crossref 仍只有 2023 年在线信息；期刊页面已列 70(9):6158-6178，按 2024 年卷期收录。</x:v>
-      </x:c>
+      <x:c r="P159" s="20" t="str"/>
+      <x:c r="Q159" s="20" t="str"/>
     </x:row>
     <x:row r="160" ht="46" customHeight="1">
       <x:c r="A160" s="12" t="str">
-        <x:v>P150</x:v>
+        <x:v>P148</x:v>
       </x:c>
       <x:c r="B160" s="18" t="str">
         <x:v>供应链、企业应用与金融包容</x:v>
       </x:c>
       <x:c r="C160" s="15" t="n">
-        <x:v>2025</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="D160" s="24" t="d">
-        <x:v>2025-08-01T00:00:00.000Z</x:v>
+        <x:v>2024-05-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E160" s="14" t="str">
         <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F160" s="20" t="str">
-        <x:v>The Blockchain Newsvendor: Value of Freshness Transparency and Smart Contracts</x:v>
+        <x:v>Supply Chain Transparency and Blockchain Design</x:v>
       </x:c>
       <x:c r="G160" s="20" t="str">
-        <x:v>N. Bora Keskin; Chenghuai Li; Jing-Sheng Song</x:v>
+        <x:v>Yao Cui; Vishal Gaur; Jingchen Liu</x:v>
       </x:c>
       <x:c r="H160" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I160" s="20" t="str">
-        <x:v>生鲜供应链透明度、报童模型与智能合约</x:v>
+        <x:v>供应链透明度与区块链设计选择</x:v>
       </x:c>
       <x:c r="J160" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K160" s="20" t="str">
-        <x:v>71(8): 6666-6682</x:v>
+        <x:v>70(5): 3245-3263</x:v>
       </x:c>
       <x:c r="L160" s="22"/>
       <x:c r="M160" s="20" t="str">
-        <x:v>10.1287/mnsc.2021.02949</x:v>
+        <x:v>10.1287/mnsc.2023.4851</x:v>
       </x:c>
       <x:c r="N160" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2021.02949</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2023.4851</x:v>
       </x:c>
       <x:c r="O160" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -9022,93 +9141,97 @@
     </x:row>
     <x:row r="161" ht="46" customHeight="1">
       <x:c r="A161" s="12" t="str">
-        <x:v>P151</x:v>
+        <x:v>P149</x:v>
       </x:c>
       <x:c r="B161" s="18" t="str">
         <x:v>供应链、企业应用与金融包容</x:v>
       </x:c>
       <x:c r="C161" s="15" t="n">
-        <x:v>2025</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="D161" s="24" t="d">
-        <x:v>2025-09-01T00:00:00.000Z</x:v>
+        <x:v>2024-09-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E161" s="14" t="str">
-        <x:v>ISR</x:v>
+        <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F161" s="20" t="str">
-        <x:v>And No One Gets the Short End of the Stick: A Blockchain-Based Approach to Solving the Two-Sided Opportunism Problem in Interorganizational Information Sharing</x:v>
+        <x:v>Blockchain Adoption in a Supply Chain with Manufacturer Market Power</x:v>
       </x:c>
       <x:c r="G161" s="20" t="str">
-        <x:v>Lukas Florian Bossler; Arne Buchwald; Kai Spohrer</x:v>
+        <x:v>Garud Iyengar; Fahad Saleh; Jay Sethuraman; Wenjun Wang</x:v>
       </x:c>
       <x:c r="H161" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I161" s="20" t="str">
-        <x:v>区块链缓解组织间信息共享的双边机会主义</x:v>
+        <x:v>制造商市场势力与供应链区块链采用</x:v>
       </x:c>
       <x:c r="J161" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K161" s="20" t="str">
-        <x:v>36(3): 1565-1586</x:v>
-      </x:c>
-      <x:c r="L161" s="22"/>
+        <x:v>70(9): 6158-6178</x:v>
+      </x:c>
+      <x:c r="L161" s="22" t="d">
+        <x:v>2023-10-27T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="M161" s="20" t="str">
-        <x:v>10.1287/isre.2022.0065</x:v>
+        <x:v>10.1287/mnsc.2022.02505</x:v>
       </x:c>
       <x:c r="N161" s="20" t="str">
-        <x:v>https://doi.org/10.1287/isre.2022.0065</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2022.02505</x:v>
       </x:c>
       <x:c r="O161" s="23" t="str">
         <x:v>打开来源</x:v>
       </x:c>
-      <x:c r="P161" s="20" t="str"/>
-      <x:c r="Q161" s="20" t="str"/>
+      <x:c r="P161" s="20" t="str">
+        <x:v>https://pubsonline.informs.org/doi/abs/10.1287/mnsc.2022.02505</x:v>
+      </x:c>
+      <x:c r="Q161" s="20" t="str">
+        <x:v>Crossref 仍只有 2023 年在线信息；期刊页面已列 70(9):6158-6178，按 2024 年卷期收录。</x:v>
+      </x:c>
     </x:row>
     <x:row r="162" ht="46" customHeight="1">
       <x:c r="A162" s="12" t="str">
-        <x:v>P152</x:v>
+        <x:v>P150</x:v>
       </x:c>
       <x:c r="B162" s="18" t="str">
         <x:v>供应链、企业应用与金融包容</x:v>
       </x:c>
       <x:c r="C162" s="15" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="D162" s="16" t="d">
-        <x:v>2026-05-13T00:00:00.000Z</x:v>
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="D162" s="24" t="d">
+        <x:v>2025-08-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E162" s="14" t="str">
         <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F162" s="20" t="str">
-        <x:v>Financial Inclusion via Blockchain: Evidence from a Natural Experiment</x:v>
+        <x:v>The Blockchain Newsvendor: Value of Freshness Transparency and Smart Contracts</x:v>
       </x:c>
       <x:c r="G162" s="20" t="str">
-        <x:v>Shangrong Jiang; Yuze Li; Shouyang Wang</x:v>
+        <x:v>N. Bora Keskin; Chenghuai Li; Jing-Sheng Song</x:v>
       </x:c>
       <x:c r="H162" s="21" t="str">
-        <x:v>在线发表</x:v>
+        <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I162" s="20" t="str">
-        <x:v>区块链征信真实性与金融包容的自然实验</x:v>
+        <x:v>生鲜供应链透明度、报童模型与智能合约</x:v>
       </x:c>
       <x:c r="J162" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K162" s="20" t="str">
-        <x:v>未编入卷期</x:v>
-      </x:c>
-      <x:c r="L162" s="22" t="d">
-        <x:v>2026-05-13T00:00:00.000Z</x:v>
-      </x:c>
+        <x:v>71(8): 6666-6682</x:v>
+      </x:c>
+      <x:c r="L162" s="22"/>
       <x:c r="M162" s="20" t="str">
-        <x:v>10.1287/mnsc.2023.02303</x:v>
+        <x:v>10.1287/mnsc.2021.02949</x:v>
       </x:c>
       <x:c r="N162" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2023.02303</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2021.02949</x:v>
       </x:c>
       <x:c r="O162" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -9118,44 +9241,44 @@
     </x:row>
     <x:row r="163" ht="46" customHeight="1">
       <x:c r="A163" s="12" t="str">
-        <x:v>P153</x:v>
+        <x:v>P151</x:v>
       </x:c>
       <x:c r="B163" s="18" t="str">
         <x:v>供应链、企业应用与金融包容</x:v>
       </x:c>
       <x:c r="C163" s="15" t="n">
-        <x:v>2026</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="D163" s="24" t="d">
-        <x:v>2026-08-01T00:00:00.000Z</x:v>
+        <x:v>2025-09-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E163" s="14" t="str">
-        <x:v>Management Science</x:v>
+        <x:v>ISR</x:v>
       </x:c>
       <x:c r="F163" s="20" t="str">
-        <x:v>Behavioral Simulation of Blockchain-Enabled Market for Supplier Capacity Trading Among Retailers</x:v>
+        <x:v>And No One Gets the Short End of the Stick: A Blockchain-Based Approach to Solving the Two-Sided Opportunism Problem in Interorganizational Information Sharing</x:v>
       </x:c>
       <x:c r="G163" s="20" t="str">
-        <x:v>Kai Wendt; Volodymyr Babich; Daniel Hellwig; Arnd Huchzermeier</x:v>
+        <x:v>Lukas Florian Bossler; Arne Buchwald; Kai Spohrer</x:v>
       </x:c>
       <x:c r="H163" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I163" s="20" t="str">
-        <x:v>区块链赋能的零售商供应能力交易</x:v>
+        <x:v>区块链缓解组织间信息共享的双边机会主义</x:v>
       </x:c>
       <x:c r="J163" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K163" s="20" t="str">
-        <x:v>72(8): 6762-6791</x:v>
+        <x:v>36(3): 1565-1586</x:v>
       </x:c>
       <x:c r="L163" s="22"/>
       <x:c r="M163" s="20" t="str">
-        <x:v>10.1287/mnsc.2023.03771</x:v>
+        <x:v>10.1287/isre.2022.0065</x:v>
       </x:c>
       <x:c r="N163" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2023.03771</x:v>
+        <x:v>https://doi.org/10.1287/isre.2022.0065</x:v>
       </x:c>
       <x:c r="O163" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -9164,92 +9287,94 @@
       <x:c r="Q163" s="20" t="str"/>
     </x:row>
     <x:row r="164" ht="46" customHeight="1">
-      <x:c r="A164" s="25" t="str">
-        <x:v>P154</x:v>
-      </x:c>
-      <x:c r="B164" s="34" t="str">
-        <x:v>NFT、艺术品与创作者经济</x:v>
-      </x:c>
-      <x:c r="C164" s="27" t="n">
-        <x:v>2020</x:v>
-      </x:c>
-      <x:c r="D164" s="28" t="d">
-        <x:v>2020-10-01T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="E164" s="29" t="str">
+      <x:c r="A164" s="12" t="str">
+        <x:v>P152</x:v>
+      </x:c>
+      <x:c r="B164" s="18" t="str">
+        <x:v>供应链、企业应用与金融包容</x:v>
+      </x:c>
+      <x:c r="C164" s="15" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="D164" s="16" t="d">
+        <x:v>2026-05-13T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E164" s="14" t="str">
         <x:v>Management Science</x:v>
       </x:c>
-      <x:c r="F164" s="30" t="str">
-        <x:v>Fractional Equity, Blockchain, and the Future of Creative Work</x:v>
-      </x:c>
-      <x:c r="G164" s="30" t="str">
-        <x:v>Amy Whitaker; Roman Kräussl</x:v>
-      </x:c>
-      <x:c r="H164" s="31" t="str">
-        <x:v>卷期发表</x:v>
-      </x:c>
-      <x:c r="I164" s="30" t="str">
-        <x:v>艺术品权益分割、区块链与创作者收益</x:v>
-      </x:c>
-      <x:c r="J164" s="30" t="str">
-        <x:v>直接相关</x:v>
-      </x:c>
-      <x:c r="K164" s="30" t="str">
-        <x:v>66(10): 4594-4611</x:v>
-      </x:c>
-      <x:c r="L164" s="32"/>
-      <x:c r="M164" s="30" t="str">
-        <x:v>10.1287/mnsc.2020.3633</x:v>
-      </x:c>
-      <x:c r="N164" s="30" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2020.3633</x:v>
-      </x:c>
-      <x:c r="O164" s="33" t="str">
-        <x:v>打开来源</x:v>
-      </x:c>
-      <x:c r="P164" s="30" t="str"/>
-      <x:c r="Q164" s="30" t="str"/>
+      <x:c r="F164" s="20" t="str">
+        <x:v>Financial Inclusion via Blockchain: Evidence from a Natural Experiment</x:v>
+      </x:c>
+      <x:c r="G164" s="20" t="str">
+        <x:v>Shangrong Jiang; Yuze Li; Shouyang Wang</x:v>
+      </x:c>
+      <x:c r="H164" s="21" t="str">
+        <x:v>在线发表</x:v>
+      </x:c>
+      <x:c r="I164" s="20" t="str">
+        <x:v>区块链征信真实性与金融包容的自然实验</x:v>
+      </x:c>
+      <x:c r="J164" s="20" t="str">
+        <x:v>直接相关</x:v>
+      </x:c>
+      <x:c r="K164" s="20" t="str">
+        <x:v>未编入卷期</x:v>
+      </x:c>
+      <x:c r="L164" s="22" t="d">
+        <x:v>2026-05-13T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="M164" s="20" t="str">
+        <x:v>10.1287/mnsc.2023.02303</x:v>
+      </x:c>
+      <x:c r="N164" s="20" t="str">
+        <x:v>https://doi.org/10.1287/mnsc.2023.02303</x:v>
+      </x:c>
+      <x:c r="O164" s="23" t="str">
+        <x:v>打开来源</x:v>
+      </x:c>
+      <x:c r="P164" s="20" t="str"/>
+      <x:c r="Q164" s="20" t="str"/>
     </x:row>
     <x:row r="165" ht="46" customHeight="1">
       <x:c r="A165" s="12" t="str">
-        <x:v>P155</x:v>
+        <x:v>P153</x:v>
       </x:c>
       <x:c r="B165" s="18" t="str">
-        <x:v>NFT、艺术品与创作者经济</x:v>
+        <x:v>供应链、企业应用与金融包容</x:v>
       </x:c>
       <x:c r="C165" s="15" t="n">
-        <x:v>2025</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="D165" s="24" t="d">
-        <x:v>2025-09-01T00:00:00.000Z</x:v>
+        <x:v>2026-08-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E165" s="14" t="str">
-        <x:v>ISR</x:v>
+        <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F165" s="20" t="str">
-        <x:v>Resale Royalty in Non-Fungible Token Marketplaces: Blessing or Burden for Creators and Platforms?</x:v>
+        <x:v>Behavioral Simulation of Blockchain-Enabled Market for Supplier Capacity Trading Among Retailers</x:v>
       </x:c>
       <x:c r="G165" s="20" t="str">
-        <x:v>Murat M. Tunc; Hasan Cavusoglu; Zhiqiang (Eric) Zheng</x:v>
+        <x:v>Kai Wendt; Volodymyr Babich; Daniel Hellwig; Arnd Huchzermeier</x:v>
       </x:c>
       <x:c r="H165" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I165" s="20" t="str">
-        <x:v>NFT 二次销售版税对创作者与平台的影响</x:v>
+        <x:v>区块链赋能的零售商供应能力交易</x:v>
       </x:c>
       <x:c r="J165" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K165" s="20" t="str">
-        <x:v>36(3): 1543-1564</x:v>
+        <x:v>72(8): 6762-6791</x:v>
       </x:c>
       <x:c r="L165" s="22"/>
       <x:c r="M165" s="20" t="str">
-        <x:v>10.1287/isre.2023.0035</x:v>
+        <x:v>10.1287/mnsc.2023.03771</x:v>
       </x:c>
       <x:c r="N165" s="20" t="str">
-        <x:v>https://doi.org/10.1287/isre.2023.0035</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2023.03771</x:v>
       </x:c>
       <x:c r="O165" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -9258,96 +9383,92 @@
       <x:c r="Q165" s="20" t="str"/>
     </x:row>
     <x:row r="166" ht="46" customHeight="1">
-      <x:c r="A166" s="12" t="str">
-        <x:v>P156</x:v>
-      </x:c>
-      <x:c r="B166" s="18" t="str">
+      <x:c r="A166" s="25" t="str">
+        <x:v>P154</x:v>
+      </x:c>
+      <x:c r="B166" s="34" t="str">
         <x:v>NFT、艺术品与创作者经济</x:v>
       </x:c>
-      <x:c r="C166" s="15" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="D166" s="16" t="d">
-        <x:v>2026-03-04T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="E166" s="14" t="str">
-        <x:v>MISQ</x:v>
-      </x:c>
-      <x:c r="F166" s="20" t="str">
-        <x:v>Extending the Digital Divide: The Role of Unequal Analytical Abilities</x:v>
-      </x:c>
-      <x:c r="G166" s="20" t="str">
-        <x:v>Hong Zhang; Zhiqiang (Eric) Zheng; Amit Mehra</x:v>
-      </x:c>
-      <x:c r="H166" s="21" t="str">
-        <x:v>在线发表</x:v>
-      </x:c>
-      <x:c r="I166" s="20" t="str">
-        <x:v>NFT 市场上的分析能力差异与交易表现</x:v>
-      </x:c>
-      <x:c r="J166" s="20" t="str">
-        <x:v>加密场景</x:v>
-      </x:c>
-      <x:c r="K166" s="20" t="str">
-        <x:v>未编入卷期</x:v>
-      </x:c>
-      <x:c r="L166" s="22" t="d">
-        <x:v>2026-03-04T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="M166" s="20" t="str">
-        <x:v>10.25300/misq/2026/19079</x:v>
-      </x:c>
-      <x:c r="N166" s="20" t="str">
-        <x:v>https://doi.org/10.25300/MISQ/2026/19079</x:v>
-      </x:c>
-      <x:c r="O166" s="23" t="str">
-        <x:v>打开来源</x:v>
-      </x:c>
-      <x:c r="P166" s="20" t="str"/>
-      <x:c r="Q166" s="20" t="str"/>
+      <x:c r="C166" s="27" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="D166" s="28" t="d">
+        <x:v>2020-10-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E166" s="29" t="str">
+        <x:v>Management Science</x:v>
+      </x:c>
+      <x:c r="F166" s="30" t="str">
+        <x:v>Fractional Equity, Blockchain, and the Future of Creative Work</x:v>
+      </x:c>
+      <x:c r="G166" s="30" t="str">
+        <x:v>Amy Whitaker; Roman Kräussl</x:v>
+      </x:c>
+      <x:c r="H166" s="31" t="str">
+        <x:v>卷期发表</x:v>
+      </x:c>
+      <x:c r="I166" s="30" t="str">
+        <x:v>艺术品权益分割、区块链与创作者收益</x:v>
+      </x:c>
+      <x:c r="J166" s="30" t="str">
+        <x:v>直接相关</x:v>
+      </x:c>
+      <x:c r="K166" s="30" t="str">
+        <x:v>66(10): 4594-4611</x:v>
+      </x:c>
+      <x:c r="L166" s="32"/>
+      <x:c r="M166" s="30" t="str">
+        <x:v>10.1287/mnsc.2020.3633</x:v>
+      </x:c>
+      <x:c r="N166" s="30" t="str">
+        <x:v>https://doi.org/10.1287/mnsc.2020.3633</x:v>
+      </x:c>
+      <x:c r="O166" s="33" t="str">
+        <x:v>打开来源</x:v>
+      </x:c>
+      <x:c r="P166" s="30" t="str"/>
+      <x:c r="Q166" s="30" t="str"/>
     </x:row>
     <x:row r="167" ht="46" customHeight="1">
       <x:c r="A167" s="12" t="str">
-        <x:v>P157</x:v>
+        <x:v>P155</x:v>
       </x:c>
       <x:c r="B167" s="18" t="str">
         <x:v>NFT、艺术品与创作者经济</x:v>
       </x:c>
       <x:c r="C167" s="15" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="D167" s="16" t="d">
-        <x:v>2026-04-21T00:00:00.000Z</x:v>
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="D167" s="24" t="d">
+        <x:v>2025-09-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E167" s="14" t="str">
         <x:v>ISR</x:v>
       </x:c>
       <x:c r="F167" s="20" t="str">
-        <x:v>The Market Consequences of Perceived Strategic Generosity: An Empirical Examination of NFT Charity Fundraisers</x:v>
+        <x:v>Resale Royalty in Non-Fungible Token Marketplaces: Blessing or Burden for Creators and Platforms?</x:v>
       </x:c>
       <x:c r="G167" s="20" t="str">
-        <x:v>Chen Liang; Murat Tunç; Gordon Burtch</x:v>
+        <x:v>Murat M. Tunc; Hasan Cavusoglu; Zhiqiang (Eric) Zheng</x:v>
       </x:c>
       <x:c r="H167" s="21" t="str">
-        <x:v>在线发表</x:v>
+        <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I167" s="20" t="str">
-        <x:v>NFT 慈善募资中的战略慷慨及市场反应</x:v>
+        <x:v>NFT 二次销售版税对创作者与平台的影响</x:v>
       </x:c>
       <x:c r="J167" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K167" s="20" t="str">
-        <x:v>未编入卷期</x:v>
-      </x:c>
-      <x:c r="L167" s="22" t="d">
-        <x:v>2026-04-21T00:00:00.000Z</x:v>
-      </x:c>
+        <x:v>36(3): 1543-1564</x:v>
+      </x:c>
+      <x:c r="L167" s="22"/>
       <x:c r="M167" s="20" t="str">
-        <x:v>10.1287/isre.2024.1004</x:v>
+        <x:v>10.1287/isre.2023.0035</x:v>
       </x:c>
       <x:c r="N167" s="20" t="str">
-        <x:v>https://doi.org/10.1287/isre.2024.1004</x:v>
+        <x:v>https://doi.org/10.1287/isre.2023.0035</x:v>
       </x:c>
       <x:c r="O167" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -9357,7 +9478,7 @@
     </x:row>
     <x:row r="168" ht="46" customHeight="1">
       <x:c r="A168" s="12" t="str">
-        <x:v>P158</x:v>
+        <x:v>P156</x:v>
       </x:c>
       <x:c r="B168" s="18" t="str">
         <x:v>NFT、艺术品与创作者经济</x:v>
@@ -9366,37 +9487,37 @@
         <x:v>2026</x:v>
       </x:c>
       <x:c r="D168" s="16" t="d">
-        <x:v>2026-08-04T00:00:00.000Z</x:v>
+        <x:v>2026-03-04T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E168" s="14" t="str">
-        <x:v>Management Science</x:v>
+        <x:v>MISQ</x:v>
       </x:c>
       <x:c r="F168" s="20" t="str">
-        <x:v>From Canvas to Blockchain: Impact of Royalties on Art Market Efficiency</x:v>
+        <x:v>Extending the Digital Divide: The Role of Unequal Analytical Abilities</x:v>
       </x:c>
       <x:c r="G168" s="20" t="str">
-        <x:v>Xinyu Cao; Jieteng Chen; T. Tony Ke</x:v>
+        <x:v>Hong Zhang; Zhiqiang (Eric) Zheng; Amit Mehra</x:v>
       </x:c>
       <x:c r="H168" s="21" t="str">
         <x:v>在线发表</x:v>
       </x:c>
       <x:c r="I168" s="20" t="str">
-        <x:v>区块链艺术品版税与市场效率</x:v>
+        <x:v>NFT 市场上的分析能力差异与交易表现</x:v>
       </x:c>
       <x:c r="J168" s="20" t="str">
-        <x:v>直接相关</x:v>
+        <x:v>加密场景</x:v>
       </x:c>
       <x:c r="K168" s="20" t="str">
         <x:v>未编入卷期</x:v>
       </x:c>
       <x:c r="L168" s="22" t="d">
-        <x:v>2026-08-04T00:00:00.000Z</x:v>
+        <x:v>2026-03-04T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="M168" s="20" t="str">
-        <x:v>10.1287/mnsc.2023.03810</x:v>
+        <x:v>10.25300/misq/2026/19079</x:v>
       </x:c>
       <x:c r="N168" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2023.03810</x:v>
+        <x:v>https://doi.org/10.25300/MISQ/2026/19079</x:v>
       </x:c>
       <x:c r="O168" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -9406,7 +9527,7 @@
     </x:row>
     <x:row r="169" ht="46" customHeight="1">
       <x:c r="A169" s="12" t="str">
-        <x:v>P159</x:v>
+        <x:v>P157</x:v>
       </x:c>
       <x:c r="B169" s="18" t="str">
         <x:v>NFT、艺术品与创作者经济</x:v>
@@ -9414,36 +9535,38 @@
       <x:c r="C169" s="15" t="n">
         <x:v>2026</x:v>
       </x:c>
-      <x:c r="D169" s="24" t="d">
-        <x:v>2026-09-01T00:00:00.000Z</x:v>
+      <x:c r="D169" s="16" t="d">
+        <x:v>2026-04-21T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E169" s="14" t="str">
         <x:v>ISR</x:v>
       </x:c>
       <x:c r="F169" s="20" t="str">
-        <x:v>NFT Disruption in Platform Competition: Evidence from Trading Card Collectibles</x:v>
+        <x:v>The Market Consequences of Perceived Strategic Generosity: An Empirical Examination of NFT Charity Fundraisers</x:v>
       </x:c>
       <x:c r="G169" s="20" t="str">
-        <x:v>Ioannis Filippos Kanellopoulos; Dominik Gutt; Ting Li</x:v>
+        <x:v>Chen Liang; Murat Tunç; Gordon Burtch</x:v>
       </x:c>
       <x:c r="H169" s="21" t="str">
-        <x:v>卷期发表</x:v>
+        <x:v>在线发表</x:v>
       </x:c>
       <x:c r="I169" s="20" t="str">
-        <x:v>NFT 对收藏卡交易平台竞争的影响</x:v>
+        <x:v>NFT 慈善募资中的战略慷慨及市场反应</x:v>
       </x:c>
       <x:c r="J169" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K169" s="20" t="str">
-        <x:v>37(3): 1596-1620</x:v>
-      </x:c>
-      <x:c r="L169" s="22"/>
+        <x:v>未编入卷期</x:v>
+      </x:c>
+      <x:c r="L169" s="22" t="d">
+        <x:v>2026-04-21T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="M169" s="20" t="str">
-        <x:v>10.1287/isre.2024.0829</x:v>
+        <x:v>10.1287/isre.2024.1004</x:v>
       </x:c>
       <x:c r="N169" s="20" t="str">
-        <x:v>https://doi.org/10.1287/isre.2024.0829</x:v>
+        <x:v>https://doi.org/10.1287/isre.2024.1004</x:v>
       </x:c>
       <x:c r="O169" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -9453,7 +9576,7 @@
     </x:row>
     <x:row r="170" ht="46" customHeight="1">
       <x:c r="A170" s="12" t="str">
-        <x:v>P160</x:v>
+        <x:v>P158</x:v>
       </x:c>
       <x:c r="B170" s="18" t="str">
         <x:v>NFT、艺术品与创作者经济</x:v>
@@ -9461,36 +9584,38 @@
       <x:c r="C170" s="15" t="n">
         <x:v>2026</x:v>
       </x:c>
-      <x:c r="D170" s="24" t="d">
-        <x:v>2026-10-01T00:00:00.000Z</x:v>
+      <x:c r="D170" s="16" t="d">
+        <x:v>2026-08-04T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E170" s="14" t="str">
         <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F170" s="20" t="str">
-        <x:v>Chasing Market Growth and Matching Performance in Two-Sided Platforms: Evidence from the Lazy-Minting Policy in an NFT Marketplace</x:v>
+        <x:v>From Canvas to Blockchain: Impact of Royalties on Art Market Efficiency</x:v>
       </x:c>
       <x:c r="G170" s="20" t="str">
-        <x:v>Hong Zhang; Hongchang Wang; Amit Mehra; Zhiqiang (Eric) Zheng</x:v>
+        <x:v>Xinyu Cao; Jieteng Chen; T. Tony Ke</x:v>
       </x:c>
       <x:c r="H170" s="21" t="str">
-        <x:v>卷期发表</x:v>
+        <x:v>在线发表</x:v>
       </x:c>
       <x:c r="I170" s="20" t="str">
-        <x:v>NFT 市场懒铸造政策、增长与匹配效率</x:v>
+        <x:v>区块链艺术品版税与市场效率</x:v>
       </x:c>
       <x:c r="J170" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K170" s="20" t="str">
-        <x:v>72(10): 8416-8439</x:v>
-      </x:c>
-      <x:c r="L170" s="22"/>
+        <x:v>未编入卷期</x:v>
+      </x:c>
+      <x:c r="L170" s="22" t="d">
+        <x:v>2026-08-04T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="M170" s="20" t="str">
-        <x:v>10.1287/mnsc.2022.03573</x:v>
+        <x:v>10.1287/mnsc.2023.03810</x:v>
       </x:c>
       <x:c r="N170" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2022.03573</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2023.03810</x:v>
       </x:c>
       <x:c r="O170" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -9499,55 +9624,149 @@
       <x:c r="Q170" s="20" t="str"/>
     </x:row>
     <x:row r="171" ht="46" customHeight="1">
-      <x:c r="A171" s="25" t="str">
+      <x:c r="A171" s="12" t="str">
+        <x:v>P159</x:v>
+      </x:c>
+      <x:c r="B171" s="18" t="str">
+        <x:v>NFT、艺术品与创作者经济</x:v>
+      </x:c>
+      <x:c r="C171" s="15" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="D171" s="24" t="d">
+        <x:v>2026-09-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E171" s="14" t="str">
+        <x:v>ISR</x:v>
+      </x:c>
+      <x:c r="F171" s="20" t="str">
+        <x:v>NFT Disruption in Platform Competition: Evidence from Trading Card Collectibles</x:v>
+      </x:c>
+      <x:c r="G171" s="20" t="str">
+        <x:v>Ioannis Filippos Kanellopoulos; Dominik Gutt; Ting Li</x:v>
+      </x:c>
+      <x:c r="H171" s="21" t="str">
+        <x:v>卷期发表</x:v>
+      </x:c>
+      <x:c r="I171" s="20" t="str">
+        <x:v>NFT 对收藏卡交易平台竞争的影响</x:v>
+      </x:c>
+      <x:c r="J171" s="20" t="str">
+        <x:v>直接相关</x:v>
+      </x:c>
+      <x:c r="K171" s="20" t="str">
+        <x:v>37(3): 1596-1620</x:v>
+      </x:c>
+      <x:c r="L171" s="22"/>
+      <x:c r="M171" s="20" t="str">
+        <x:v>10.1287/isre.2024.0829</x:v>
+      </x:c>
+      <x:c r="N171" s="20" t="str">
+        <x:v>https://doi.org/10.1287/isre.2024.0829</x:v>
+      </x:c>
+      <x:c r="O171" s="23" t="str">
+        <x:v>打开来源</x:v>
+      </x:c>
+      <x:c r="P171" s="20" t="str"/>
+      <x:c r="Q171" s="20" t="str"/>
+    </x:row>
+    <x:row r="172" ht="46" customHeight="1">
+      <x:c r="A172" s="12" t="str">
+        <x:v>P160</x:v>
+      </x:c>
+      <x:c r="B172" s="18" t="str">
+        <x:v>NFT、艺术品与创作者经济</x:v>
+      </x:c>
+      <x:c r="C172" s="15" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="D172" s="24" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E172" s="14" t="str">
+        <x:v>Management Science</x:v>
+      </x:c>
+      <x:c r="F172" s="20" t="str">
+        <x:v>Chasing Market Growth and Matching Performance in Two-Sided Platforms: Evidence from the Lazy-Minting Policy in an NFT Marketplace</x:v>
+      </x:c>
+      <x:c r="G172" s="20" t="str">
+        <x:v>Hong Zhang; Hongchang Wang; Amit Mehra; Zhiqiang (Eric) Zheng</x:v>
+      </x:c>
+      <x:c r="H172" s="21" t="str">
+        <x:v>卷期发表</x:v>
+      </x:c>
+      <x:c r="I172" s="20" t="str">
+        <x:v>NFT 市场懒铸造政策、增长与匹配效率</x:v>
+      </x:c>
+      <x:c r="J172" s="20" t="str">
+        <x:v>直接相关</x:v>
+      </x:c>
+      <x:c r="K172" s="20" t="str">
+        <x:v>72(10): 8416-8439</x:v>
+      </x:c>
+      <x:c r="L172" s="22"/>
+      <x:c r="M172" s="20" t="str">
+        <x:v>10.1287/mnsc.2022.03573</x:v>
+      </x:c>
+      <x:c r="N172" s="20" t="str">
+        <x:v>https://doi.org/10.1287/mnsc.2022.03573</x:v>
+      </x:c>
+      <x:c r="O172" s="23" t="str">
+        <x:v>打开来源</x:v>
+      </x:c>
+      <x:c r="P172" s="20" t="str"/>
+      <x:c r="Q172" s="20" t="str"/>
+    </x:row>
+    <x:row r="173" ht="46" customHeight="1">
+      <x:c r="A173" s="25" t="str">
         <x:v>P161</x:v>
       </x:c>
-      <x:c r="B171" s="34" t="str">
+      <x:c r="B173" s="34" t="str">
         <x:v>综述与研究议程</x:v>
       </x:c>
-      <x:c r="C171" s="27" t="n">
+      <x:c r="C173" s="27" t="n">
         <x:v>2023</x:v>
       </x:c>
-      <x:c r="D171" s="28" t="d">
+      <x:c r="D173" s="28" t="d">
         <x:v>2023-11-01T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E171" s="29" t="str">
+      <x:c r="E173" s="29" t="str">
         <x:v>Management Science</x:v>
       </x:c>
-      <x:c r="F171" s="30" t="str">
+      <x:c r="F173" s="30" t="str">
         <x:v>Advances in Blockchain and Crypto Economics</x:v>
       </x:c>
-      <x:c r="G171" s="30" t="str">
+      <x:c r="G173" s="30" t="str">
         <x:v>Bruno Biais; Agostino Capponi; Lin William Cong; Vishal Gaur; Kay Giesecke</x:v>
       </x:c>
-      <x:c r="H171" s="31" t="str">
-        <x:v>卷期发表</x:v>
-      </x:c>
-      <x:c r="I171" s="30" t="str">
+      <x:c r="H173" s="31" t="str">
+        <x:v>卷期发表</x:v>
+      </x:c>
+      <x:c r="I173" s="30" t="str">
         <x:v>区块链与加密经济学专辑导论及研究议程</x:v>
       </x:c>
-      <x:c r="J171" s="30" t="str">
+      <x:c r="J173" s="30" t="str">
         <x:v>综述导论</x:v>
       </x:c>
-      <x:c r="K171" s="30" t="str">
+      <x:c r="K173" s="30" t="str">
         <x:v>69(11): 6417-6426</x:v>
       </x:c>
-      <x:c r="L171" s="32"/>
-      <x:c r="M171" s="30" t="str">
+      <x:c r="L173" s="32"/>
+      <x:c r="M173" s="30" t="str">
         <x:v>10.1287/mnsc.2023.intro.v69.n11</x:v>
       </x:c>
-      <x:c r="N171" s="30" t="str">
+      <x:c r="N173" s="30" t="str">
         <x:v>https://doi.org/10.1287/mnsc.2023.intro.v69.n11</x:v>
       </x:c>
-      <x:c r="O171" s="33" t="str">
-        <x:v>打开来源</x:v>
-      </x:c>
-      <x:c r="P171" s="30" t="str"/>
-      <x:c r="Q171" s="30" t="str"/>
+      <x:c r="O173" s="33" t="str">
+        <x:v>打开来源</x:v>
+      </x:c>
+      <x:c r="P173" s="30" t="str"/>
+      <x:c r="Q173" s="30" t="str"/>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="H6:H171">
-    <x:cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="已接收"/>
+  <x:conditionalFormatting sqref="H6:H173">
+    <x:cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="已接收"/>
   </x:conditionalFormatting>
   <x:hyperlinks>
     <x:hyperlink ref="O6" r:id="Hyperlink6" display="打开来源"/>
@@ -9716,10 +9935,12 @@
     <x:hyperlink ref="O169" r:id="Hyperlink169" display="打开来源"/>
     <x:hyperlink ref="O170" r:id="Hyperlink170" display="打开来源"/>
     <x:hyperlink ref="O171" r:id="Hyperlink171" display="打开来源"/>
+    <x:hyperlink ref="O172" r:id="Hyperlink172" display="打开来源"/>
+    <x:hyperlink ref="O173" r:id="Hyperlink173" display="打开来源"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart r:id="R6b0dc0b0005d4395"/>
+    <x:tablePart r:id="R5288ea5c385540f8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9831,145 +10052,151 @@
       <x:c r="Q4" s="2"/>
     </x:row>
     <x:row r="5" ht="29" customHeight="1">
-      <x:c r="A5" s="9" t="str">
+      <x:c r="A5" s="72" t="str">
         <x:v>编号</x:v>
       </x:c>
-      <x:c r="B5" s="10" t="str">
+      <x:c r="B5" s="73" t="str">
         <x:v>研究主题</x:v>
       </x:c>
-      <x:c r="C5" s="10" t="str">
+      <x:c r="C5" s="73" t="str">
         <x:v>年份</x:v>
       </x:c>
-      <x:c r="D5" s="10" t="str">
+      <x:c r="D5" s="73" t="str">
         <x:v>年月或日期</x:v>
       </x:c>
-      <x:c r="E5" s="10" t="str">
+      <x:c r="E5" s="73" t="str">
         <x:v>期刊</x:v>
       </x:c>
-      <x:c r="F5" s="10" t="str">
+      <x:c r="F5" s="73" t="str">
         <x:v>英文题名</x:v>
       </x:c>
-      <x:c r="G5" s="10" t="str">
+      <x:c r="G5" s="73" t="str">
         <x:v>完整作者</x:v>
       </x:c>
-      <x:c r="H5" s="10" t="str">
+      <x:c r="H5" s="73" t="str">
         <x:v>发表状态</x:v>
       </x:c>
-      <x:c r="I5" s="10" t="str">
+      <x:c r="I5" s="73" t="str">
         <x:v>研究焦点</x:v>
       </x:c>
-      <x:c r="J5" s="10" t="str">
+      <x:c r="J5" s="73" t="str">
         <x:v>文献类型</x:v>
       </x:c>
-      <x:c r="K5" s="10" t="str">
+      <x:c r="K5" s="73" t="str">
         <x:v>卷期与页码</x:v>
       </x:c>
-      <x:c r="L5" s="10" t="str">
+      <x:c r="L5" s="73" t="str">
         <x:v>首次在线日期</x:v>
       </x:c>
-      <x:c r="M5" s="10" t="str">
+      <x:c r="M5" s="73" t="str">
         <x:v>DOI</x:v>
       </x:c>
-      <x:c r="N5" s="10" t="str">
+      <x:c r="N5" s="73" t="str">
         <x:v>来源网址</x:v>
       </x:c>
-      <x:c r="O5" s="10" t="str">
-        <x:v>打开来源</x:v>
-      </x:c>
-      <x:c r="P5" s="10" t="str">
+      <x:c r="O5" s="73" t="str">
+        <x:v>打开来源</x:v>
+      </x:c>
+      <x:c r="P5" s="73" t="str">
         <x:v>补充核验来源</x:v>
       </x:c>
-      <x:c r="Q5" s="11" t="str">
+      <x:c r="Q5" s="74" t="str">
         <x:v>核验说明</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="46" customHeight="1">
+    <x:row r="6" ht="64" customHeight="1">
       <x:c r="A6" s="25" t="str">
-        <x:v>R01</x:v>
+        <x:v>R08</x:v>
       </x:c>
       <x:c r="B6" s="34" t="str">
-        <x:v>交易费用、支付与区块链扩容</x:v>
+        <x:v>货币竞争、加密资产估值与收益</x:v>
       </x:c>
       <x:c r="C6" s="27" t="n">
-        <x:v>2020</x:v>
+        <x:v>2019</x:v>
       </x:c>
       <x:c r="D6" s="28" t="d">
-        <x:v>2020-05-01T00:00:00.000Z</x:v>
+        <x:v>2019-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E6" s="29" t="str">
-        <x:v>Management Science</x:v>
+        <x:v>JME</x:v>
       </x:c>
       <x:c r="F6" s="30" t="str">
-        <x:v>Channel Auctions</x:v>
+        <x:v>On the equivalence of private and public money</x:v>
       </x:c>
       <x:c r="G6" s="30" t="str">
-        <x:v>Eduardo M. Azevedo; David M. Pennock; Bo Waggoner; E. Glen Weyl</x:v>
+        <x:v>Markus K. Brunnermeier; Dirk Niepelt</x:v>
       </x:c>
       <x:c r="H6" s="31" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I6" s="30" t="str">
-        <x:v>拍卖机制与信息获取；区块链交易排序是其应用之一</x:v>
+        <x:v>公私货币等价的一般理论；第 5.3 节讨论加密货币、许可链与 PoW 成本</x:v>
       </x:c>
       <x:c r="J6" s="30" t="str">
         <x:v>相关理论</x:v>
       </x:c>
       <x:c r="K6" s="30" t="str">
-        <x:v>66(5): 2075-2082</x:v>
-      </x:c>
-      <x:c r="L6" s="32"/>
+        <x:v>106: 27-41</x:v>
+      </x:c>
+      <x:c r="L6" s="32" t="d">
+        <x:v>2019-07-06T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="M6" s="30" t="str">
-        <x:v>10.1287/mnsc.2019.3487</x:v>
+        <x:v>10.1016/j.jmoneco.2019.07.004</x:v>
       </x:c>
       <x:c r="N6" s="30" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2019.3487</x:v>
+        <x:v>https://doi.org/10.1016/j.jmoneco.2019.07.004</x:v>
       </x:c>
       <x:c r="O6" s="33" t="str">
         <x:v>打开来源</x:v>
       </x:c>
-      <x:c r="P6" s="30" t="str"/>
-      <x:c r="Q6" s="30" t="str"/>
+      <x:c r="P6" s="30" t="str">
+        <x:v>https://mfm.uchicago.edu/wp-content/uploads/2020/06/Brunnermeier-Niepelt-On-the-Equivalence-of-Private-and-Public-Money.pdf</x:v>
+      </x:c>
+      <x:c r="Q6" s="30" t="str">
+        <x:v>v3 五刊定向复核补入边界相关。JME 正式卷期 106 (2019-10):27-41；公开期刊版首页确认接收 2019-07-05、首次在线 2019-07-06。第 5.3 节 Cryptocurrency 分析许可链与 PoW 对公私货币等价的约束。主体是一般货币等价理论，单列且不计入主目录。</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="46" customHeight="1">
       <x:c r="A7" s="25" t="str">
-        <x:v>R02</x:v>
+        <x:v>R01</x:v>
       </x:c>
       <x:c r="B7" s="34" t="str">
-        <x:v>智能合约、DAO、社区与制度治理</x:v>
+        <x:v>交易费用、支付与区块链扩容</x:v>
       </x:c>
       <x:c r="C7" s="27" t="n">
-        <x:v>2022</x:v>
+        <x:v>2020</x:v>
       </x:c>
       <x:c r="D7" s="28" t="d">
-        <x:v>2022-08-01T00:00:00.000Z</x:v>
+        <x:v>2020-05-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E7" s="29" t="str">
         <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F7" s="30" t="str">
-        <x:v>Optimal Management of Evolving Hierarchies</x:v>
+        <x:v>Channel Auctions</x:v>
       </x:c>
       <x:c r="G7" s="30" t="str">
-        <x:v>Jens Leth Hougaard; Juan D. Moreno-Ternero; Lars Peter Østerdal</x:v>
+        <x:v>Eduardo M. Azevedo; David M. Pennock; Bo Waggoner; E. Glen Weyl</x:v>
       </x:c>
       <x:c r="H7" s="31" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I7" s="30" t="str">
-        <x:v>一般层级组织的激励分配；区块链是潜在应用</x:v>
+        <x:v>拍卖机制与信息获取；区块链交易排序是其应用之一</x:v>
       </x:c>
       <x:c r="J7" s="30" t="str">
         <x:v>相关理论</x:v>
       </x:c>
       <x:c r="K7" s="30" t="str">
-        <x:v>68(8): 6024-6038</x:v>
+        <x:v>66(5): 2075-2082</x:v>
       </x:c>
       <x:c r="L7" s="32"/>
       <x:c r="M7" s="30" t="str">
-        <x:v>10.1287/mnsc.2021.4185</x:v>
+        <x:v>10.1287/mnsc.2019.3487</x:v>
       </x:c>
       <x:c r="N7" s="30" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2021.4185</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2019.3487</x:v>
       </x:c>
       <x:c r="O7" s="33" t="str">
         <x:v>打开来源</x:v>
@@ -9977,189 +10204,203 @@
       <x:c r="P7" s="30" t="str"/>
       <x:c r="Q7" s="30" t="str"/>
     </x:row>
-    <x:row r="8" ht="46" customHeight="1">
+    <x:row r="8" ht="77" customHeight="1">
       <x:c r="A8" s="12" t="str">
-        <x:v>R03</x:v>
+        <x:v>R09</x:v>
       </x:c>
       <x:c r="B8" s="18" t="str">
-        <x:v>智能合约、DAO、社区与制度治理</x:v>
+        <x:v>交易费用、支付与区块链扩容</x:v>
       </x:c>
       <x:c r="C8" s="15" t="n">
-        <x:v>2023</x:v>
+        <x:v>2021</x:v>
       </x:c>
       <x:c r="D8" s="24" t="d">
-        <x:v>2023-05-01T00:00:00.000Z</x:v>
+        <x:v>2021-07-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E8" s="14" t="str">
-        <x:v>AER</x:v>
+        <x:v>JPE</x:v>
       </x:c>
       <x:c r="F8" s="20" t="str">
-        <x:v>Smart Contracts and the Coase Conjecture</x:v>
+        <x:v>Privacy as a Public Good: A Case for Electronic Cash</x:v>
       </x:c>
       <x:c r="G8" s="20" t="str">
-        <x:v>Thomas Brzustowski; Alkis Georgiadis-Harris; Balázs Szentes</x:v>
+        <x:v>Rodney J. Garratt; Maarten R. C. van Oordt</x:v>
       </x:c>
       <x:c r="H8" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I8" s="20" t="str">
-        <x:v>动态智能合约与耐用品垄断；一般契约理论，不直接建模区块链</x:v>
+        <x:v>支付隐私的公共品属性；公开作者稿讨论比特币作为电子现金替代方案的局限</x:v>
       </x:c>
       <x:c r="J8" s="20" t="str">
         <x:v>相关理论</x:v>
       </x:c>
       <x:c r="K8" s="20" t="str">
-        <x:v>113(5): 1334-1359</x:v>
-      </x:c>
-      <x:c r="L8" s="22"/>
+        <x:v>129(7): 2157-2180</x:v>
+      </x:c>
+      <x:c r="L8" s="22" t="d">
+        <x:v>2021-05-26T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="M8" s="20" t="str">
-        <x:v>10.1257/aer.20220357</x:v>
+        <x:v>10.1086/714133</x:v>
       </x:c>
       <x:c r="N8" s="20" t="str">
-        <x:v>https://doi.org/10.1257/aer.20220357</x:v>
+        <x:v>https://doi.org/10.1086/714133</x:v>
       </x:c>
       <x:c r="O8" s="23" t="str">
         <x:v>打开来源</x:v>
       </x:c>
-      <x:c r="P8" s="20" t="str"/>
-      <x:c r="Q8" s="20" t="str"/>
-    </x:row>
-    <x:row r="9" ht="46" customHeight="1">
-      <x:c r="A9" s="25" t="str">
-        <x:v>R04</x:v>
-      </x:c>
-      <x:c r="B9" s="34" t="str">
-        <x:v>供应链、企业应用与金融包容</x:v>
-      </x:c>
-      <x:c r="C9" s="27" t="n">
-        <x:v>2022</x:v>
-      </x:c>
-      <x:c r="D9" s="28" t="d">
-        <x:v>2022-09-01T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="E9" s="29" t="str">
-        <x:v>ISR</x:v>
-      </x:c>
-      <x:c r="F9" s="30" t="str">
-        <x:v>The Dark Side of Technological Modularity: Opportunistic Information Hiding During Interorganizational System Adoption</x:v>
-      </x:c>
-      <x:c r="G9" s="30" t="str">
-        <x:v>Sanjith Gopalakrishnan; Moksh Matta; Hasan Cavusoglu</x:v>
-      </x:c>
-      <x:c r="H9" s="31" t="str">
-        <x:v>卷期发表</x:v>
-      </x:c>
-      <x:c r="I9" s="30" t="str">
-        <x:v>模块化与组织间系统采用；区块链是应用场景之一</x:v>
-      </x:c>
-      <x:c r="J9" s="30" t="str">
+      <x:c r="P8" s="20" t="str">
+        <x:v>https://www.bankofcanada.ca/wp-content/uploads/2019/07/swp2019-24.pdf</x:v>
+      </x:c>
+      <x:c r="Q8" s="20" t="str">
+        <x:v>v3 五刊定向复核补入边界相关。JPE 出版页面确认 2021 年 129(7):2157-2180，首次在线 2021-05-26。已核对加拿大央行公开作者稿的相关讨论：结论将 Bitcoin 视为数字现金替代方案，并指出 PoW 成本及扩容局限；模型主体为一般支付隐私，不直接刻画区块链，故不计入主目录。公开作者稿与正式期刊版的核验范围分别说明。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="64" customHeight="1">
+      <x:c r="A9" s="12" t="str">
+        <x:v>R10</x:v>
+      </x:c>
+      <x:c r="B9" s="18" t="str">
+        <x:v>交易费用、支付与区块链扩容</x:v>
+      </x:c>
+      <x:c r="C9" s="15" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="D9" s="24" t="d">
+        <x:v>2025-07-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E9" s="14" t="str">
+        <x:v>JFE</x:v>
+      </x:c>
+      <x:c r="F9" s="20" t="str">
+        <x:v>Payments and privacy in the digital economy</x:v>
+      </x:c>
+      <x:c r="G9" s="20" t="str">
+        <x:v>Toni Ahnert; Peter Hoffmann; Cyril Monnet</x:v>
+      </x:c>
+      <x:c r="H9" s="21" t="str">
+        <x:v>卷期发表</x:v>
+      </x:c>
+      <x:c r="I9" s="20" t="str">
+        <x:v>一般支付隐私与信贷理论；讨论区块链实现隐私保护型数字支付的可能性</x:v>
+      </x:c>
+      <x:c r="J9" s="20" t="str">
         <x:v>相关理论</x:v>
       </x:c>
-      <x:c r="K9" s="30" t="str">
-        <x:v>33(3): 1072-1092</x:v>
-      </x:c>
-      <x:c r="L9" s="32"/>
-      <x:c r="M9" s="30" t="str">
-        <x:v>10.1287/isre.2022.1100</x:v>
-      </x:c>
-      <x:c r="N9" s="30" t="str">
-        <x:v>https://doi.org/10.1287/isre.2022.1100</x:v>
-      </x:c>
-      <x:c r="O9" s="33" t="str">
-        <x:v>打开来源</x:v>
-      </x:c>
-      <x:c r="P9" s="30" t="str"/>
-      <x:c r="Q9" s="30" t="str"/>
-    </x:row>
-    <x:row r="10" ht="46" customHeight="1">
+      <x:c r="K9" s="20" t="str">
+        <x:v>169: 104050</x:v>
+      </x:c>
+      <x:c r="L9" s="22"/>
+      <x:c r="M9" s="20" t="str">
+        <x:v>10.1016/j.jfineco.2025.104050</x:v>
+      </x:c>
+      <x:c r="N9" s="20" t="str">
+        <x:v>https://doi.org/10.1016/j.jfineco.2025.104050</x:v>
+      </x:c>
+      <x:c r="O9" s="23" t="str">
+        <x:v>打开来源</x:v>
+      </x:c>
+      <x:c r="P9" s="20" t="str">
+        <x:v>https://www.ecb.europa.eu/pub/pdf/scpwps/ecb.wp2662~fa8429a967.en.pdf</x:v>
+      </x:c>
+      <x:c r="Q9" s="20" t="str">
+        <x:v>v3 五刊定向复核补入边界相关。JFE 出版记录确认 169 (2025-07):104050。出版方可检索正文提到区块链与密码学可实现保护隐私的去中心化结算；主体为一般贷款、支付选择和数据隐私模型，不直接建模加密资产，故不计入主目录。补充链接为 ECB 公开工作论文版本，不将其日期冒充正式发表日期。首次在线日期未单独核实，留空。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="64" customHeight="1">
       <x:c r="A10" s="25" t="str">
-        <x:v>R05</x:v>
+        <x:v>R11</x:v>
       </x:c>
       <x:c r="B10" s="34" t="str">
-        <x:v>综述与研究议程</x:v>
+        <x:v>智能合约、DAO、社区与制度治理</x:v>
       </x:c>
       <x:c r="C10" s="27" t="n">
-        <x:v>2021</x:v>
+        <x:v>2019</x:v>
       </x:c>
       <x:c r="D10" s="28" t="d">
-        <x:v>2021-03-01T00:00:00.000Z</x:v>
+        <x:v>2019-11-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E10" s="29" t="str">
-        <x:v>ISR</x:v>
+        <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F10" s="30" t="str">
-        <x:v>FinTech as a Game Changer: Overview of Research Frontiers</x:v>
+        <x:v>A Flexible Design for Funding Public Goods</x:v>
       </x:c>
       <x:c r="G10" s="30" t="str">
-        <x:v>Terrence Hendershott; Xiaoquan (Michael) Zhang; J. Leon Zhao; Zhiqiang (Eric) Zheng</x:v>
+        <x:v>Vitalik Buterin; Zoë Hitzig; E. Glen Weyl</x:v>
       </x:c>
       <x:c r="H10" s="31" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I10" s="30" t="str">
-        <x:v>FinTech 研究前沿导论，涵盖区块链与加密货币</x:v>
+        <x:v>二次融资与公共品供给；区块链社区是适用场景之一，模型为一般机制设计</x:v>
       </x:c>
       <x:c r="J10" s="30" t="str">
-        <x:v>相关综述</x:v>
+        <x:v>相关理论</x:v>
       </x:c>
       <x:c r="K10" s="30" t="str">
-        <x:v>32(1): 1-17</x:v>
-      </x:c>
-      <x:c r="L10" s="32"/>
+        <x:v>65(11): 5171-5187</x:v>
+      </x:c>
+      <x:c r="L10" s="32" t="d">
+        <x:v>2019-07-02T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="M10" s="30" t="str">
-        <x:v>10.1287/isre.2021.0997</x:v>
+        <x:v>10.1287/mnsc.2019.3337</x:v>
       </x:c>
       <x:c r="N10" s="30" t="str">
-        <x:v>https://doi.org/10.1287/isre.2021.0997</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2019.3337</x:v>
       </x:c>
       <x:c r="O10" s="33" t="str">
         <x:v>打开来源</x:v>
       </x:c>
-      <x:c r="P10" s="30" t="str"/>
-      <x:c r="Q10" s="30" t="str"/>
+      <x:c r="P10" s="30" t="str">
+        <x:v>https://arxiv.org/html/1809.06421</x:v>
+      </x:c>
+      <x:c r="Q10" s="30" t="str">
+        <x:v>v4 根据用户表格第 99 行补入边界相关。出版方确认 2019 年 65(11):5171-5187，首次在线 2019-07-02，接收 2019-02-26。公开作者稿第 5.2 节讨论区块链社区中的合谋问题，但主体为一般公共品二次融资机制，故单列相关理论；未仅因首作者与 Ethereum 的关系而计为加密资产原创研究。</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="46" customHeight="1">
       <x:c r="A11" s="12" t="str">
-        <x:v>R06</x:v>
+        <x:v>R02</x:v>
       </x:c>
       <x:c r="B11" s="18" t="str">
-        <x:v>综述与研究议程</x:v>
+        <x:v>智能合约、DAO、社区与制度治理</x:v>
       </x:c>
       <x:c r="C11" s="15" t="n">
-        <x:v>2025</x:v>
+        <x:v>2022</x:v>
       </x:c>
       <x:c r="D11" s="24" t="d">
-        <x:v>2025-11-01T00:00:00.000Z</x:v>
+        <x:v>2022-08-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E11" s="14" t="str">
-        <x:v>TAR</x:v>
+        <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F11" s="20" t="str">
-        <x:v>Innovative Capital Markets Research and Accounting Practitioners</x:v>
+        <x:v>Optimal Management of Evolving Hierarchies</x:v>
       </x:c>
       <x:c r="G11" s="20" t="str">
-        <x:v>Carolyn M. Callahan</x:v>
+        <x:v>Jens Leth Hougaard; Juan D. Moreno-Ternero; Lars Peter Østerdal</x:v>
       </x:c>
       <x:c r="H11" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I11" s="20" t="str">
-        <x:v>面向实务的会计研究议程，其中包括加密和数字资产</x:v>
+        <x:v>一般层级组织的激励分配；区块链是潜在应用</x:v>
       </x:c>
       <x:c r="J11" s="20" t="str">
-        <x:v>相关综述</x:v>
+        <x:v>相关理论</x:v>
       </x:c>
       <x:c r="K11" s="20" t="str">
-        <x:v>100(6): 419-430</x:v>
-      </x:c>
-      <x:c r="L11" s="22" t="d">
-        <x:v>2025-10-17T00:00:00.000Z</x:v>
-      </x:c>
+        <x:v>68(8): 6024-6038</x:v>
+      </x:c>
+      <x:c r="L11" s="22"/>
       <x:c r="M11" s="20" t="str">
-        <x:v>10.2308/tar-2025-0273</x:v>
+        <x:v>10.1287/mnsc.2021.4185</x:v>
       </x:c>
       <x:c r="N11" s="20" t="str">
-        <x:v>https://doi.org/10.2308/tar-2025-0273</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2021.4185</x:v>
       </x:c>
       <x:c r="O11" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -10169,44 +10410,44 @@
     </x:row>
     <x:row r="12" ht="46" customHeight="1">
       <x:c r="A12" s="12" t="str">
-        <x:v>R07</x:v>
+        <x:v>R03</x:v>
       </x:c>
       <x:c r="B12" s="18" t="str">
-        <x:v>综述与研究议程</x:v>
+        <x:v>智能合约、DAO、社区与制度治理</x:v>
       </x:c>
       <x:c r="C12" s="15" t="n">
-        <x:v>2025</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="D12" s="24" t="d">
-        <x:v>2025-11-01T00:00:00.000Z</x:v>
+        <x:v>2023-05-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E12" s="14" t="str">
-        <x:v>JME</x:v>
+        <x:v>AER</x:v>
       </x:c>
       <x:c r="F12" s="20" t="str">
-        <x:v>“Information frictions in macroeconomics: The legacy of Robert E. Lucas, Jr.”</x:v>
+        <x:v>Smart Contracts and the Coase Conjecture</x:v>
       </x:c>
       <x:c r="G12" s="20" t="str">
-        <x:v>Robert M. Townsend</x:v>
+        <x:v>Thomas Brzustowski; Alkis Georgiadis-Harris; Balázs Szentes</x:v>
       </x:c>
       <x:c r="H12" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I12" s="20" t="str">
-        <x:v>宏观信息摩擦综述，专门讨论分布式账本与可编程数字资产</x:v>
+        <x:v>动态智能合约与耐用品垄断；一般契约理论，不直接建模区块链</x:v>
       </x:c>
       <x:c r="J12" s="20" t="str">
-        <x:v>相关综述</x:v>
+        <x:v>相关理论</x:v>
       </x:c>
       <x:c r="K12" s="20" t="str">
-        <x:v>155: 103842</x:v>
+        <x:v>113(5): 1334-1359</x:v>
       </x:c>
       <x:c r="L12" s="22"/>
       <x:c r="M12" s="20" t="str">
-        <x:v>10.1016/j.jmoneco.2025.103842</x:v>
+        <x:v>10.1257/aer.20220357</x:v>
       </x:c>
       <x:c r="N12" s="20" t="str">
-        <x:v>https://doi.org/10.1016/j.jmoneco.2025.103842</x:v>
+        <x:v>https://doi.org/10.1257/aer.20220357</x:v>
       </x:c>
       <x:c r="O12" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -10214,9 +10455,199 @@
       <x:c r="P12" s="20" t="str"/>
       <x:c r="Q12" s="20" t="str"/>
     </x:row>
+    <x:row r="13" ht="46" customHeight="1">
+      <x:c r="A13" s="25" t="str">
+        <x:v>R04</x:v>
+      </x:c>
+      <x:c r="B13" s="34" t="str">
+        <x:v>供应链、企业应用与金融包容</x:v>
+      </x:c>
+      <x:c r="C13" s="27" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="D13" s="28" t="d">
+        <x:v>2022-09-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E13" s="29" t="str">
+        <x:v>ISR</x:v>
+      </x:c>
+      <x:c r="F13" s="30" t="str">
+        <x:v>The Dark Side of Technological Modularity: Opportunistic Information Hiding During Interorganizational System Adoption</x:v>
+      </x:c>
+      <x:c r="G13" s="30" t="str">
+        <x:v>Sanjith Gopalakrishnan; Moksh Matta; Hasan Cavusoglu</x:v>
+      </x:c>
+      <x:c r="H13" s="31" t="str">
+        <x:v>卷期发表</x:v>
+      </x:c>
+      <x:c r="I13" s="30" t="str">
+        <x:v>模块化与组织间系统采用；区块链是应用场景之一</x:v>
+      </x:c>
+      <x:c r="J13" s="30" t="str">
+        <x:v>相关理论</x:v>
+      </x:c>
+      <x:c r="K13" s="30" t="str">
+        <x:v>33(3): 1072-1092</x:v>
+      </x:c>
+      <x:c r="L13" s="32"/>
+      <x:c r="M13" s="30" t="str">
+        <x:v>10.1287/isre.2022.1100</x:v>
+      </x:c>
+      <x:c r="N13" s="30" t="str">
+        <x:v>https://doi.org/10.1287/isre.2022.1100</x:v>
+      </x:c>
+      <x:c r="O13" s="33" t="str">
+        <x:v>打开来源</x:v>
+      </x:c>
+      <x:c r="P13" s="30" t="str"/>
+      <x:c r="Q13" s="30" t="str"/>
+    </x:row>
+    <x:row r="14" ht="46" customHeight="1">
+      <x:c r="A14" s="25" t="str">
+        <x:v>R05</x:v>
+      </x:c>
+      <x:c r="B14" s="34" t="str">
+        <x:v>综述与研究议程</x:v>
+      </x:c>
+      <x:c r="C14" s="27" t="n">
+        <x:v>2021</x:v>
+      </x:c>
+      <x:c r="D14" s="28" t="d">
+        <x:v>2021-03-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E14" s="29" t="str">
+        <x:v>ISR</x:v>
+      </x:c>
+      <x:c r="F14" s="30" t="str">
+        <x:v>FinTech as a Game Changer: Overview of Research Frontiers</x:v>
+      </x:c>
+      <x:c r="G14" s="30" t="str">
+        <x:v>Terrence Hendershott; Xiaoquan (Michael) Zhang; J. Leon Zhao; Zhiqiang (Eric) Zheng</x:v>
+      </x:c>
+      <x:c r="H14" s="31" t="str">
+        <x:v>卷期发表</x:v>
+      </x:c>
+      <x:c r="I14" s="30" t="str">
+        <x:v>FinTech 研究前沿导论，涵盖区块链与加密货币</x:v>
+      </x:c>
+      <x:c r="J14" s="30" t="str">
+        <x:v>相关综述</x:v>
+      </x:c>
+      <x:c r="K14" s="30" t="str">
+        <x:v>32(1): 1-17</x:v>
+      </x:c>
+      <x:c r="L14" s="32"/>
+      <x:c r="M14" s="30" t="str">
+        <x:v>10.1287/isre.2021.0997</x:v>
+      </x:c>
+      <x:c r="N14" s="30" t="str">
+        <x:v>https://doi.org/10.1287/isre.2021.0997</x:v>
+      </x:c>
+      <x:c r="O14" s="33" t="str">
+        <x:v>打开来源</x:v>
+      </x:c>
+      <x:c r="P14" s="30" t="str"/>
+      <x:c r="Q14" s="30" t="str"/>
+    </x:row>
+    <x:row r="15" ht="46" customHeight="1">
+      <x:c r="A15" s="12" t="str">
+        <x:v>R06</x:v>
+      </x:c>
+      <x:c r="B15" s="18" t="str">
+        <x:v>综述与研究议程</x:v>
+      </x:c>
+      <x:c r="C15" s="15" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="D15" s="24" t="d">
+        <x:v>2025-11-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E15" s="14" t="str">
+        <x:v>TAR</x:v>
+      </x:c>
+      <x:c r="F15" s="20" t="str">
+        <x:v>Innovative Capital Markets Research and Accounting Practitioners</x:v>
+      </x:c>
+      <x:c r="G15" s="20" t="str">
+        <x:v>Carolyn M. Callahan</x:v>
+      </x:c>
+      <x:c r="H15" s="21" t="str">
+        <x:v>卷期发表</x:v>
+      </x:c>
+      <x:c r="I15" s="20" t="str">
+        <x:v>面向实务的会计研究议程，其中包括加密和数字资产</x:v>
+      </x:c>
+      <x:c r="J15" s="20" t="str">
+        <x:v>相关综述</x:v>
+      </x:c>
+      <x:c r="K15" s="20" t="str">
+        <x:v>100(6): 419-430</x:v>
+      </x:c>
+      <x:c r="L15" s="22" t="d">
+        <x:v>2025-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="M15" s="20" t="str">
+        <x:v>10.2308/tar-2025-0273</x:v>
+      </x:c>
+      <x:c r="N15" s="20" t="str">
+        <x:v>https://doi.org/10.2308/tar-2025-0273</x:v>
+      </x:c>
+      <x:c r="O15" s="23" t="str">
+        <x:v>打开来源</x:v>
+      </x:c>
+      <x:c r="P15" s="20" t="str"/>
+      <x:c r="Q15" s="20" t="str"/>
+    </x:row>
+    <x:row r="16" ht="46" customHeight="1">
+      <x:c r="A16" s="12" t="str">
+        <x:v>R07</x:v>
+      </x:c>
+      <x:c r="B16" s="18" t="str">
+        <x:v>综述与研究议程</x:v>
+      </x:c>
+      <x:c r="C16" s="15" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="D16" s="24" t="d">
+        <x:v>2025-11-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E16" s="14" t="str">
+        <x:v>JME</x:v>
+      </x:c>
+      <x:c r="F16" s="20" t="str">
+        <x:v>“Information frictions in macroeconomics: The legacy of Robert E. Lucas, Jr.”</x:v>
+      </x:c>
+      <x:c r="G16" s="20" t="str">
+        <x:v>Robert M. Townsend</x:v>
+      </x:c>
+      <x:c r="H16" s="21" t="str">
+        <x:v>卷期发表</x:v>
+      </x:c>
+      <x:c r="I16" s="20" t="str">
+        <x:v>宏观信息摩擦综述，专门讨论分布式账本与可编程数字资产</x:v>
+      </x:c>
+      <x:c r="J16" s="20" t="str">
+        <x:v>相关综述</x:v>
+      </x:c>
+      <x:c r="K16" s="20" t="str">
+        <x:v>155: 103842</x:v>
+      </x:c>
+      <x:c r="L16" s="22"/>
+      <x:c r="M16" s="20" t="str">
+        <x:v>10.1016/j.jmoneco.2025.103842</x:v>
+      </x:c>
+      <x:c r="N16" s="20" t="str">
+        <x:v>https://doi.org/10.1016/j.jmoneco.2025.103842</x:v>
+      </x:c>
+      <x:c r="O16" s="23" t="str">
+        <x:v>打开来源</x:v>
+      </x:c>
+      <x:c r="P16" s="20" t="str"/>
+      <x:c r="Q16" s="20" t="str"/>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="H6:H12">
-    <x:cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="已接收"/>
+  <x:conditionalFormatting sqref="H6:H16">
+    <x:cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="已接收"/>
   </x:conditionalFormatting>
   <x:hyperlinks>
     <x:hyperlink ref="O6" r:id="Hyperlink6" display="打开来源"/>
@@ -10226,10 +10657,14 @@
     <x:hyperlink ref="O10" r:id="Hyperlink10" display="打开来源"/>
     <x:hyperlink ref="O11" r:id="Hyperlink11" display="打开来源"/>
     <x:hyperlink ref="O12" r:id="Hyperlink12" display="打开来源"/>
+    <x:hyperlink ref="O13" r:id="Hyperlink13" display="打开来源"/>
+    <x:hyperlink ref="O14" r:id="Hyperlink14" display="打开来源"/>
+    <x:hyperlink ref="O15" r:id="Hyperlink15" display="打开来源"/>
+    <x:hyperlink ref="O16" r:id="Hyperlink16" display="打开来源"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart r:id="Ra7f63ced920f4d35"/>
+    <x:tablePart r:id="R625a90e6e01e4a1d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Remove accounting journals from catalogue: 16 journals, 159 main and 10 related works
</commit_message>
<xml_diff>
--- a/downloads/catalogue.xlsx
+++ b/downloads/catalogue.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="目录总览" sheetId="1" r:id="R211faeb502164b50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="论文目录" sheetId="2" r:id="R8dbbff83562b4659"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="边界相关" sheetId="3" r:id="Re6d7832b0cbb4e02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="目录总览" sheetId="1" r:id="Rd0bf3b5679d04ec5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="论文目录" sheetId="2" r:id="R0cdf193586204968"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="边界相关" sheetId="3" r:id="Rc277b6002fea486d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -73,7 +73,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="10">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -113,6 +113,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF243D59"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEDF2F7"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -171,7 +176,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="79">
+  <x:cellXfs count="82">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -405,11 +410,36 @@
     <x:xf numFmtId="200" fontId="4" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="5" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="6">
+  <x:dxfs count="8">
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF795400"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF795400"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
@@ -481,8 +511,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MainBibliography" displayName="MainBibliography" ref="A5:Q173" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:Q173"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="MainBibliography" displayName="MainBibliography" ref="A5:Q164" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:Q164"/>
   <x:tableColumns count="17">
     <x:tableColumn id="1" name="编号"/>
     <x:tableColumn id="2" name="研究主题"/>
@@ -507,8 +537,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="AdjacentBibliography" displayName="AdjacentBibliography" ref="A5:Q16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:Q16"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="AdjacentBibliography" displayName="AdjacentBibliography" ref="A5:Q15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:Q15"/>
   <x:tableColumns count="17">
     <x:tableColumn id="1" name="编号"/>
     <x:tableColumn id="2" name="研究主题"/>
@@ -774,7 +804,7 @@
       <x:c r="E3" s="2"/>
       <x:c r="F3" s="2"/>
       <x:c r="G3" s="4" t="str">
-        <x:v>19 本指定期刊主刊；每篇仅归入一个主主题</x:v>
+        <x:v>16 本指定期刊主刊；每篇仅归入一个主主题</x:v>
       </x:c>
       <x:c r="H3" s="2"/>
     </x:row>
@@ -820,11 +850,11 @@
         <x:v>American Economic Review</x:v>
       </x:c>
       <x:c r="C6" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A6)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$164,A6)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D6" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A6)</x:f>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$15,A6)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="E6" s="14" t="str">
@@ -835,7 +865,7 @@
         <x:v>货币竞争、加密资产估值与收益</x:v>
       </x:c>
       <x:c r="H6" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$B$6:$B$173,G6)</x:f>
+        <x:f>COUNTIFS('论文目录'!$B$6:$B$164,G6)</x:f>
         <x:v>14</x:v>
       </x:c>
     </x:row>
@@ -847,11 +877,11 @@
         <x:v>Econometrica</x:v>
       </x:c>
       <x:c r="C7" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A7)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$164,A7)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D7" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A7)</x:f>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$15,A7)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E7" s="14" t="str">
@@ -862,7 +892,7 @@
         <x:v>ICO、代币融资与平台经济</x:v>
       </x:c>
       <x:c r="H7" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$B$6:$B$173,G7)</x:f>
+        <x:f>COUNTIFS('论文目录'!$B$6:$B$164,G7)</x:f>
         <x:v>23</x:v>
       </x:c>
     </x:row>
@@ -874,11 +904,11 @@
         <x:v>The Quarterly Journal of Economics</x:v>
       </x:c>
       <x:c r="C8" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A8)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$164,A8)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D8" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A8)</x:f>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$15,A8)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E8" s="14" t="str">
@@ -889,7 +919,7 @@
         <x:v>共识机制、挖矿与去中心化安全</x:v>
       </x:c>
       <x:c r="H8" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$B$6:$B$173,G8)</x:f>
+        <x:f>COUNTIFS('论文目录'!$B$6:$B$164,G8)</x:f>
         <x:v>19</x:v>
       </x:c>
     </x:row>
@@ -901,11 +931,11 @@
         <x:v>Journal of Political Economy</x:v>
       </x:c>
       <x:c r="C9" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A9)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$164,A9)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D9" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A9)</x:f>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$15,A9)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="E9" s="14" t="str">
@@ -916,7 +946,7 @@
         <x:v>交易费用、支付与区块链扩容</x:v>
       </x:c>
       <x:c r="H9" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$B$6:$B$173,G9)</x:f>
+        <x:f>COUNTIFS('论文目录'!$B$6:$B$164,G9)</x:f>
         <x:v>11</x:v>
       </x:c>
     </x:row>
@@ -928,11 +958,11 @@
         <x:v>The Review of Economic Studies</x:v>
       </x:c>
       <x:c r="C10" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A10)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$164,A10)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D10" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A10)</x:f>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$15,A10)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E10" s="14" t="str">
@@ -943,7 +973,7 @@
         <x:v>交易市场、衍生品与投资者行为</x:v>
       </x:c>
       <x:c r="H10" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$B$6:$B$173,G10)</x:f>
+        <x:f>COUNTIFS('论文目录'!$B$6:$B$164,G10)</x:f>
         <x:v>19</x:v>
       </x:c>
     </x:row>
@@ -955,11 +985,11 @@
         <x:v>Journal of Monetary Economics</x:v>
       </x:c>
       <x:c r="C11" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A11)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$164,A11)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="D11" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A11)</x:f>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$15,A11)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="E11" s="14" t="str">
@@ -970,7 +1000,7 @@
         <x:v>去中心化交易所、自动做市与流动性</x:v>
       </x:c>
       <x:c r="H11" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$B$6:$B$173,G11)</x:f>
+        <x:f>COUNTIFS('论文目录'!$B$6:$B$164,G11)</x:f>
         <x:v>13</x:v>
       </x:c>
     </x:row>
@@ -982,11 +1012,11 @@
         <x:v>The Review of Financial Studies</x:v>
       </x:c>
       <x:c r="C12" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A12)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$164,A12)</x:f>
         <x:v>19</x:v>
       </x:c>
       <x:c r="D12" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A12)</x:f>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$15,A12)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E12" s="14" t="str">
@@ -997,7 +1027,7 @@
         <x:v>稳定币、DeFi 借贷与预测市场</x:v>
       </x:c>
       <x:c r="H12" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$B$6:$B$173,G12)</x:f>
+        <x:f>COUNTIFS('论文目录'!$B$6:$B$164,G12)</x:f>
         <x:v>8</x:v>
       </x:c>
     </x:row>
@@ -1009,11 +1039,11 @@
         <x:v>Journal of Financial Economics</x:v>
       </x:c>
       <x:c r="C13" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A13)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$164,A13)</x:f>
         <x:v>13</x:v>
       </x:c>
       <x:c r="D13" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A13)</x:f>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$15,A13)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="E13" s="14" t="str">
@@ -1024,7 +1054,7 @@
         <x:v>智能合约、DAO、社区与制度治理</x:v>
       </x:c>
       <x:c r="H13" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$B$6:$B$173,G13)</x:f>
+        <x:f>COUNTIFS('论文目录'!$B$6:$B$164,G13)</x:f>
         <x:v>20</x:v>
       </x:c>
     </x:row>
@@ -1036,11 +1066,11 @@
         <x:v>The Journal of Finance</x:v>
       </x:c>
       <x:c r="C14" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A14)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$164,A14)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="D14" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A14)</x:f>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$15,A14)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E14" s="14" t="str">
@@ -1051,8 +1081,8 @@
         <x:v>企业披露、财务会计与审计</x:v>
       </x:c>
       <x:c r="H14" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$B$6:$B$173,G14)</x:f>
-        <x:v>11</x:v>
+        <x:f>COUNTIFS('论文目录'!$B$6:$B$164,G14)</x:f>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="26" customHeight="1">
@@ -1063,11 +1093,11 @@
         <x:v>Mathematical Finance</x:v>
       </x:c>
       <x:c r="C15" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A15)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$164,A15)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="D15" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A15)</x:f>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$15,A15)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E15" s="14" t="str">
@@ -1078,8 +1108,8 @@
         <x:v>市场操纵、非法活动、网络犯罪与税收</x:v>
       </x:c>
       <x:c r="H15" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$B$6:$B$173,G15)</x:f>
-        <x:v>11</x:v>
+        <x:f>COUNTIFS('论文目录'!$B$6:$B$164,G15)</x:f>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="26" customHeight="1">
@@ -1090,11 +1120,11 @@
         <x:v>Finance and Stochastics</x:v>
       </x:c>
       <x:c r="C16" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A16)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$164,A16)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D16" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A16)</x:f>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$15,A16)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E16" s="14" t="str">
@@ -1105,7 +1135,7 @@
         <x:v>供应链、企业应用与金融包容</x:v>
       </x:c>
       <x:c r="H16" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$B$6:$B$173,G16)</x:f>
+        <x:f>COUNTIFS('论文目录'!$B$6:$B$164,G16)</x:f>
         <x:v>11</x:v>
       </x:c>
     </x:row>
@@ -1117,11 +1147,11 @@
         <x:v>SIAM Journal on Financial Mathematics</x:v>
       </x:c>
       <x:c r="C17" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A17)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$164,A17)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="D17" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A17)</x:f>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$15,A17)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E17" s="14" t="str">
@@ -1132,7 +1162,7 @@
         <x:v>NFT、艺术品与创作者经济</x:v>
       </x:c>
       <x:c r="H17" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$B$6:$B$173,G17)</x:f>
+        <x:f>COUNTIFS('论文目录'!$B$6:$B$164,G17)</x:f>
         <x:v>7</x:v>
       </x:c>
     </x:row>
@@ -1144,11 +1174,11 @@
         <x:v>Management Science</x:v>
       </x:c>
       <x:c r="C18" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A18)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$164,A18)</x:f>
         <x:v>68</x:v>
       </x:c>
       <x:c r="D18" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A18)</x:f>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$15,A18)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="E18" s="14" t="str">
@@ -1159,7 +1189,7 @@
         <x:v>综述与研究议程</x:v>
       </x:c>
       <x:c r="H18" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$B$6:$B$173,G18)</x:f>
+        <x:f>COUNTIFS('论文目录'!$B$6:$B$164,G18)</x:f>
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -1171,11 +1201,11 @@
         <x:v>Operations Research</x:v>
       </x:c>
       <x:c r="C19" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A19)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$164,A19)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="D19" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A19)</x:f>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$15,A19)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E19" s="14" t="str">
@@ -1187,7 +1217,7 @@
       </x:c>
       <x:c r="H19" s="76" t="n">
         <x:f>SUM(H6:H18)</x:f>
-        <x:v>168</x:v>
+        <x:v>159</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="26" customHeight="1">
@@ -1198,11 +1228,11 @@
         <x:v>Information Systems Research</x:v>
       </x:c>
       <x:c r="C20" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A20)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$164,A20)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="D20" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A20)</x:f>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$15,A20)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="E20" s="14" t="str">
@@ -1220,11 +1250,11 @@
         <x:v>MIS Quarterly</x:v>
       </x:c>
       <x:c r="C21" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A21)</x:f>
+        <x:f>COUNTIFS('论文目录'!$E$6:$E$164,A21)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="D21" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A21)</x:f>
+        <x:f>COUNTIFS('边界相关'!$E$6:$E$15,A21)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E21" s="14" t="str">
@@ -1239,107 +1269,71 @@
       </x:c>
     </x:row>
     <x:row r="22" ht="26" customHeight="1">
-      <x:c r="A22" s="2" t="str">
-        <x:v>JAE</x:v>
-      </x:c>
-      <x:c r="B22" s="2" t="str">
-        <x:v>Journal of Accounting and Economics</x:v>
-      </x:c>
-      <x:c r="C22" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A22)</x:f>
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D22" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A22)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E22" s="14" t="str">
-        <x:v>会计学</x:v>
-      </x:c>
+      <x:c r="A22" s="80" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B22" s="80"/>
+      <x:c r="C22" s="81" t="n">
+        <x:f>SUM(C6:C21)</x:f>
+        <x:v>159</x:v>
+      </x:c>
+      <x:c r="D22" s="81" t="n">
+        <x:f>SUM(D6:D21)</x:f>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E22" s="80"/>
       <x:c r="F22" s="2"/>
       <x:c r="G22" s="2" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="H22" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$H$6:$H$173,G22)</x:f>
-        <x:v>144</x:v>
+        <x:f>COUNTIFS('论文目录'!$H$6:$H$164,G22)</x:f>
+        <x:v>137</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="26" customHeight="1">
-      <x:c r="A23" s="2" t="str">
-        <x:v>JAR</x:v>
-      </x:c>
-      <x:c r="B23" s="2" t="str">
-        <x:v>Journal of Accounting Research</x:v>
-      </x:c>
-      <x:c r="C23" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A23)</x:f>
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D23" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A23)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E23" s="14" t="str">
-        <x:v>会计学</x:v>
-      </x:c>
+      <x:c r="A23"/>
+      <x:c r="B23"/>
+      <x:c r="C23"/>
+      <x:c r="D23"/>
+      <x:c r="E23"/>
       <x:c r="F23" s="2"/>
       <x:c r="G23" s="2" t="str">
         <x:v>在线发表</x:v>
       </x:c>
       <x:c r="H23" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$H$6:$H$173,G23)</x:f>
-        <x:v>22</x:v>
+        <x:f>COUNTIFS('论文目录'!$H$6:$H$164,G23)</x:f>
+        <x:v>20</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="26" customHeight="1">
-      <x:c r="A24" s="2" t="str">
-        <x:v>TAR</x:v>
-      </x:c>
-      <x:c r="B24" s="2" t="str">
-        <x:v>The Accounting Review</x:v>
-      </x:c>
-      <x:c r="C24" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$E$6:$E$173,A24)</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D24" s="38" t="n">
-        <x:f>COUNTIFS('边界相关'!$E$6:$E$16,A24)</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E24" s="14" t="str">
-        <x:v>会计学</x:v>
-      </x:c>
+      <x:c r="A24"/>
+      <x:c r="B24"/>
+      <x:c r="C24"/>
+      <x:c r="D24"/>
+      <x:c r="E24"/>
       <x:c r="F24" s="2"/>
       <x:c r="G24" s="2" t="str">
         <x:v>已接收</x:v>
       </x:c>
       <x:c r="H24" s="38" t="n">
-        <x:f>COUNTIFS('论文目录'!$H$6:$H$173,G24)</x:f>
+        <x:f>COUNTIFS('论文目录'!$H$6:$H$164,G24)</x:f>
         <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="26" customHeight="1">
-      <x:c r="A25" s="75" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B25" s="75"/>
-      <x:c r="C25" s="76" t="n">
-        <x:f>SUM(C6:C24)</x:f>
-        <x:v>168</x:v>
-      </x:c>
-      <x:c r="D25" s="76" t="n">
-        <x:f>SUM(D6:D24)</x:f>
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="E25" s="75"/>
+      <x:c r="A25"/>
+      <x:c r="B25"/>
+      <x:c r="C25"/>
+      <x:c r="D25"/>
+      <x:c r="E25"/>
       <x:c r="F25" s="2"/>
       <x:c r="G25" s="75" t="str">
         <x:v>状态合计</x:v>
       </x:c>
       <x:c r="H25" s="76" t="n">
         <x:f>SUM(H22:H24)</x:f>
-        <x:v>168</x:v>
+        <x:v>159</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="20" customHeight="1">
@@ -1389,7 +1383,7 @@
         <x:v>范围</x:v>
       </x:c>
       <x:c r="B30" s="20" t="str">
-        <x:v>限定 19 刊主刊。主目录含直接主题、加密数据场景、评论和专辑导论。</x:v>
+        <x:v>限定 16 刊主刊。已移除三本会计学期刊，保留其余题录原编号。</x:v>
       </x:c>
       <x:c r="C30" s="2"/>
       <x:c r="D30" s="2"/>
@@ -1487,7 +1481,7 @@
         <x:v>题录覆盖</x:v>
       </x:c>
       <x:c r="B37" s="20" t="str">
-        <x:v>v4 逐行对照用户表格 167 条。补入主目录 P167–P168、边界相关 R11。旧记录及编号保留。</x:v>
+        <x:v>2026-10-31 调整网站范围：移除 9 条主目录、1 条边界相关。原始核验截止日仍为 2026-10-27。</x:v>
       </x:c>
       <x:c r="C37" s="2"/>
       <x:c r="D37" s="2"/>
@@ -1501,7 +1495,7 @@
         <x:v>类型与数量</x:v>
       </x:c>
       <x:c r="B38" s="20" t="str">
-        <x:v>主目录含 3 篇评论、1 篇专辑导论、1 篇社论和 4 篇加密数据场景研究。另列 11 篇边界相关文献。</x:v>
+        <x:v>主目录含 1 篇评论、1 篇专辑导论、1 篇社论和 3 篇加密数据场景研究。另列 10 条边界相关。</x:v>
       </x:c>
       <x:c r="C38" s="2"/>
       <x:c r="D38" s="2"/>
@@ -1526,7 +1520,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr>
     <x:tabColor rgb="FF243D59"/>
   </x:sheetPr>
@@ -7854,46 +7848,44 @@
     </x:row>
     <x:row r="134" ht="46" customHeight="1">
       <x:c r="A134" s="12" t="str">
-        <x:v>P122</x:v>
+        <x:v>P123</x:v>
       </x:c>
       <x:c r="B134" s="18" t="str">
         <x:v>企业披露、财务会计与审计</x:v>
       </x:c>
       <x:c r="C134" s="15" t="n">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="D134" s="24" t="d">
-        <x:v>2022-03-01T00:00:00.000Z</x:v>
+        <x:v>2023-11-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E134" s="14" t="str">
-        <x:v>JAR</x:v>
+        <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F134" s="20" t="str">
-        <x:v>The Role of Disclosure and Information Intermediaries in an Unregulated Capital Market: Evidence from Initial Coin Offerings</x:v>
+        <x:v>Conflicted Analysts and Initial Coin Offerings</x:v>
       </x:c>
       <x:c r="G134" s="20" t="str">
-        <x:v>Thomas Bourveau; Emmanuel T. De George; Atif Ellahie; Daniele Macciocchi</x:v>
+        <x:v>Andreas Barth; Valerie Laturnus; Sasan Mansouri; Alexander F. Wagner</x:v>
       </x:c>
       <x:c r="H134" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I134" s="20" t="str">
-        <x:v>ICO 自愿披露与信息中介</x:v>
+        <x:v>ICO 分析师利益冲突与评级</x:v>
       </x:c>
       <x:c r="J134" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K134" s="20" t="str">
-        <x:v>60(1): 129-167</x:v>
-      </x:c>
-      <x:c r="L134" s="35" t="d">
-        <x:v>2021-11-01T00:00:00.000Z</x:v>
-      </x:c>
+        <x:v>69(11): 6641-6666</x:v>
+      </x:c>
+      <x:c r="L134" s="22"/>
       <x:c r="M134" s="20" t="str">
-        <x:v>10.1111/1475-679x.12404</x:v>
+        <x:v>10.1287/mnsc.2021.02928</x:v>
       </x:c>
       <x:c r="N134" s="20" t="str">
-        <x:v>https://doi.org/10.1111/1475-679x.12404</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2021.02928</x:v>
       </x:c>
       <x:c r="O134" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -7903,44 +7895,44 @@
     </x:row>
     <x:row r="135" ht="46" customHeight="1">
       <x:c r="A135" s="12" t="str">
-        <x:v>P123</x:v>
+        <x:v>P124</x:v>
       </x:c>
       <x:c r="B135" s="18" t="str">
         <x:v>企业披露、财务会计与审计</x:v>
       </x:c>
       <x:c r="C135" s="15" t="n">
-        <x:v>2023</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="D135" s="24" t="d">
-        <x:v>2023-11-01T00:00:00.000Z</x:v>
+        <x:v>2024-02-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E135" s="14" t="str">
         <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F135" s="20" t="str">
-        <x:v>Conflicted Analysts and Initial Coin Offerings</x:v>
+        <x:v>The (Limited) Power of Blockchain Networks for Information Provision</x:v>
       </x:c>
       <x:c r="G135" s="20" t="str">
-        <x:v>Andreas Barth; Valerie Laturnus; Sasan Mansouri; Alexander F. Wagner</x:v>
+        <x:v>Benedikt Franke; Qi Gao Fritz; André Stenzel</x:v>
       </x:c>
       <x:c r="H135" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I135" s="20" t="str">
-        <x:v>ICO 分析师利益冲突与评级</x:v>
+        <x:v>企业区块链的信息提供能力与边界</x:v>
       </x:c>
       <x:c r="J135" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K135" s="20" t="str">
-        <x:v>69(11): 6641-6666</x:v>
+        <x:v>70(2): 971-990</x:v>
       </x:c>
       <x:c r="L135" s="22"/>
       <x:c r="M135" s="20" t="str">
-        <x:v>10.1287/mnsc.2021.02928</x:v>
+        <x:v>10.1287/mnsc.2023.4718</x:v>
       </x:c>
       <x:c r="N135" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2021.02928</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2023.4718</x:v>
       </x:c>
       <x:c r="O135" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -7950,44 +7942,44 @@
     </x:row>
     <x:row r="136" ht="46" customHeight="1">
       <x:c r="A136" s="12" t="str">
-        <x:v>P124</x:v>
+        <x:v>P126</x:v>
       </x:c>
       <x:c r="B136" s="18" t="str">
         <x:v>企业披露、财务会计与审计</x:v>
       </x:c>
       <x:c r="C136" s="15" t="n">
-        <x:v>2024</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="D136" s="24" t="d">
-        <x:v>2024-02-01T00:00:00.000Z</x:v>
+        <x:v>2025-05-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E136" s="14" t="str">
         <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F136" s="20" t="str">
-        <x:v>The (Limited) Power of Blockchain Networks for Information Provision</x:v>
+        <x:v>Distributed Ledgers and Secure Multiparty Computation for Financial Reporting and Auditing</x:v>
       </x:c>
       <x:c r="G136" s="20" t="str">
-        <x:v>Benedikt Franke; Qi Gao Fritz; André Stenzel</x:v>
+        <x:v>Sean Shun Cao; Lin William Cong; Baozhong Yang</x:v>
       </x:c>
       <x:c r="H136" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I136" s="20" t="str">
-        <x:v>企业区块链的信息提供能力与边界</x:v>
+        <x:v>分布式账本、安全多方计算与报告审计</x:v>
       </x:c>
       <x:c r="J136" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K136" s="20" t="str">
-        <x:v>70(2): 971-990</x:v>
+        <x:v>71(5): 3852-3872</x:v>
       </x:c>
       <x:c r="L136" s="22"/>
       <x:c r="M136" s="20" t="str">
-        <x:v>10.1287/mnsc.2023.4718</x:v>
+        <x:v>10.1287/mnsc.2023.02577</x:v>
       </x:c>
       <x:c r="N136" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2023.4718</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2023.02577</x:v>
       </x:c>
       <x:c r="O136" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -7997,46 +7989,44 @@
     </x:row>
     <x:row r="137" ht="46" customHeight="1">
       <x:c r="A137" s="12" t="str">
-        <x:v>P125</x:v>
+        <x:v>P129</x:v>
       </x:c>
       <x:c r="B137" s="18" t="str">
         <x:v>企业披露、财务会计与审计</x:v>
       </x:c>
       <x:c r="C137" s="15" t="n">
-        <x:v>2025</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="D137" s="24" t="d">
-        <x:v>2025-05-01T00:00:00.000Z</x:v>
+        <x:v>2026-06-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E137" s="14" t="str">
-        <x:v>TAR</x:v>
+        <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F137" s="20" t="str">
-        <x:v>Using Blockchain, Non-Fungible Tokens, and Smart Contracts to Track and Report Greenhouse Gas Emissions</x:v>
+        <x:v>The Role of Auditor Reputation in an Emerging Audit Marketplace: Evidence from Decentralized Finance (DeFi)</x:v>
       </x:c>
       <x:c r="G137" s="20" t="str">
-        <x:v>J. Gregory Jenkins; Eric M. Negangard; Mark D. Sheldon</x:v>
+        <x:v>W. Robert Knechel; Steven A. Maex; Hyun Jong Park</x:v>
       </x:c>
       <x:c r="H137" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I137" s="20" t="str">
-        <x:v>区块链、NFT 与智能合约支持温室气体排放报告</x:v>
+        <x:v>DeFi 审计市场中的审计师声誉</x:v>
       </x:c>
       <x:c r="J137" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K137" s="20" t="str">
-        <x:v>100(3): 277-305</x:v>
-      </x:c>
-      <x:c r="L137" s="22" t="d">
-        <x:v>2025-04-08T00:00:00.000Z</x:v>
-      </x:c>
+        <x:v>72(6): 5083-5105</x:v>
+      </x:c>
+      <x:c r="L137" s="22"/>
       <x:c r="M137" s="20" t="str">
-        <x:v>10.2308/tar-2023-0222</x:v>
+        <x:v>10.1287/mnsc.2023.02245</x:v>
       </x:c>
       <x:c r="N137" s="20" t="str">
-        <x:v>https://doi.org/10.2308/tar-2023-0222</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2023.02245</x:v>
       </x:c>
       <x:c r="O137" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -8045,94 +8035,94 @@
       <x:c r="Q137" s="20" t="str"/>
     </x:row>
     <x:row r="138" ht="46" customHeight="1">
-      <x:c r="A138" s="12" t="str">
-        <x:v>P126</x:v>
-      </x:c>
-      <x:c r="B138" s="18" t="str">
-        <x:v>企业披露、财务会计与审计</x:v>
-      </x:c>
-      <x:c r="C138" s="15" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="D138" s="24" t="d">
-        <x:v>2025-05-01T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="E138" s="14" t="str">
-        <x:v>Management Science</x:v>
-      </x:c>
-      <x:c r="F138" s="20" t="str">
-        <x:v>Distributed Ledgers and Secure Multiparty Computation for Financial Reporting and Auditing</x:v>
-      </x:c>
-      <x:c r="G138" s="20" t="str">
-        <x:v>Sean Shun Cao; Lin William Cong; Baozhong Yang</x:v>
-      </x:c>
-      <x:c r="H138" s="21" t="str">
-        <x:v>卷期发表</x:v>
-      </x:c>
-      <x:c r="I138" s="20" t="str">
-        <x:v>分布式账本、安全多方计算与报告审计</x:v>
-      </x:c>
-      <x:c r="J138" s="20" t="str">
-        <x:v>直接相关</x:v>
-      </x:c>
-      <x:c r="K138" s="20" t="str">
-        <x:v>71(5): 3852-3872</x:v>
-      </x:c>
-      <x:c r="L138" s="22"/>
-      <x:c r="M138" s="20" t="str">
-        <x:v>10.1287/mnsc.2023.02577</x:v>
-      </x:c>
-      <x:c r="N138" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2023.02577</x:v>
-      </x:c>
-      <x:c r="O138" s="23" t="str">
-        <x:v>打开来源</x:v>
-      </x:c>
-      <x:c r="P138" s="20" t="str"/>
-      <x:c r="Q138" s="20" t="str"/>
+      <x:c r="A138" s="25" t="str">
+        <x:v>P132</x:v>
+      </x:c>
+      <x:c r="B138" s="34" t="str">
+        <x:v>市场操纵、非法活动、网络犯罪与税收</x:v>
+      </x:c>
+      <x:c r="C138" s="27" t="n">
+        <x:v>2018</x:v>
+      </x:c>
+      <x:c r="D138" s="28" t="d">
+        <x:v>2018-05-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E138" s="29" t="str">
+        <x:v>JME</x:v>
+      </x:c>
+      <x:c r="F138" s="30" t="str">
+        <x:v>Price manipulation in the Bitcoin ecosystem</x:v>
+      </x:c>
+      <x:c r="G138" s="30" t="str">
+        <x:v>Neil Gandal; JT Hamrick; Tyler Moore; Tali Oberman</x:v>
+      </x:c>
+      <x:c r="H138" s="31" t="str">
+        <x:v>卷期发表</x:v>
+      </x:c>
+      <x:c r="I138" s="30" t="str">
+        <x:v>比特币交易所价格操纵</x:v>
+      </x:c>
+      <x:c r="J138" s="30" t="str">
+        <x:v>直接相关</x:v>
+      </x:c>
+      <x:c r="K138" s="30" t="str">
+        <x:v>95: 86-96</x:v>
+      </x:c>
+      <x:c r="L138" s="32"/>
+      <x:c r="M138" s="30" t="str">
+        <x:v>10.1016/j.jmoneco.2017.12.004</x:v>
+      </x:c>
+      <x:c r="N138" s="30" t="str">
+        <x:v>https://doi.org/10.1016/j.jmoneco.2017.12.004</x:v>
+      </x:c>
+      <x:c r="O138" s="33" t="str">
+        <x:v>打开来源</x:v>
+      </x:c>
+      <x:c r="P138" s="30"/>
+      <x:c r="Q138" s="30"/>
     </x:row>
     <x:row r="139" ht="46" customHeight="1">
       <x:c r="A139" s="12" t="str">
-        <x:v>P127</x:v>
+        <x:v>P133</x:v>
       </x:c>
       <x:c r="B139" s="18" t="str">
-        <x:v>企业披露、财务会计与审计</x:v>
+        <x:v>市场操纵、非法活动、网络犯罪与税收</x:v>
       </x:c>
       <x:c r="C139" s="15" t="n">
-        <x:v>2025</x:v>
+        <x:v>2019</x:v>
       </x:c>
       <x:c r="D139" s="24" t="d">
-        <x:v>2025-06-01T00:00:00.000Z</x:v>
+        <x:v>2019-05-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E139" s="14" t="str">
-        <x:v>JAR</x:v>
+        <x:v>RFS</x:v>
       </x:c>
       <x:c r="F139" s="20" t="str">
-        <x:v>The Effect of Intangible Asset Classification on Professional Financial Statement Users’ Assessments</x:v>
+        <x:v>Sex, Drugs, and Bitcoin: How Much Illegal Activity Is Financed through Cryptocurrencies?</x:v>
       </x:c>
       <x:c r="G139" s="20" t="str">
-        <x:v>Spencer B. Anderson; Kim I. Mendoza; Cassie Mongold</x:v>
+        <x:v>Sean Foley; Jonathan R Karlsen; Tālis J Putniņš</x:v>
       </x:c>
       <x:c r="H139" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I139" s="20" t="str">
-        <x:v>以加密资产分类为场景的财务报表使用者实验</x:v>
+        <x:v>比特币非法活动的规模与资金流</x:v>
       </x:c>
       <x:c r="J139" s="20" t="str">
-        <x:v>加密场景</x:v>
+        <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K139" s="20" t="str">
-        <x:v>63(3): 1107-1143</x:v>
+        <x:v>32(5): 1798-1853</x:v>
       </x:c>
       <x:c r="L139" s="22" t="d">
-        <x:v>2025-03-04T00:00:00.000Z</x:v>
+        <x:v>2019-04-04T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="M139" s="20" t="str">
-        <x:v>10.1111/1475-679x.12604</x:v>
+        <x:v>10.1093/rfs/hhz015</x:v>
       </x:c>
       <x:c r="N139" s="20" t="str">
-        <x:v>https://doi.org/10.1111/1475-679x.12604</x:v>
+        <x:v>https://doi.org/10.1093/rfs/hhz015</x:v>
       </x:c>
       <x:c r="O139" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -8142,95 +8132,93 @@
     </x:row>
     <x:row r="140" ht="46" customHeight="1">
       <x:c r="A140" s="12" t="str">
-        <x:v>P128</x:v>
+        <x:v>P134</x:v>
       </x:c>
       <x:c r="B140" s="18" t="str">
-        <x:v>企业披露、财务会计与审计</x:v>
+        <x:v>市场操纵、非法活动、网络犯罪与税收</x:v>
       </x:c>
       <x:c r="C140" s="15" t="n">
-        <x:v>2026</x:v>
+        <x:v>2020</x:v>
       </x:c>
       <x:c r="D140" s="24" t="d">
-        <x:v>2026-03-01T00:00:00.000Z</x:v>
+        <x:v>2020-08-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E140" s="14" t="str">
-        <x:v>JAR</x:v>
+        <x:v>JF</x:v>
       </x:c>
       <x:c r="F140" s="20" t="str">
-        <x:v>Accounting for Cryptocurrencies</x:v>
+        <x:v>Is Bitcoin Really Untethered?</x:v>
       </x:c>
       <x:c r="G140" s="20" t="str">
-        <x:v>Chelsea M. Anderson; Vivian W. Fang; James R. Moon Jr.; Jonathan E. Shipman</x:v>
+        <x:v>John M. Griffin; Amin Shams</x:v>
       </x:c>
       <x:c r="H140" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I140" s="20" t="str">
-        <x:v>上市公司加密资产持有与会计处理</x:v>
+        <x:v>Tether 交易与比特币价格操纵</x:v>
       </x:c>
       <x:c r="J140" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K140" s="20" t="str">
-        <x:v>64(1): 45-79</x:v>
+        <x:v>75(4): 1913-1964</x:v>
       </x:c>
       <x:c r="L140" s="22" t="d">
-        <x:v>2025-09-15T00:00:00.000Z</x:v>
+        <x:v>2020-06-15T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="M140" s="20" t="str">
-        <x:v>10.1111/1475-679x.70018</x:v>
+        <x:v>10.1111/jofi.12903</x:v>
       </x:c>
       <x:c r="N140" s="20" t="str">
-        <x:v>https://doi.org/10.1111/1475-679x.70018</x:v>
+        <x:v>https://doi.org/10.1111/jofi.12903</x:v>
       </x:c>
       <x:c r="O140" s="23" t="str">
         <x:v>打开来源</x:v>
       </x:c>
       <x:c r="P140" s="20" t="str"/>
-      <x:c r="Q140" s="20" t="str">
-        <x:v>正式卷期为 2026 年 64(1)，首次在线为 2025-09-15。</x:v>
-      </x:c>
+      <x:c r="Q140" s="20"/>
     </x:row>
     <x:row r="141" ht="46" customHeight="1">
       <x:c r="A141" s="12" t="str">
-        <x:v>P129</x:v>
+        <x:v>P137</x:v>
       </x:c>
       <x:c r="B141" s="18" t="str">
-        <x:v>企业披露、财务会计与审计</x:v>
+        <x:v>市场操纵、非法活动、网络犯罪与税收</x:v>
       </x:c>
       <x:c r="C141" s="15" t="n">
-        <x:v>2026</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="D141" s="24" t="d">
-        <x:v>2026-06-01T00:00:00.000Z</x:v>
+        <x:v>2023-11-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E141" s="14" t="str">
         <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F141" s="20" t="str">
-        <x:v>The Role of Auditor Reputation in an Emerging Audit Marketplace: Evidence from Decentralized Finance (DeFi)</x:v>
+        <x:v>Crypto Wash Trading</x:v>
       </x:c>
       <x:c r="G141" s="20" t="str">
-        <x:v>W. Robert Knechel; Steven A. Maex; Hyun Jong Park</x:v>
+        <x:v>Lin William Cong; Xi Li; Ke Tang; Yang Yang</x:v>
       </x:c>
       <x:c r="H141" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I141" s="20" t="str">
-        <x:v>DeFi 审计市场中的审计师声誉</x:v>
+        <x:v>加密交易所虚假交易量与对刷</x:v>
       </x:c>
       <x:c r="J141" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K141" s="20" t="str">
-        <x:v>72(6): 5083-5105</x:v>
+        <x:v>69(11): 6427-6454</x:v>
       </x:c>
       <x:c r="L141" s="22"/>
       <x:c r="M141" s="20" t="str">
-        <x:v>10.1287/mnsc.2023.02245</x:v>
+        <x:v>10.1287/mnsc.2021.02709</x:v>
       </x:c>
       <x:c r="N141" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2023.02245</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2021.02709</x:v>
       </x:c>
       <x:c r="O141" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -8240,44 +8228,44 @@
     </x:row>
     <x:row r="142" ht="46" customHeight="1">
       <x:c r="A142" s="12" t="str">
-        <x:v>P130</x:v>
+        <x:v>P139</x:v>
       </x:c>
       <x:c r="B142" s="18" t="str">
-        <x:v>企业披露、财务会计与审计</x:v>
+        <x:v>市场操纵、非法活动、网络犯罪与税收</x:v>
       </x:c>
       <x:c r="C142" s="15" t="n">
-        <x:v>2026</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="D142" s="24" t="d">
-        <x:v>2026-07-01T00:00:00.000Z</x:v>
+        <x:v>2024-12-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E142" s="14" t="str">
-        <x:v>JAE</x:v>
+        <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F142" s="20" t="str">
-        <x:v>Auditing smart contracts</x:v>
+        <x:v>Direct Evidence of Bitcoin Wash Trading</x:v>
       </x:c>
       <x:c r="G142" s="20" t="str">
-        <x:v>Wayne Landsman; Evgeny Lyandres; Edward Maydew; Daniel Rabetti; Che Zhang</x:v>
+        <x:v>Arash Aloosh; Jiasun Li</x:v>
       </x:c>
       <x:c r="H142" s="21" t="str">
-        <x:v>在线发表</x:v>
+        <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I142" s="20" t="str">
-        <x:v>DeFi 智能合约审计的决定因素与后果</x:v>
+        <x:v>比特币对刷交易的直接证据</x:v>
       </x:c>
       <x:c r="J142" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K142" s="20" t="str">
-        <x:v>未编入卷期</x:v>
+        <x:v>70(12): 8875-8921</x:v>
       </x:c>
       <x:c r="L142" s="22"/>
       <x:c r="M142" s="20" t="str">
-        <x:v>10.1016/j.jacceco.2026.101911</x:v>
+        <x:v>10.1287/mnsc.2021.01448</x:v>
       </x:c>
       <x:c r="N142" s="20" t="str">
-        <x:v>https://doi.org/10.1016/j.jacceco.2026.101911</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2021.01448</x:v>
       </x:c>
       <x:c r="O142" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -8287,44 +8275,44 @@
     </x:row>
     <x:row r="143" ht="46" customHeight="1">
       <x:c r="A143" s="12" t="str">
-        <x:v>P131</x:v>
+        <x:v>P140</x:v>
       </x:c>
       <x:c r="B143" s="18" t="str">
-        <x:v>企业披露、财务会计与审计</x:v>
+        <x:v>市场操纵、非法活动、网络犯罪与税收</x:v>
       </x:c>
       <x:c r="C143" s="15" t="n">
-        <x:v>2026</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="D143" s="24" t="d">
-        <x:v>2026-07-01T00:00:00.000Z</x:v>
+        <x:v>2025-04-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E143" s="14" t="str">
-        <x:v>JAE</x:v>
+        <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F143" s="20" t="str">
-        <x:v>Discussion of “Auditing smart contracts”: Assurance in the world of decentralized finance</x:v>
+        <x:v>An Anatomy of Crypto-Enabled Cybercrimes</x:v>
       </x:c>
       <x:c r="G143" s="20" t="str">
-        <x:v>Andreas Park</x:v>
+        <x:v>Will Cong; Campbell Harvey; Daniel Rabetti; Zong-Yu Wu</x:v>
       </x:c>
       <x:c r="H143" s="21" t="str">
-        <x:v>在线发表</x:v>
+        <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I143" s="20" t="str">
-        <x:v>对智能合约审计与 DeFi 鉴证的讨论</x:v>
+        <x:v>加密资产支持的网络犯罪及链上资金追踪</x:v>
       </x:c>
       <x:c r="J143" s="20" t="str">
-        <x:v>评论</x:v>
+        <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K143" s="20" t="str">
-        <x:v>未编入卷期</x:v>
+        <x:v>71(4): 3622-3633</x:v>
       </x:c>
       <x:c r="L143" s="22"/>
       <x:c r="M143" s="20" t="str">
-        <x:v>10.1016/j.jacceco.2026.101925</x:v>
+        <x:v>10.1287/mnsc.2023.03691</x:v>
       </x:c>
       <x:c r="N143" s="20" t="str">
-        <x:v>https://doi.org/10.1016/j.jacceco.2026.101925</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2023.03691</x:v>
       </x:c>
       <x:c r="O143" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -8333,94 +8321,92 @@
       <x:c r="Q143" s="20" t="str"/>
     </x:row>
     <x:row r="144" ht="46" customHeight="1">
-      <x:c r="A144" s="25" t="str">
-        <x:v>P132</x:v>
-      </x:c>
-      <x:c r="B144" s="34" t="str">
+      <x:c r="A144" s="12" t="str">
+        <x:v>P141</x:v>
+      </x:c>
+      <x:c r="B144" s="18" t="str">
         <x:v>市场操纵、非法活动、网络犯罪与税收</x:v>
       </x:c>
-      <x:c r="C144" s="27" t="n">
-        <x:v>2018</x:v>
-      </x:c>
-      <x:c r="D144" s="28" t="d">
-        <x:v>2018-05-01T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="E144" s="29" t="str">
-        <x:v>JME</x:v>
-      </x:c>
-      <x:c r="F144" s="30" t="str">
-        <x:v>Price manipulation in the Bitcoin ecosystem</x:v>
-      </x:c>
-      <x:c r="G144" s="30" t="str">
-        <x:v>Neil Gandal; JT Hamrick; Tyler Moore; Tali Oberman</x:v>
-      </x:c>
-      <x:c r="H144" s="31" t="str">
-        <x:v>卷期发表</x:v>
-      </x:c>
-      <x:c r="I144" s="30" t="str">
-        <x:v>比特币交易所价格操纵</x:v>
-      </x:c>
-      <x:c r="J144" s="30" t="str">
-        <x:v>直接相关</x:v>
-      </x:c>
-      <x:c r="K144" s="30" t="str">
-        <x:v>95: 86-96</x:v>
-      </x:c>
-      <x:c r="L144" s="32"/>
-      <x:c r="M144" s="30" t="str">
-        <x:v>10.1016/j.jmoneco.2017.12.004</x:v>
-      </x:c>
-      <x:c r="N144" s="30" t="str">
-        <x:v>https://doi.org/10.1016/j.jmoneco.2017.12.004</x:v>
-      </x:c>
-      <x:c r="O144" s="33" t="str">
-        <x:v>打开来源</x:v>
-      </x:c>
-      <x:c r="P144" s="30" t="str"/>
-      <x:c r="Q144" s="30" t="str"/>
+      <x:c r="C144" s="15" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="D144" s="24" t="d">
+        <x:v>2025-10-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E144" s="14" t="str">
+        <x:v>Management Science</x:v>
+      </x:c>
+      <x:c r="F144" s="20" t="str">
+        <x:v>Trading Volume Manipulation and Competition Among Centralized Crypto Exchanges</x:v>
+      </x:c>
+      <x:c r="G144" s="20" t="str">
+        <x:v>Dan Amiram; Evgeny Lyandres; Daniel Rabetti</x:v>
+      </x:c>
+      <x:c r="H144" s="21" t="str">
+        <x:v>卷期发表</x:v>
+      </x:c>
+      <x:c r="I144" s="20" t="str">
+        <x:v>中心化加密交易所竞争与成交量操纵</x:v>
+      </x:c>
+      <x:c r="J144" s="20" t="str">
+        <x:v>直接相关</x:v>
+      </x:c>
+      <x:c r="K144" s="20" t="str">
+        <x:v>71(10): 8604-8622</x:v>
+      </x:c>
+      <x:c r="L144" s="22"/>
+      <x:c r="M144" s="20" t="str">
+        <x:v>10.1287/mnsc.2021.02903</x:v>
+      </x:c>
+      <x:c r="N144" s="20" t="str">
+        <x:v>https://doi.org/10.1287/mnsc.2021.02903</x:v>
+      </x:c>
+      <x:c r="O144" s="23" t="str">
+        <x:v>打开来源</x:v>
+      </x:c>
+      <x:c r="P144" s="20"/>
+      <x:c r="Q144" s="20"/>
     </x:row>
     <x:row r="145" ht="46" customHeight="1">
       <x:c r="A145" s="12" t="str">
-        <x:v>P133</x:v>
+        <x:v>P142</x:v>
       </x:c>
       <x:c r="B145" s="18" t="str">
         <x:v>市场操纵、非法活动、网络犯罪与税收</x:v>
       </x:c>
       <x:c r="C145" s="15" t="n">
-        <x:v>2019</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="D145" s="24" t="d">
-        <x:v>2019-05-01T00:00:00.000Z</x:v>
+        <x:v>2025-11-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E145" s="14" t="str">
-        <x:v>RFS</x:v>
+        <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F145" s="20" t="str">
-        <x:v>Sex, Drugs, and Bitcoin: How Much Illegal Activity Is Financed through Cryptocurrencies?</x:v>
+        <x:v>The Impact of Cryptocurrency on Cybersecurity</x:v>
       </x:c>
       <x:c r="G145" s="20" t="str">
-        <x:v>Sean Foley; Jonathan R Karlsen; Tālis J Putniņš</x:v>
+        <x:v>Terrence August; Duy Dao; Kihoon Kim; Marius Florin Niculescu</x:v>
       </x:c>
       <x:c r="H145" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I145" s="20" t="str">
-        <x:v>比特币非法活动的规模与资金流</x:v>
+        <x:v>加密货币发展对网络安全激励的影响</x:v>
       </x:c>
       <x:c r="J145" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K145" s="20" t="str">
-        <x:v>32(5): 1798-1853</x:v>
-      </x:c>
-      <x:c r="L145" s="22" t="d">
-        <x:v>2019-04-04T00:00:00.000Z</x:v>
-      </x:c>
+        <x:v>71(11): 9606-9627</x:v>
+      </x:c>
+      <x:c r="L145" s="22"/>
       <x:c r="M145" s="20" t="str">
-        <x:v>10.1093/rfs/hhz015</x:v>
+        <x:v>10.1287/mnsc.2023.00969</x:v>
       </x:c>
       <x:c r="N145" s="20" t="str">
-        <x:v>https://doi.org/10.1093/rfs/hhz015</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2023.00969</x:v>
       </x:c>
       <x:c r="O145" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -8429,96 +8415,94 @@
       <x:c r="Q145" s="20" t="str"/>
     </x:row>
     <x:row r="146" ht="46" customHeight="1">
-      <x:c r="A146" s="12" t="str">
-        <x:v>P134</x:v>
-      </x:c>
-      <x:c r="B146" s="18" t="str">
-        <x:v>市场操纵、非法活动、网络犯罪与税收</x:v>
-      </x:c>
-      <x:c r="C146" s="15" t="n">
-        <x:v>2020</x:v>
-      </x:c>
-      <x:c r="D146" s="24" t="d">
-        <x:v>2020-08-01T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="E146" s="14" t="str">
-        <x:v>JF</x:v>
-      </x:c>
-      <x:c r="F146" s="20" t="str">
-        <x:v>Is Bitcoin Really Untethered?</x:v>
-      </x:c>
-      <x:c r="G146" s="20" t="str">
-        <x:v>John M. Griffin; Amin Shams</x:v>
-      </x:c>
-      <x:c r="H146" s="21" t="str">
-        <x:v>卷期发表</x:v>
-      </x:c>
-      <x:c r="I146" s="20" t="str">
-        <x:v>Tether 交易与比特币价格操纵</x:v>
-      </x:c>
-      <x:c r="J146" s="20" t="str">
-        <x:v>直接相关</x:v>
-      </x:c>
-      <x:c r="K146" s="20" t="str">
-        <x:v>75(4): 1913-1964</x:v>
-      </x:c>
-      <x:c r="L146" s="22" t="d">
-        <x:v>2020-06-15T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="M146" s="20" t="str">
-        <x:v>10.1111/jofi.12903</x:v>
-      </x:c>
-      <x:c r="N146" s="20" t="str">
-        <x:v>https://doi.org/10.1111/jofi.12903</x:v>
-      </x:c>
-      <x:c r="O146" s="23" t="str">
-        <x:v>打开来源</x:v>
-      </x:c>
-      <x:c r="P146" s="20" t="str"/>
-      <x:c r="Q146" s="20" t="str"/>
+      <x:c r="A146" s="25" t="str">
+        <x:v>P143</x:v>
+      </x:c>
+      <x:c r="B146" s="34" t="str">
+        <x:v>供应链、企业应用与金融包容</x:v>
+      </x:c>
+      <x:c r="C146" s="27" t="n">
+        <x:v>2019</x:v>
+      </x:c>
+      <x:c r="D146" s="28" t="d">
+        <x:v>2019-05-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E146" s="29" t="str">
+        <x:v>RFS</x:v>
+      </x:c>
+      <x:c r="F146" s="30" t="str">
+        <x:v>Blockchain-Based Settlement for Asset Trading</x:v>
+      </x:c>
+      <x:c r="G146" s="30" t="str">
+        <x:v>Jonathan Chiu; Thorsten V Koeppl</x:v>
+      </x:c>
+      <x:c r="H146" s="31" t="str">
+        <x:v>卷期发表</x:v>
+      </x:c>
+      <x:c r="I146" s="30" t="str">
+        <x:v>区块链在资产交易结算中的应用</x:v>
+      </x:c>
+      <x:c r="J146" s="30" t="str">
+        <x:v>直接相关</x:v>
+      </x:c>
+      <x:c r="K146" s="30" t="str">
+        <x:v>32(5): 1716-1753</x:v>
+      </x:c>
+      <x:c r="L146" s="32" t="d">
+        <x:v>2019-04-04T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="M146" s="30" t="str">
+        <x:v>10.1093/rfs/hhy122</x:v>
+      </x:c>
+      <x:c r="N146" s="30" t="str">
+        <x:v>https://doi.org/10.1093/rfs/hhy122</x:v>
+      </x:c>
+      <x:c r="O146" s="33" t="str">
+        <x:v>打开来源</x:v>
+      </x:c>
+      <x:c r="P146" s="30"/>
+      <x:c r="Q146" s="30"/>
     </x:row>
     <x:row r="147" ht="46" customHeight="1">
       <x:c r="A147" s="12" t="str">
-        <x:v>P135</x:v>
+        <x:v>P144</x:v>
       </x:c>
       <x:c r="B147" s="18" t="str">
-        <x:v>市场操纵、非法活动、网络犯罪与税收</x:v>
+        <x:v>供应链、企业应用与金融包容</x:v>
       </x:c>
       <x:c r="C147" s="15" t="n">
-        <x:v>2022</x:v>
+        <x:v>2020</x:v>
       </x:c>
       <x:c r="D147" s="24" t="d">
-        <x:v>2022-05-01T00:00:00.000Z</x:v>
+        <x:v>2020-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E147" s="14" t="str">
-        <x:v>JAR</x:v>
+        <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F147" s="20" t="str">
-        <x:v>Coins for Bombs: The Predictive Ability of On‐Chain Transfers for Terrorist Attacks</x:v>
+        <x:v>On the Financing Benefits of Supply Chain Transparency and Blockchain Adoption</x:v>
       </x:c>
       <x:c r="G147" s="20" t="str">
-        <x:v>Dan Amiram; Bjørn N. Jørgensen; Daniel Rabetti</x:v>
+        <x:v>Jiri Chod; Nikolaos Trichakis; Gerry Tsoukalas; Henry Aspegren; Mark Weber</x:v>
       </x:c>
       <x:c r="H147" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I147" s="20" t="str">
-        <x:v>链上资金转移与恐怖袭击的预测</x:v>
+        <x:v>供应链透明度、区块链采用与融资收益</x:v>
       </x:c>
       <x:c r="J147" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K147" s="20" t="str">
-        <x:v>60(2): 427-466</x:v>
-      </x:c>
-      <x:c r="L147" s="22" t="d">
-        <x:v>2022-04-13T00:00:00.000Z</x:v>
-      </x:c>
+        <x:v>66(10): 4378-4396</x:v>
+      </x:c>
+      <x:c r="L147" s="22"/>
       <x:c r="M147" s="20" t="str">
-        <x:v>10.1111/1475-679x.12430</x:v>
+        <x:v>10.1287/mnsc.2019.3434</x:v>
       </x:c>
       <x:c r="N147" s="20" t="str">
-        <x:v>https://doi.org/10.1111/1475-679x.12430</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2019.3434</x:v>
       </x:c>
       <x:c r="O147" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -8528,44 +8512,44 @@
     </x:row>
     <x:row r="148" ht="46" customHeight="1">
       <x:c r="A148" s="12" t="str">
-        <x:v>P136</x:v>
+        <x:v>P145</x:v>
       </x:c>
       <x:c r="B148" s="18" t="str">
-        <x:v>市场操纵、非法活动、网络犯罪与税收</x:v>
+        <x:v>供应链、企业应用与金融包容</x:v>
       </x:c>
       <x:c r="C148" s="15" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="D148" s="24" t="d">
-        <x:v>2023-11-01T00:00:00.000Z</x:v>
+        <x:v>2023-03-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E148" s="14" t="str">
-        <x:v>JAE</x:v>
+        <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F148" s="20" t="str">
-        <x:v>Comment on Cong et al., “Tax loss harvesting with cryptocurrencies”</x:v>
+        <x:v>Impact of Traceability Technology Adoption in Food Supply Chain Networks</x:v>
       </x:c>
       <x:c r="G148" s="20" t="str">
-        <x:v>Reuven Avi-Yonah</x:v>
+        <x:v>Lingxiu Dong; Puping (Phil) Jiang; Fasheng Xu</x:v>
       </x:c>
       <x:c r="H148" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I148" s="20" t="str">
-        <x:v>对加密资产税损收割研究的税务评论</x:v>
+        <x:v>食品供应链中区块链等追溯技术的采用</x:v>
       </x:c>
       <x:c r="J148" s="20" t="str">
-        <x:v>评论</x:v>
+        <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K148" s="20" t="str">
-        <x:v>76(2-3): 101612</x:v>
+        <x:v>69(3): 1518-1535</x:v>
       </x:c>
       <x:c r="L148" s="22"/>
       <x:c r="M148" s="20" t="str">
-        <x:v>10.1016/j.jacceco.2023.101612</x:v>
+        <x:v>10.1287/mnsc.2022.4440</x:v>
       </x:c>
       <x:c r="N148" s="20" t="str">
-        <x:v>https://doi.org/10.1016/j.jacceco.2023.101612</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2022.4440</x:v>
       </x:c>
       <x:c r="O148" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -8575,44 +8559,44 @@
     </x:row>
     <x:row r="149" ht="46" customHeight="1">
       <x:c r="A149" s="12" t="str">
-        <x:v>P137</x:v>
+        <x:v>P146</x:v>
       </x:c>
       <x:c r="B149" s="18" t="str">
-        <x:v>市场操纵、非法活动、网络犯罪与税收</x:v>
+        <x:v>供应链、企业应用与金融包容</x:v>
       </x:c>
       <x:c r="C149" s="15" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="D149" s="24" t="d">
-        <x:v>2023-11-01T00:00:00.000Z</x:v>
+        <x:v>2023-06-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E149" s="14" t="str">
         <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F149" s="20" t="str">
-        <x:v>Crypto Wash Trading</x:v>
+        <x:v>Economics of Permissioned Blockchain Adoption</x:v>
       </x:c>
       <x:c r="G149" s="20" t="str">
-        <x:v>Lin William Cong; Xi Li; Ke Tang; Yang Yang</x:v>
+        <x:v>Garud Iyengar; Fahad Saleh; Jay Sethuraman; Wenjun Wang</x:v>
       </x:c>
       <x:c r="H149" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I149" s="20" t="str">
-        <x:v>加密交易所虚假交易量与对刷</x:v>
+        <x:v>许可链采用的经济条件与激励</x:v>
       </x:c>
       <x:c r="J149" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K149" s="20" t="str">
-        <x:v>69(11): 6427-6454</x:v>
+        <x:v>69(6): 3415-3436</x:v>
       </x:c>
       <x:c r="L149" s="22"/>
       <x:c r="M149" s="20" t="str">
-        <x:v>10.1287/mnsc.2021.02709</x:v>
+        <x:v>10.1287/mnsc.2022.4532</x:v>
       </x:c>
       <x:c r="N149" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2021.02709</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2022.4532</x:v>
       </x:c>
       <x:c r="O149" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -8622,44 +8606,44 @@
     </x:row>
     <x:row r="150" ht="46" customHeight="1">
       <x:c r="A150" s="12" t="str">
-        <x:v>P138</x:v>
+        <x:v>P147</x:v>
       </x:c>
       <x:c r="B150" s="18" t="str">
-        <x:v>市场操纵、非法活动、网络犯罪与税收</x:v>
+        <x:v>供应链、企业应用与金融包容</x:v>
       </x:c>
       <x:c r="C150" s="15" t="n">
-        <x:v>2023</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="D150" s="24" t="d">
-        <x:v>2023-11-01T00:00:00.000Z</x:v>
+        <x:v>2024-01-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E150" s="14" t="str">
-        <x:v>JAE</x:v>
+        <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F150" s="20" t="str">
-        <x:v>Tax-loss harvesting with cryptocurrencies</x:v>
+        <x:v>The Economic Value of Blockchain Applications: Early Evidence from Asset-Backed Securities</x:v>
       </x:c>
       <x:c r="G150" s="20" t="str">
-        <x:v>Lin William Cong; Wayne Landsman; Edward Maydew; Daniel Rabetti</x:v>
+        <x:v>Xia Chen; Qiang Cheng; Ting Luo</x:v>
       </x:c>
       <x:c r="H150" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I150" s="20" t="str">
-        <x:v>加密资产税损收割与投资者交易</x:v>
+        <x:v>资产支持证券中的区块链应用价值</x:v>
       </x:c>
       <x:c r="J150" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K150" s="20" t="str">
-        <x:v>76(2-3): 101607</x:v>
+        <x:v>70(1): 439-463</x:v>
       </x:c>
       <x:c r="L150" s="22"/>
       <x:c r="M150" s="20" t="str">
-        <x:v>10.1016/j.jacceco.2023.101607</x:v>
+        <x:v>10.1287/mnsc.2023.4671</x:v>
       </x:c>
       <x:c r="N150" s="20" t="str">
-        <x:v>https://doi.org/10.1016/j.jacceco.2023.101607</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2023.4671</x:v>
       </x:c>
       <x:c r="O150" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -8669,44 +8653,44 @@
     </x:row>
     <x:row r="151" ht="46" customHeight="1">
       <x:c r="A151" s="12" t="str">
-        <x:v>P139</x:v>
+        <x:v>P148</x:v>
       </x:c>
       <x:c r="B151" s="18" t="str">
-        <x:v>市场操纵、非法活动、网络犯罪与税收</x:v>
+        <x:v>供应链、企业应用与金融包容</x:v>
       </x:c>
       <x:c r="C151" s="15" t="n">
         <x:v>2024</x:v>
       </x:c>
       <x:c r="D151" s="24" t="d">
-        <x:v>2024-12-01T00:00:00.000Z</x:v>
+        <x:v>2024-05-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E151" s="14" t="str">
         <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F151" s="20" t="str">
-        <x:v>Direct Evidence of Bitcoin Wash Trading</x:v>
+        <x:v>Supply Chain Transparency and Blockchain Design</x:v>
       </x:c>
       <x:c r="G151" s="20" t="str">
-        <x:v>Arash Aloosh; Jiasun Li</x:v>
+        <x:v>Yao Cui; Vishal Gaur; Jingchen Liu</x:v>
       </x:c>
       <x:c r="H151" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I151" s="20" t="str">
-        <x:v>比特币对刷交易的直接证据</x:v>
+        <x:v>供应链透明度与区块链设计选择</x:v>
       </x:c>
       <x:c r="J151" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K151" s="20" t="str">
-        <x:v>70(12): 8875-8921</x:v>
+        <x:v>70(5): 3245-3263</x:v>
       </x:c>
       <x:c r="L151" s="22"/>
       <x:c r="M151" s="20" t="str">
-        <x:v>10.1287/mnsc.2021.01448</x:v>
+        <x:v>10.1287/mnsc.2023.4851</x:v>
       </x:c>
       <x:c r="N151" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2021.01448</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2023.4851</x:v>
       </x:c>
       <x:c r="O151" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -8716,91 +8700,97 @@
     </x:row>
     <x:row r="152" ht="46" customHeight="1">
       <x:c r="A152" s="12" t="str">
-        <x:v>P140</x:v>
+        <x:v>P149</x:v>
       </x:c>
       <x:c r="B152" s="18" t="str">
-        <x:v>市场操纵、非法活动、网络犯罪与税收</x:v>
+        <x:v>供应链、企业应用与金融包容</x:v>
       </x:c>
       <x:c r="C152" s="15" t="n">
-        <x:v>2025</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="D152" s="24" t="d">
-        <x:v>2025-04-01T00:00:00.000Z</x:v>
+        <x:v>2024-09-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E152" s="14" t="str">
         <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F152" s="20" t="str">
-        <x:v>An Anatomy of Crypto-Enabled Cybercrimes</x:v>
+        <x:v>Blockchain Adoption in a Supply Chain with Manufacturer Market Power</x:v>
       </x:c>
       <x:c r="G152" s="20" t="str">
-        <x:v>Will Cong; Campbell Harvey; Daniel Rabetti; Zong-Yu Wu</x:v>
+        <x:v>Garud Iyengar; Fahad Saleh; Jay Sethuraman; Wenjun Wang</x:v>
       </x:c>
       <x:c r="H152" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I152" s="20" t="str">
-        <x:v>加密资产支持的网络犯罪及链上资金追踪</x:v>
+        <x:v>制造商市场势力与供应链区块链采用</x:v>
       </x:c>
       <x:c r="J152" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K152" s="20" t="str">
-        <x:v>71(4): 3622-3633</x:v>
-      </x:c>
-      <x:c r="L152" s="22"/>
+        <x:v>70(9): 6158-6178</x:v>
+      </x:c>
+      <x:c r="L152" s="22" t="d">
+        <x:v>2023-10-27T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="M152" s="20" t="str">
-        <x:v>10.1287/mnsc.2023.03691</x:v>
+        <x:v>10.1287/mnsc.2022.02505</x:v>
       </x:c>
       <x:c r="N152" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2023.03691</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2022.02505</x:v>
       </x:c>
       <x:c r="O152" s="23" t="str">
         <x:v>打开来源</x:v>
       </x:c>
-      <x:c r="P152" s="20" t="str"/>
-      <x:c r="Q152" s="20" t="str"/>
+      <x:c r="P152" s="20" t="str">
+        <x:v>https://pubsonline.informs.org/doi/abs/10.1287/mnsc.2022.02505</x:v>
+      </x:c>
+      <x:c r="Q152" s="20" t="str">
+        <x:v>Crossref 仍只有 2023 年在线信息；期刊页面已列 70(9):6158-6178，按 2024 年卷期收录。</x:v>
+      </x:c>
     </x:row>
     <x:row r="153" ht="46" customHeight="1">
       <x:c r="A153" s="12" t="str">
-        <x:v>P141</x:v>
+        <x:v>P150</x:v>
       </x:c>
       <x:c r="B153" s="18" t="str">
-        <x:v>市场操纵、非法活动、网络犯罪与税收</x:v>
+        <x:v>供应链、企业应用与金融包容</x:v>
       </x:c>
       <x:c r="C153" s="15" t="n">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="D153" s="24" t="d">
-        <x:v>2025-10-01T00:00:00.000Z</x:v>
+        <x:v>2025-08-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E153" s="14" t="str">
         <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F153" s="20" t="str">
-        <x:v>Trading Volume Manipulation and Competition Among Centralized Crypto Exchanges</x:v>
+        <x:v>The Blockchain Newsvendor: Value of Freshness Transparency and Smart Contracts</x:v>
       </x:c>
       <x:c r="G153" s="20" t="str">
-        <x:v>Dan Amiram; Evgeny Lyandres; Daniel Rabetti</x:v>
+        <x:v>N. Bora Keskin; Chenghuai Li; Jing-Sheng Song</x:v>
       </x:c>
       <x:c r="H153" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I153" s="20" t="str">
-        <x:v>中心化加密交易所竞争与成交量操纵</x:v>
+        <x:v>生鲜供应链透明度、报童模型与智能合约</x:v>
       </x:c>
       <x:c r="J153" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K153" s="20" t="str">
-        <x:v>71(10): 8604-8622</x:v>
+        <x:v>71(8): 6666-6682</x:v>
       </x:c>
       <x:c r="L153" s="22"/>
       <x:c r="M153" s="20" t="str">
-        <x:v>10.1287/mnsc.2021.02903</x:v>
+        <x:v>10.1287/mnsc.2021.02949</x:v>
       </x:c>
       <x:c r="N153" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2021.02903</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2021.02949</x:v>
       </x:c>
       <x:c r="O153" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -8810,44 +8800,44 @@
     </x:row>
     <x:row r="154" ht="46" customHeight="1">
       <x:c r="A154" s="12" t="str">
-        <x:v>P142</x:v>
+        <x:v>P151</x:v>
       </x:c>
       <x:c r="B154" s="18" t="str">
-        <x:v>市场操纵、非法活动、网络犯罪与税收</x:v>
+        <x:v>供应链、企业应用与金融包容</x:v>
       </x:c>
       <x:c r="C154" s="15" t="n">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="D154" s="24" t="d">
-        <x:v>2025-11-01T00:00:00.000Z</x:v>
+        <x:v>2025-09-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E154" s="14" t="str">
-        <x:v>Management Science</x:v>
+        <x:v>ISR</x:v>
       </x:c>
       <x:c r="F154" s="20" t="str">
-        <x:v>The Impact of Cryptocurrency on Cybersecurity</x:v>
+        <x:v>And No One Gets the Short End of the Stick: A Blockchain-Based Approach to Solving the Two-Sided Opportunism Problem in Interorganizational Information Sharing</x:v>
       </x:c>
       <x:c r="G154" s="20" t="str">
-        <x:v>Terrence August; Duy Dao; Kihoon Kim; Marius Florin Niculescu</x:v>
+        <x:v>Lukas Florian Bossler; Arne Buchwald; Kai Spohrer</x:v>
       </x:c>
       <x:c r="H154" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I154" s="20" t="str">
-        <x:v>加密货币发展对网络安全激励的影响</x:v>
+        <x:v>区块链缓解组织间信息共享的双边机会主义</x:v>
       </x:c>
       <x:c r="J154" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K154" s="20" t="str">
-        <x:v>71(11): 9606-9627</x:v>
+        <x:v>36(3): 1565-1586</x:v>
       </x:c>
       <x:c r="L154" s="22"/>
       <x:c r="M154" s="20" t="str">
-        <x:v>10.1287/mnsc.2023.00969</x:v>
+        <x:v>10.1287/isre.2022.0065</x:v>
       </x:c>
       <x:c r="N154" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2023.00969</x:v>
+        <x:v>https://doi.org/10.1287/isre.2022.0065</x:v>
       </x:c>
       <x:c r="O154" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -8856,94 +8846,94 @@
       <x:c r="Q154" s="20" t="str"/>
     </x:row>
     <x:row r="155" ht="46" customHeight="1">
-      <x:c r="A155" s="25" t="str">
-        <x:v>P143</x:v>
-      </x:c>
-      <x:c r="B155" s="34" t="str">
+      <x:c r="A155" s="12" t="str">
+        <x:v>P152</x:v>
+      </x:c>
+      <x:c r="B155" s="18" t="str">
         <x:v>供应链、企业应用与金融包容</x:v>
       </x:c>
-      <x:c r="C155" s="27" t="n">
-        <x:v>2019</x:v>
-      </x:c>
-      <x:c r="D155" s="28" t="d">
-        <x:v>2019-05-01T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="E155" s="29" t="str">
-        <x:v>RFS</x:v>
-      </x:c>
-      <x:c r="F155" s="30" t="str">
-        <x:v>Blockchain-Based Settlement for Asset Trading</x:v>
-      </x:c>
-      <x:c r="G155" s="30" t="str">
-        <x:v>Jonathan Chiu; Thorsten V Koeppl</x:v>
-      </x:c>
-      <x:c r="H155" s="31" t="str">
-        <x:v>卷期发表</x:v>
-      </x:c>
-      <x:c r="I155" s="30" t="str">
-        <x:v>区块链在资产交易结算中的应用</x:v>
-      </x:c>
-      <x:c r="J155" s="30" t="str">
-        <x:v>直接相关</x:v>
-      </x:c>
-      <x:c r="K155" s="30" t="str">
-        <x:v>32(5): 1716-1753</x:v>
-      </x:c>
-      <x:c r="L155" s="32" t="d">
-        <x:v>2019-04-04T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="M155" s="30" t="str">
-        <x:v>10.1093/rfs/hhy122</x:v>
-      </x:c>
-      <x:c r="N155" s="30" t="str">
-        <x:v>https://doi.org/10.1093/rfs/hhy122</x:v>
-      </x:c>
-      <x:c r="O155" s="33" t="str">
-        <x:v>打开来源</x:v>
-      </x:c>
-      <x:c r="P155" s="30" t="str"/>
-      <x:c r="Q155" s="30" t="str"/>
+      <x:c r="C155" s="15" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="D155" s="16" t="d">
+        <x:v>2026-05-13T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E155" s="14" t="str">
+        <x:v>Management Science</x:v>
+      </x:c>
+      <x:c r="F155" s="20" t="str">
+        <x:v>Financial Inclusion via Blockchain: Evidence from a Natural Experiment</x:v>
+      </x:c>
+      <x:c r="G155" s="20" t="str">
+        <x:v>Shangrong Jiang; Yuze Li; Shouyang Wang</x:v>
+      </x:c>
+      <x:c r="H155" s="21" t="str">
+        <x:v>在线发表</x:v>
+      </x:c>
+      <x:c r="I155" s="20" t="str">
+        <x:v>区块链征信真实性与金融包容的自然实验</x:v>
+      </x:c>
+      <x:c r="J155" s="20" t="str">
+        <x:v>直接相关</x:v>
+      </x:c>
+      <x:c r="K155" s="20" t="str">
+        <x:v>未编入卷期</x:v>
+      </x:c>
+      <x:c r="L155" s="22" t="d">
+        <x:v>2026-05-13T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="M155" s="20" t="str">
+        <x:v>10.1287/mnsc.2023.02303</x:v>
+      </x:c>
+      <x:c r="N155" s="20" t="str">
+        <x:v>https://doi.org/10.1287/mnsc.2023.02303</x:v>
+      </x:c>
+      <x:c r="O155" s="23" t="str">
+        <x:v>打开来源</x:v>
+      </x:c>
+      <x:c r="P155" s="20"/>
+      <x:c r="Q155" s="20"/>
     </x:row>
     <x:row r="156" ht="46" customHeight="1">
       <x:c r="A156" s="12" t="str">
-        <x:v>P144</x:v>
+        <x:v>P153</x:v>
       </x:c>
       <x:c r="B156" s="18" t="str">
         <x:v>供应链、企业应用与金融包容</x:v>
       </x:c>
       <x:c r="C156" s="15" t="n">
-        <x:v>2020</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="D156" s="24" t="d">
-        <x:v>2020-10-01T00:00:00.000Z</x:v>
+        <x:v>2026-08-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E156" s="14" t="str">
         <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F156" s="20" t="str">
-        <x:v>On the Financing Benefits of Supply Chain Transparency and Blockchain Adoption</x:v>
+        <x:v>Behavioral Simulation of Blockchain-Enabled Market for Supplier Capacity Trading Among Retailers</x:v>
       </x:c>
       <x:c r="G156" s="20" t="str">
-        <x:v>Jiri Chod; Nikolaos Trichakis; Gerry Tsoukalas; Henry Aspegren; Mark Weber</x:v>
+        <x:v>Kai Wendt; Volodymyr Babich; Daniel Hellwig; Arnd Huchzermeier</x:v>
       </x:c>
       <x:c r="H156" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I156" s="20" t="str">
-        <x:v>供应链透明度、区块链采用与融资收益</x:v>
+        <x:v>区块链赋能的零售商供应能力交易</x:v>
       </x:c>
       <x:c r="J156" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K156" s="20" t="str">
-        <x:v>66(10): 4378-4396</x:v>
+        <x:v>72(8): 6762-6791</x:v>
       </x:c>
       <x:c r="L156" s="22"/>
       <x:c r="M156" s="20" t="str">
-        <x:v>10.1287/mnsc.2019.3434</x:v>
+        <x:v>10.1287/mnsc.2023.03771</x:v>
       </x:c>
       <x:c r="N156" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2019.3434</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2023.03771</x:v>
       </x:c>
       <x:c r="O156" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -8952,92 +8942,92 @@
       <x:c r="Q156" s="20" t="str"/>
     </x:row>
     <x:row r="157" ht="46" customHeight="1">
-      <x:c r="A157" s="12" t="str">
-        <x:v>P145</x:v>
-      </x:c>
-      <x:c r="B157" s="18" t="str">
-        <x:v>供应链、企业应用与金融包容</x:v>
-      </x:c>
-      <x:c r="C157" s="15" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="D157" s="24" t="d">
-        <x:v>2023-03-01T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="E157" s="14" t="str">
+      <x:c r="A157" s="25" t="str">
+        <x:v>P154</x:v>
+      </x:c>
+      <x:c r="B157" s="34" t="str">
+        <x:v>NFT、艺术品与创作者经济</x:v>
+      </x:c>
+      <x:c r="C157" s="27" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="D157" s="28" t="d">
+        <x:v>2020-10-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E157" s="29" t="str">
         <x:v>Management Science</x:v>
       </x:c>
-      <x:c r="F157" s="20" t="str">
-        <x:v>Impact of Traceability Technology Adoption in Food Supply Chain Networks</x:v>
-      </x:c>
-      <x:c r="G157" s="20" t="str">
-        <x:v>Lingxiu Dong; Puping (Phil) Jiang; Fasheng Xu</x:v>
-      </x:c>
-      <x:c r="H157" s="21" t="str">
-        <x:v>卷期发表</x:v>
-      </x:c>
-      <x:c r="I157" s="20" t="str">
-        <x:v>食品供应链中区块链等追溯技术的采用</x:v>
-      </x:c>
-      <x:c r="J157" s="20" t="str">
-        <x:v>直接相关</x:v>
-      </x:c>
-      <x:c r="K157" s="20" t="str">
-        <x:v>69(3): 1518-1535</x:v>
-      </x:c>
-      <x:c r="L157" s="22"/>
-      <x:c r="M157" s="20" t="str">
-        <x:v>10.1287/mnsc.2022.4440</x:v>
-      </x:c>
-      <x:c r="N157" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2022.4440</x:v>
-      </x:c>
-      <x:c r="O157" s="23" t="str">
-        <x:v>打开来源</x:v>
-      </x:c>
-      <x:c r="P157" s="20" t="str"/>
-      <x:c r="Q157" s="20" t="str"/>
+      <x:c r="F157" s="30" t="str">
+        <x:v>Fractional Equity, Blockchain, and the Future of Creative Work</x:v>
+      </x:c>
+      <x:c r="G157" s="30" t="str">
+        <x:v>Amy Whitaker; Roman Kräussl</x:v>
+      </x:c>
+      <x:c r="H157" s="31" t="str">
+        <x:v>卷期发表</x:v>
+      </x:c>
+      <x:c r="I157" s="30" t="str">
+        <x:v>艺术品权益分割、区块链与创作者收益</x:v>
+      </x:c>
+      <x:c r="J157" s="30" t="str">
+        <x:v>直接相关</x:v>
+      </x:c>
+      <x:c r="K157" s="30" t="str">
+        <x:v>66(10): 4594-4611</x:v>
+      </x:c>
+      <x:c r="L157" s="32"/>
+      <x:c r="M157" s="30" t="str">
+        <x:v>10.1287/mnsc.2020.3633</x:v>
+      </x:c>
+      <x:c r="N157" s="30" t="str">
+        <x:v>https://doi.org/10.1287/mnsc.2020.3633</x:v>
+      </x:c>
+      <x:c r="O157" s="33" t="str">
+        <x:v>打开来源</x:v>
+      </x:c>
+      <x:c r="P157" s="30"/>
+      <x:c r="Q157" s="30"/>
     </x:row>
     <x:row r="158" ht="46" customHeight="1">
       <x:c r="A158" s="12" t="str">
-        <x:v>P146</x:v>
+        <x:v>P155</x:v>
       </x:c>
       <x:c r="B158" s="18" t="str">
-        <x:v>供应链、企业应用与金融包容</x:v>
+        <x:v>NFT、艺术品与创作者经济</x:v>
       </x:c>
       <x:c r="C158" s="15" t="n">
-        <x:v>2023</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="D158" s="24" t="d">
-        <x:v>2023-06-01T00:00:00.000Z</x:v>
+        <x:v>2025-09-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E158" s="14" t="str">
-        <x:v>Management Science</x:v>
+        <x:v>ISR</x:v>
       </x:c>
       <x:c r="F158" s="20" t="str">
-        <x:v>Economics of Permissioned Blockchain Adoption</x:v>
+        <x:v>Resale Royalty in Non-Fungible Token Marketplaces: Blessing or Burden for Creators and Platforms?</x:v>
       </x:c>
       <x:c r="G158" s="20" t="str">
-        <x:v>Garud Iyengar; Fahad Saleh; Jay Sethuraman; Wenjun Wang</x:v>
+        <x:v>Murat M. Tunc; Hasan Cavusoglu; Zhiqiang (Eric) Zheng</x:v>
       </x:c>
       <x:c r="H158" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I158" s="20" t="str">
-        <x:v>许可链采用的经济条件与激励</x:v>
+        <x:v>NFT 二次销售版税对创作者与平台的影响</x:v>
       </x:c>
       <x:c r="J158" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K158" s="20" t="str">
-        <x:v>69(6): 3415-3436</x:v>
+        <x:v>36(3): 1543-1564</x:v>
       </x:c>
       <x:c r="L158" s="22"/>
       <x:c r="M158" s="20" t="str">
-        <x:v>10.1287/mnsc.2022.4532</x:v>
+        <x:v>10.1287/isre.2023.0035</x:v>
       </x:c>
       <x:c r="N158" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2022.4532</x:v>
+        <x:v>https://doi.org/10.1287/isre.2023.0035</x:v>
       </x:c>
       <x:c r="O158" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -9047,44 +9037,46 @@
     </x:row>
     <x:row r="159" ht="46" customHeight="1">
       <x:c r="A159" s="12" t="str">
-        <x:v>P147</x:v>
+        <x:v>P156</x:v>
       </x:c>
       <x:c r="B159" s="18" t="str">
-        <x:v>供应链、企业应用与金融包容</x:v>
+        <x:v>NFT、艺术品与创作者经济</x:v>
       </x:c>
       <x:c r="C159" s="15" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="D159" s="24" t="d">
-        <x:v>2024-01-01T00:00:00.000Z</x:v>
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="D159" s="16" t="d">
+        <x:v>2026-03-04T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E159" s="14" t="str">
-        <x:v>Management Science</x:v>
+        <x:v>MISQ</x:v>
       </x:c>
       <x:c r="F159" s="20" t="str">
-        <x:v>The Economic Value of Blockchain Applications: Early Evidence from Asset-Backed Securities</x:v>
+        <x:v>Extending the Digital Divide: The Role of Unequal Analytical Abilities</x:v>
       </x:c>
       <x:c r="G159" s="20" t="str">
-        <x:v>Xia Chen; Qiang Cheng; Ting Luo</x:v>
+        <x:v>Hong Zhang; Zhiqiang (Eric) Zheng; Amit Mehra</x:v>
       </x:c>
       <x:c r="H159" s="21" t="str">
-        <x:v>卷期发表</x:v>
+        <x:v>在线发表</x:v>
       </x:c>
       <x:c r="I159" s="20" t="str">
-        <x:v>资产支持证券中的区块链应用价值</x:v>
+        <x:v>NFT 市场上的分析能力差异与交易表现</x:v>
       </x:c>
       <x:c r="J159" s="20" t="str">
-        <x:v>直接相关</x:v>
+        <x:v>加密场景</x:v>
       </x:c>
       <x:c r="K159" s="20" t="str">
-        <x:v>70(1): 439-463</x:v>
-      </x:c>
-      <x:c r="L159" s="22"/>
+        <x:v>未编入卷期</x:v>
+      </x:c>
+      <x:c r="L159" s="22" t="d">
+        <x:v>2026-03-04T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="M159" s="20" t="str">
-        <x:v>10.1287/mnsc.2023.4671</x:v>
+        <x:v>10.25300/misq/2026/19079</x:v>
       </x:c>
       <x:c r="N159" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2023.4671</x:v>
+        <x:v>https://doi.org/10.25300/MISQ/2026/19079</x:v>
       </x:c>
       <x:c r="O159" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -9094,44 +9086,46 @@
     </x:row>
     <x:row r="160" ht="46" customHeight="1">
       <x:c r="A160" s="12" t="str">
-        <x:v>P148</x:v>
+        <x:v>P157</x:v>
       </x:c>
       <x:c r="B160" s="18" t="str">
-        <x:v>供应链、企业应用与金融包容</x:v>
+        <x:v>NFT、艺术品与创作者经济</x:v>
       </x:c>
       <x:c r="C160" s="15" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="D160" s="24" t="d">
-        <x:v>2024-05-01T00:00:00.000Z</x:v>
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="D160" s="16" t="d">
+        <x:v>2026-04-21T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E160" s="14" t="str">
-        <x:v>Management Science</x:v>
+        <x:v>ISR</x:v>
       </x:c>
       <x:c r="F160" s="20" t="str">
-        <x:v>Supply Chain Transparency and Blockchain Design</x:v>
+        <x:v>The Market Consequences of Perceived Strategic Generosity: An Empirical Examination of NFT Charity Fundraisers</x:v>
       </x:c>
       <x:c r="G160" s="20" t="str">
-        <x:v>Yao Cui; Vishal Gaur; Jingchen Liu</x:v>
+        <x:v>Chen Liang; Murat Tunç; Gordon Burtch</x:v>
       </x:c>
       <x:c r="H160" s="21" t="str">
-        <x:v>卷期发表</x:v>
+        <x:v>在线发表</x:v>
       </x:c>
       <x:c r="I160" s="20" t="str">
-        <x:v>供应链透明度与区块链设计选择</x:v>
+        <x:v>NFT 慈善募资中的战略慷慨及市场反应</x:v>
       </x:c>
       <x:c r="J160" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K160" s="20" t="str">
-        <x:v>70(5): 3245-3263</x:v>
-      </x:c>
-      <x:c r="L160" s="22"/>
+        <x:v>未编入卷期</x:v>
+      </x:c>
+      <x:c r="L160" s="22" t="d">
+        <x:v>2026-04-21T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="M160" s="20" t="str">
-        <x:v>10.1287/mnsc.2023.4851</x:v>
+        <x:v>10.1287/isre.2024.1004</x:v>
       </x:c>
       <x:c r="N160" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2023.4851</x:v>
+        <x:v>https://doi.org/10.1287/isre.2024.1004</x:v>
       </x:c>
       <x:c r="O160" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -9141,97 +9135,93 @@
     </x:row>
     <x:row r="161" ht="46" customHeight="1">
       <x:c r="A161" s="12" t="str">
-        <x:v>P149</x:v>
+        <x:v>P158</x:v>
       </x:c>
       <x:c r="B161" s="18" t="str">
-        <x:v>供应链、企业应用与金融包容</x:v>
+        <x:v>NFT、艺术品与创作者经济</x:v>
       </x:c>
       <x:c r="C161" s="15" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="D161" s="24" t="d">
-        <x:v>2024-09-01T00:00:00.000Z</x:v>
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="D161" s="16" t="d">
+        <x:v>2026-08-04T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E161" s="14" t="str">
         <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F161" s="20" t="str">
-        <x:v>Blockchain Adoption in a Supply Chain with Manufacturer Market Power</x:v>
+        <x:v>From Canvas to Blockchain: Impact of Royalties on Art Market Efficiency</x:v>
       </x:c>
       <x:c r="G161" s="20" t="str">
-        <x:v>Garud Iyengar; Fahad Saleh; Jay Sethuraman; Wenjun Wang</x:v>
+        <x:v>Xinyu Cao; Jieteng Chen; T. Tony Ke</x:v>
       </x:c>
       <x:c r="H161" s="21" t="str">
-        <x:v>卷期发表</x:v>
+        <x:v>在线发表</x:v>
       </x:c>
       <x:c r="I161" s="20" t="str">
-        <x:v>制造商市场势力与供应链区块链采用</x:v>
+        <x:v>区块链艺术品版税与市场效率</x:v>
       </x:c>
       <x:c r="J161" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K161" s="20" t="str">
-        <x:v>70(9): 6158-6178</x:v>
+        <x:v>未编入卷期</x:v>
       </x:c>
       <x:c r="L161" s="22" t="d">
-        <x:v>2023-10-27T00:00:00.000Z</x:v>
+        <x:v>2026-08-04T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="M161" s="20" t="str">
-        <x:v>10.1287/mnsc.2022.02505</x:v>
+        <x:v>10.1287/mnsc.2023.03810</x:v>
       </x:c>
       <x:c r="N161" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2022.02505</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2023.03810</x:v>
       </x:c>
       <x:c r="O161" s="23" t="str">
         <x:v>打开来源</x:v>
       </x:c>
-      <x:c r="P161" s="20" t="str">
-        <x:v>https://pubsonline.informs.org/doi/abs/10.1287/mnsc.2022.02505</x:v>
-      </x:c>
-      <x:c r="Q161" s="20" t="str">
-        <x:v>Crossref 仍只有 2023 年在线信息；期刊页面已列 70(9):6158-6178，按 2024 年卷期收录。</x:v>
-      </x:c>
+      <x:c r="P161" s="20"/>
+      <x:c r="Q161" s="20"/>
     </x:row>
     <x:row r="162" ht="46" customHeight="1">
       <x:c r="A162" s="12" t="str">
-        <x:v>P150</x:v>
+        <x:v>P159</x:v>
       </x:c>
       <x:c r="B162" s="18" t="str">
-        <x:v>供应链、企业应用与金融包容</x:v>
+        <x:v>NFT、艺术品与创作者经济</x:v>
       </x:c>
       <x:c r="C162" s="15" t="n">
-        <x:v>2025</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="D162" s="24" t="d">
-        <x:v>2025-08-01T00:00:00.000Z</x:v>
+        <x:v>2026-09-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E162" s="14" t="str">
-        <x:v>Management Science</x:v>
+        <x:v>ISR</x:v>
       </x:c>
       <x:c r="F162" s="20" t="str">
-        <x:v>The Blockchain Newsvendor: Value of Freshness Transparency and Smart Contracts</x:v>
+        <x:v>NFT Disruption in Platform Competition: Evidence from Trading Card Collectibles</x:v>
       </x:c>
       <x:c r="G162" s="20" t="str">
-        <x:v>N. Bora Keskin; Chenghuai Li; Jing-Sheng Song</x:v>
+        <x:v>Ioannis Filippos Kanellopoulos; Dominik Gutt; Ting Li</x:v>
       </x:c>
       <x:c r="H162" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I162" s="20" t="str">
-        <x:v>生鲜供应链透明度、报童模型与智能合约</x:v>
+        <x:v>NFT 对收藏卡交易平台竞争的影响</x:v>
       </x:c>
       <x:c r="J162" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K162" s="20" t="str">
-        <x:v>71(8): 6666-6682</x:v>
+        <x:v>37(3): 1596-1620</x:v>
       </x:c>
       <x:c r="L162" s="22"/>
       <x:c r="M162" s="20" t="str">
-        <x:v>10.1287/mnsc.2021.02949</x:v>
+        <x:v>10.1287/isre.2024.0829</x:v>
       </x:c>
       <x:c r="N162" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2021.02949</x:v>
+        <x:v>https://doi.org/10.1287/isre.2024.0829</x:v>
       </x:c>
       <x:c r="O162" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -9241,44 +9231,44 @@
     </x:row>
     <x:row r="163" ht="46" customHeight="1">
       <x:c r="A163" s="12" t="str">
-        <x:v>P151</x:v>
+        <x:v>P160</x:v>
       </x:c>
       <x:c r="B163" s="18" t="str">
-        <x:v>供应链、企业应用与金融包容</x:v>
+        <x:v>NFT、艺术品与创作者经济</x:v>
       </x:c>
       <x:c r="C163" s="15" t="n">
-        <x:v>2025</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="D163" s="24" t="d">
-        <x:v>2025-09-01T00:00:00.000Z</x:v>
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E163" s="14" t="str">
-        <x:v>ISR</x:v>
+        <x:v>Management Science</x:v>
       </x:c>
       <x:c r="F163" s="20" t="str">
-        <x:v>And No One Gets the Short End of the Stick: A Blockchain-Based Approach to Solving the Two-Sided Opportunism Problem in Interorganizational Information Sharing</x:v>
+        <x:v>Chasing Market Growth and Matching Performance in Two-Sided Platforms: Evidence from the Lazy-Minting Policy in an NFT Marketplace</x:v>
       </x:c>
       <x:c r="G163" s="20" t="str">
-        <x:v>Lukas Florian Bossler; Arne Buchwald; Kai Spohrer</x:v>
+        <x:v>Hong Zhang; Hongchang Wang; Amit Mehra; Zhiqiang (Eric) Zheng</x:v>
       </x:c>
       <x:c r="H163" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I163" s="20" t="str">
-        <x:v>区块链缓解组织间信息共享的双边机会主义</x:v>
+        <x:v>NFT 市场懒铸造政策、增长与匹配效率</x:v>
       </x:c>
       <x:c r="J163" s="20" t="str">
         <x:v>直接相关</x:v>
       </x:c>
       <x:c r="K163" s="20" t="str">
-        <x:v>36(3): 1565-1586</x:v>
+        <x:v>72(10): 8416-8439</x:v>
       </x:c>
       <x:c r="L163" s="22"/>
       <x:c r="M163" s="20" t="str">
-        <x:v>10.1287/isre.2022.0065</x:v>
+        <x:v>10.1287/mnsc.2022.03573</x:v>
       </x:c>
       <x:c r="N163" s="20" t="str">
-        <x:v>https://doi.org/10.1287/isre.2022.0065</x:v>
+        <x:v>https://doi.org/10.1287/mnsc.2022.03573</x:v>
       </x:c>
       <x:c r="O163" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -9287,666 +9277,406 @@
       <x:c r="Q163" s="20" t="str"/>
     </x:row>
     <x:row r="164" ht="46" customHeight="1">
-      <x:c r="A164" s="12" t="str">
-        <x:v>P152</x:v>
-      </x:c>
-      <x:c r="B164" s="18" t="str">
-        <x:v>供应链、企业应用与金融包容</x:v>
-      </x:c>
-      <x:c r="C164" s="15" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="D164" s="16" t="d">
-        <x:v>2026-05-13T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="E164" s="14" t="str">
+      <x:c r="A164" s="25" t="str">
+        <x:v>P161</x:v>
+      </x:c>
+      <x:c r="B164" s="34" t="str">
+        <x:v>综述与研究议程</x:v>
+      </x:c>
+      <x:c r="C164" s="27" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="D164" s="28" t="d">
+        <x:v>2023-11-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E164" s="29" t="str">
         <x:v>Management Science</x:v>
       </x:c>
-      <x:c r="F164" s="20" t="str">
-        <x:v>Financial Inclusion via Blockchain: Evidence from a Natural Experiment</x:v>
-      </x:c>
-      <x:c r="G164" s="20" t="str">
-        <x:v>Shangrong Jiang; Yuze Li; Shouyang Wang</x:v>
-      </x:c>
-      <x:c r="H164" s="21" t="str">
-        <x:v>在线发表</x:v>
-      </x:c>
-      <x:c r="I164" s="20" t="str">
-        <x:v>区块链征信真实性与金融包容的自然实验</x:v>
-      </x:c>
-      <x:c r="J164" s="20" t="str">
-        <x:v>直接相关</x:v>
-      </x:c>
-      <x:c r="K164" s="20" t="str">
-        <x:v>未编入卷期</x:v>
-      </x:c>
-      <x:c r="L164" s="22" t="d">
-        <x:v>2026-05-13T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="M164" s="20" t="str">
-        <x:v>10.1287/mnsc.2023.02303</x:v>
-      </x:c>
-      <x:c r="N164" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2023.02303</x:v>
-      </x:c>
-      <x:c r="O164" s="23" t="str">
-        <x:v>打开来源</x:v>
-      </x:c>
-      <x:c r="P164" s="20" t="str"/>
-      <x:c r="Q164" s="20" t="str"/>
+      <x:c r="F164" s="30" t="str">
+        <x:v>Advances in Blockchain and Crypto Economics</x:v>
+      </x:c>
+      <x:c r="G164" s="30" t="str">
+        <x:v>Bruno Biais; Agostino Capponi; Lin William Cong; Vishal Gaur; Kay Giesecke</x:v>
+      </x:c>
+      <x:c r="H164" s="31" t="str">
+        <x:v>卷期发表</x:v>
+      </x:c>
+      <x:c r="I164" s="30" t="str">
+        <x:v>区块链与加密经济学专辑导论及研究议程</x:v>
+      </x:c>
+      <x:c r="J164" s="30" t="str">
+        <x:v>综述导论</x:v>
+      </x:c>
+      <x:c r="K164" s="30" t="str">
+        <x:v>69(11): 6417-6426</x:v>
+      </x:c>
+      <x:c r="L164" s="32"/>
+      <x:c r="M164" s="30" t="str">
+        <x:v>10.1287/mnsc.2023.intro.v69.n11</x:v>
+      </x:c>
+      <x:c r="N164" s="30" t="str">
+        <x:v>https://doi.org/10.1287/mnsc.2023.intro.v69.n11</x:v>
+      </x:c>
+      <x:c r="O164" s="33" t="str">
+        <x:v>打开来源</x:v>
+      </x:c>
+      <x:c r="P164" s="30"/>
+      <x:c r="Q164" s="30"/>
     </x:row>
     <x:row r="165" ht="46" customHeight="1">
-      <x:c r="A165" s="12" t="str">
-        <x:v>P153</x:v>
-      </x:c>
-      <x:c r="B165" s="18" t="str">
-        <x:v>供应链、企业应用与金融包容</x:v>
-      </x:c>
-      <x:c r="C165" s="15" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="D165" s="24" t="d">
-        <x:v>2026-08-01T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="E165" s="14" t="str">
-        <x:v>Management Science</x:v>
-      </x:c>
-      <x:c r="F165" s="20" t="str">
-        <x:v>Behavioral Simulation of Blockchain-Enabled Market for Supplier Capacity Trading Among Retailers</x:v>
-      </x:c>
-      <x:c r="G165" s="20" t="str">
-        <x:v>Kai Wendt; Volodymyr Babich; Daniel Hellwig; Arnd Huchzermeier</x:v>
-      </x:c>
-      <x:c r="H165" s="21" t="str">
-        <x:v>卷期发表</x:v>
-      </x:c>
-      <x:c r="I165" s="20" t="str">
-        <x:v>区块链赋能的零售商供应能力交易</x:v>
-      </x:c>
-      <x:c r="J165" s="20" t="str">
-        <x:v>直接相关</x:v>
-      </x:c>
-      <x:c r="K165" s="20" t="str">
-        <x:v>72(8): 6762-6791</x:v>
-      </x:c>
-      <x:c r="L165" s="22"/>
-      <x:c r="M165" s="20" t="str">
-        <x:v>10.1287/mnsc.2023.03771</x:v>
-      </x:c>
-      <x:c r="N165" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2023.03771</x:v>
-      </x:c>
-      <x:c r="O165" s="23" t="str">
-        <x:v>打开来源</x:v>
-      </x:c>
-      <x:c r="P165" s="20" t="str"/>
-      <x:c r="Q165" s="20" t="str"/>
+      <x:c r="A165"/>
+      <x:c r="B165"/>
+      <x:c r="C165"/>
+      <x:c r="D165"/>
+      <x:c r="E165"/>
+      <x:c r="F165"/>
+      <x:c r="G165"/>
+      <x:c r="H165"/>
+      <x:c r="I165"/>
+      <x:c r="J165"/>
+      <x:c r="K165"/>
+      <x:c r="L165"/>
+      <x:c r="M165"/>
+      <x:c r="N165"/>
+      <x:c r="O165"/>
+      <x:c r="P165"/>
+      <x:c r="Q165"/>
     </x:row>
     <x:row r="166" ht="46" customHeight="1">
-      <x:c r="A166" s="25" t="str">
-        <x:v>P154</x:v>
-      </x:c>
-      <x:c r="B166" s="34" t="str">
-        <x:v>NFT、艺术品与创作者经济</x:v>
-      </x:c>
-      <x:c r="C166" s="27" t="n">
-        <x:v>2020</x:v>
-      </x:c>
-      <x:c r="D166" s="28" t="d">
-        <x:v>2020-10-01T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="E166" s="29" t="str">
-        <x:v>Management Science</x:v>
-      </x:c>
-      <x:c r="F166" s="30" t="str">
-        <x:v>Fractional Equity, Blockchain, and the Future of Creative Work</x:v>
-      </x:c>
-      <x:c r="G166" s="30" t="str">
-        <x:v>Amy Whitaker; Roman Kräussl</x:v>
-      </x:c>
-      <x:c r="H166" s="31" t="str">
-        <x:v>卷期发表</x:v>
-      </x:c>
-      <x:c r="I166" s="30" t="str">
-        <x:v>艺术品权益分割、区块链与创作者收益</x:v>
-      </x:c>
-      <x:c r="J166" s="30" t="str">
-        <x:v>直接相关</x:v>
-      </x:c>
-      <x:c r="K166" s="30" t="str">
-        <x:v>66(10): 4594-4611</x:v>
-      </x:c>
-      <x:c r="L166" s="32"/>
-      <x:c r="M166" s="30" t="str">
-        <x:v>10.1287/mnsc.2020.3633</x:v>
-      </x:c>
-      <x:c r="N166" s="30" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2020.3633</x:v>
-      </x:c>
-      <x:c r="O166" s="33" t="str">
-        <x:v>打开来源</x:v>
-      </x:c>
-      <x:c r="P166" s="30" t="str"/>
-      <x:c r="Q166" s="30" t="str"/>
+      <x:c r="A166"/>
+      <x:c r="B166"/>
+      <x:c r="C166"/>
+      <x:c r="D166"/>
+      <x:c r="E166"/>
+      <x:c r="F166"/>
+      <x:c r="G166"/>
+      <x:c r="H166"/>
+      <x:c r="I166"/>
+      <x:c r="J166"/>
+      <x:c r="K166"/>
+      <x:c r="L166"/>
+      <x:c r="M166"/>
+      <x:c r="N166"/>
+      <x:c r="O166"/>
+      <x:c r="P166"/>
+      <x:c r="Q166"/>
     </x:row>
     <x:row r="167" ht="46" customHeight="1">
-      <x:c r="A167" s="12" t="str">
-        <x:v>P155</x:v>
-      </x:c>
-      <x:c r="B167" s="18" t="str">
-        <x:v>NFT、艺术品与创作者经济</x:v>
-      </x:c>
-      <x:c r="C167" s="15" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="D167" s="24" t="d">
-        <x:v>2025-09-01T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="E167" s="14" t="str">
-        <x:v>ISR</x:v>
-      </x:c>
-      <x:c r="F167" s="20" t="str">
-        <x:v>Resale Royalty in Non-Fungible Token Marketplaces: Blessing or Burden for Creators and Platforms?</x:v>
-      </x:c>
-      <x:c r="G167" s="20" t="str">
-        <x:v>Murat M. Tunc; Hasan Cavusoglu; Zhiqiang (Eric) Zheng</x:v>
-      </x:c>
-      <x:c r="H167" s="21" t="str">
-        <x:v>卷期发表</x:v>
-      </x:c>
-      <x:c r="I167" s="20" t="str">
-        <x:v>NFT 二次销售版税对创作者与平台的影响</x:v>
-      </x:c>
-      <x:c r="J167" s="20" t="str">
-        <x:v>直接相关</x:v>
-      </x:c>
-      <x:c r="K167" s="20" t="str">
-        <x:v>36(3): 1543-1564</x:v>
-      </x:c>
-      <x:c r="L167" s="22"/>
-      <x:c r="M167" s="20" t="str">
-        <x:v>10.1287/isre.2023.0035</x:v>
-      </x:c>
-      <x:c r="N167" s="20" t="str">
-        <x:v>https://doi.org/10.1287/isre.2023.0035</x:v>
-      </x:c>
-      <x:c r="O167" s="23" t="str">
-        <x:v>打开来源</x:v>
-      </x:c>
-      <x:c r="P167" s="20" t="str"/>
-      <x:c r="Q167" s="20" t="str"/>
+      <x:c r="A167"/>
+      <x:c r="B167"/>
+      <x:c r="C167"/>
+      <x:c r="D167"/>
+      <x:c r="E167"/>
+      <x:c r="F167"/>
+      <x:c r="G167"/>
+      <x:c r="H167"/>
+      <x:c r="I167"/>
+      <x:c r="J167"/>
+      <x:c r="K167"/>
+      <x:c r="L167"/>
+      <x:c r="M167"/>
+      <x:c r="N167"/>
+      <x:c r="O167"/>
+      <x:c r="P167"/>
+      <x:c r="Q167"/>
     </x:row>
     <x:row r="168" ht="46" customHeight="1">
-      <x:c r="A168" s="12" t="str">
-        <x:v>P156</x:v>
-      </x:c>
-      <x:c r="B168" s="18" t="str">
-        <x:v>NFT、艺术品与创作者经济</x:v>
-      </x:c>
-      <x:c r="C168" s="15" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="D168" s="16" t="d">
-        <x:v>2026-03-04T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="E168" s="14" t="str">
-        <x:v>MISQ</x:v>
-      </x:c>
-      <x:c r="F168" s="20" t="str">
-        <x:v>Extending the Digital Divide: The Role of Unequal Analytical Abilities</x:v>
-      </x:c>
-      <x:c r="G168" s="20" t="str">
-        <x:v>Hong Zhang; Zhiqiang (Eric) Zheng; Amit Mehra</x:v>
-      </x:c>
-      <x:c r="H168" s="21" t="str">
-        <x:v>在线发表</x:v>
-      </x:c>
-      <x:c r="I168" s="20" t="str">
-        <x:v>NFT 市场上的分析能力差异与交易表现</x:v>
-      </x:c>
-      <x:c r="J168" s="20" t="str">
-        <x:v>加密场景</x:v>
-      </x:c>
-      <x:c r="K168" s="20" t="str">
-        <x:v>未编入卷期</x:v>
-      </x:c>
-      <x:c r="L168" s="22" t="d">
-        <x:v>2026-03-04T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="M168" s="20" t="str">
-        <x:v>10.25300/misq/2026/19079</x:v>
-      </x:c>
-      <x:c r="N168" s="20" t="str">
-        <x:v>https://doi.org/10.25300/MISQ/2026/19079</x:v>
-      </x:c>
-      <x:c r="O168" s="23" t="str">
-        <x:v>打开来源</x:v>
-      </x:c>
-      <x:c r="P168" s="20" t="str"/>
-      <x:c r="Q168" s="20" t="str"/>
+      <x:c r="A168"/>
+      <x:c r="B168"/>
+      <x:c r="C168"/>
+      <x:c r="D168"/>
+      <x:c r="E168"/>
+      <x:c r="F168"/>
+      <x:c r="G168"/>
+      <x:c r="H168"/>
+      <x:c r="I168"/>
+      <x:c r="J168"/>
+      <x:c r="K168"/>
+      <x:c r="L168"/>
+      <x:c r="M168"/>
+      <x:c r="N168"/>
+      <x:c r="O168"/>
+      <x:c r="P168"/>
+      <x:c r="Q168"/>
     </x:row>
     <x:row r="169" ht="46" customHeight="1">
-      <x:c r="A169" s="12" t="str">
-        <x:v>P157</x:v>
-      </x:c>
-      <x:c r="B169" s="18" t="str">
-        <x:v>NFT、艺术品与创作者经济</x:v>
-      </x:c>
-      <x:c r="C169" s="15" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="D169" s="16" t="d">
-        <x:v>2026-04-21T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="E169" s="14" t="str">
-        <x:v>ISR</x:v>
-      </x:c>
-      <x:c r="F169" s="20" t="str">
-        <x:v>The Market Consequences of Perceived Strategic Generosity: An Empirical Examination of NFT Charity Fundraisers</x:v>
-      </x:c>
-      <x:c r="G169" s="20" t="str">
-        <x:v>Chen Liang; Murat Tunç; Gordon Burtch</x:v>
-      </x:c>
-      <x:c r="H169" s="21" t="str">
-        <x:v>在线发表</x:v>
-      </x:c>
-      <x:c r="I169" s="20" t="str">
-        <x:v>NFT 慈善募资中的战略慷慨及市场反应</x:v>
-      </x:c>
-      <x:c r="J169" s="20" t="str">
-        <x:v>直接相关</x:v>
-      </x:c>
-      <x:c r="K169" s="20" t="str">
-        <x:v>未编入卷期</x:v>
-      </x:c>
-      <x:c r="L169" s="22" t="d">
-        <x:v>2026-04-21T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="M169" s="20" t="str">
-        <x:v>10.1287/isre.2024.1004</x:v>
-      </x:c>
-      <x:c r="N169" s="20" t="str">
-        <x:v>https://doi.org/10.1287/isre.2024.1004</x:v>
-      </x:c>
-      <x:c r="O169" s="23" t="str">
-        <x:v>打开来源</x:v>
-      </x:c>
-      <x:c r="P169" s="20" t="str"/>
-      <x:c r="Q169" s="20" t="str"/>
+      <x:c r="A169"/>
+      <x:c r="B169"/>
+      <x:c r="C169"/>
+      <x:c r="D169"/>
+      <x:c r="E169"/>
+      <x:c r="F169"/>
+      <x:c r="G169"/>
+      <x:c r="H169"/>
+      <x:c r="I169"/>
+      <x:c r="J169"/>
+      <x:c r="K169"/>
+      <x:c r="L169"/>
+      <x:c r="M169"/>
+      <x:c r="N169"/>
+      <x:c r="O169"/>
+      <x:c r="P169"/>
+      <x:c r="Q169"/>
     </x:row>
     <x:row r="170" ht="46" customHeight="1">
-      <x:c r="A170" s="12" t="str">
-        <x:v>P158</x:v>
-      </x:c>
-      <x:c r="B170" s="18" t="str">
-        <x:v>NFT、艺术品与创作者经济</x:v>
-      </x:c>
-      <x:c r="C170" s="15" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="D170" s="16" t="d">
-        <x:v>2026-08-04T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="E170" s="14" t="str">
-        <x:v>Management Science</x:v>
-      </x:c>
-      <x:c r="F170" s="20" t="str">
-        <x:v>From Canvas to Blockchain: Impact of Royalties on Art Market Efficiency</x:v>
-      </x:c>
-      <x:c r="G170" s="20" t="str">
-        <x:v>Xinyu Cao; Jieteng Chen; T. Tony Ke</x:v>
-      </x:c>
-      <x:c r="H170" s="21" t="str">
-        <x:v>在线发表</x:v>
-      </x:c>
-      <x:c r="I170" s="20" t="str">
-        <x:v>区块链艺术品版税与市场效率</x:v>
-      </x:c>
-      <x:c r="J170" s="20" t="str">
-        <x:v>直接相关</x:v>
-      </x:c>
-      <x:c r="K170" s="20" t="str">
-        <x:v>未编入卷期</x:v>
-      </x:c>
-      <x:c r="L170" s="22" t="d">
-        <x:v>2026-08-04T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="M170" s="20" t="str">
-        <x:v>10.1287/mnsc.2023.03810</x:v>
-      </x:c>
-      <x:c r="N170" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2023.03810</x:v>
-      </x:c>
-      <x:c r="O170" s="23" t="str">
-        <x:v>打开来源</x:v>
-      </x:c>
-      <x:c r="P170" s="20" t="str"/>
-      <x:c r="Q170" s="20" t="str"/>
+      <x:c r="A170"/>
+      <x:c r="B170"/>
+      <x:c r="C170"/>
+      <x:c r="D170"/>
+      <x:c r="E170"/>
+      <x:c r="F170"/>
+      <x:c r="G170"/>
+      <x:c r="H170"/>
+      <x:c r="I170"/>
+      <x:c r="J170"/>
+      <x:c r="K170"/>
+      <x:c r="L170"/>
+      <x:c r="M170"/>
+      <x:c r="N170"/>
+      <x:c r="O170"/>
+      <x:c r="P170"/>
+      <x:c r="Q170"/>
     </x:row>
     <x:row r="171" ht="46" customHeight="1">
-      <x:c r="A171" s="12" t="str">
-        <x:v>P159</x:v>
-      </x:c>
-      <x:c r="B171" s="18" t="str">
-        <x:v>NFT、艺术品与创作者经济</x:v>
-      </x:c>
-      <x:c r="C171" s="15" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="D171" s="24" t="d">
-        <x:v>2026-09-01T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="E171" s="14" t="str">
-        <x:v>ISR</x:v>
-      </x:c>
-      <x:c r="F171" s="20" t="str">
-        <x:v>NFT Disruption in Platform Competition: Evidence from Trading Card Collectibles</x:v>
-      </x:c>
-      <x:c r="G171" s="20" t="str">
-        <x:v>Ioannis Filippos Kanellopoulos; Dominik Gutt; Ting Li</x:v>
-      </x:c>
-      <x:c r="H171" s="21" t="str">
-        <x:v>卷期发表</x:v>
-      </x:c>
-      <x:c r="I171" s="20" t="str">
-        <x:v>NFT 对收藏卡交易平台竞争的影响</x:v>
-      </x:c>
-      <x:c r="J171" s="20" t="str">
-        <x:v>直接相关</x:v>
-      </x:c>
-      <x:c r="K171" s="20" t="str">
-        <x:v>37(3): 1596-1620</x:v>
-      </x:c>
-      <x:c r="L171" s="22"/>
-      <x:c r="M171" s="20" t="str">
-        <x:v>10.1287/isre.2024.0829</x:v>
-      </x:c>
-      <x:c r="N171" s="20" t="str">
-        <x:v>https://doi.org/10.1287/isre.2024.0829</x:v>
-      </x:c>
-      <x:c r="O171" s="23" t="str">
-        <x:v>打开来源</x:v>
-      </x:c>
-      <x:c r="P171" s="20" t="str"/>
-      <x:c r="Q171" s="20" t="str"/>
+      <x:c r="A171"/>
+      <x:c r="B171"/>
+      <x:c r="C171"/>
+      <x:c r="D171"/>
+      <x:c r="E171"/>
+      <x:c r="F171"/>
+      <x:c r="G171"/>
+      <x:c r="H171"/>
+      <x:c r="I171"/>
+      <x:c r="J171"/>
+      <x:c r="K171"/>
+      <x:c r="L171"/>
+      <x:c r="M171"/>
+      <x:c r="N171"/>
+      <x:c r="O171"/>
+      <x:c r="P171"/>
+      <x:c r="Q171"/>
     </x:row>
     <x:row r="172" ht="46" customHeight="1">
-      <x:c r="A172" s="12" t="str">
-        <x:v>P160</x:v>
-      </x:c>
-      <x:c r="B172" s="18" t="str">
-        <x:v>NFT、艺术品与创作者经济</x:v>
-      </x:c>
-      <x:c r="C172" s="15" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="D172" s="24" t="d">
-        <x:v>2026-10-01T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="E172" s="14" t="str">
-        <x:v>Management Science</x:v>
-      </x:c>
-      <x:c r="F172" s="20" t="str">
-        <x:v>Chasing Market Growth and Matching Performance in Two-Sided Platforms: Evidence from the Lazy-Minting Policy in an NFT Marketplace</x:v>
-      </x:c>
-      <x:c r="G172" s="20" t="str">
-        <x:v>Hong Zhang; Hongchang Wang; Amit Mehra; Zhiqiang (Eric) Zheng</x:v>
-      </x:c>
-      <x:c r="H172" s="21" t="str">
-        <x:v>卷期发表</x:v>
-      </x:c>
-      <x:c r="I172" s="20" t="str">
-        <x:v>NFT 市场懒铸造政策、增长与匹配效率</x:v>
-      </x:c>
-      <x:c r="J172" s="20" t="str">
-        <x:v>直接相关</x:v>
-      </x:c>
-      <x:c r="K172" s="20" t="str">
-        <x:v>72(10): 8416-8439</x:v>
-      </x:c>
-      <x:c r="L172" s="22"/>
-      <x:c r="M172" s="20" t="str">
-        <x:v>10.1287/mnsc.2022.03573</x:v>
-      </x:c>
-      <x:c r="N172" s="20" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2022.03573</x:v>
-      </x:c>
-      <x:c r="O172" s="23" t="str">
-        <x:v>打开来源</x:v>
-      </x:c>
-      <x:c r="P172" s="20" t="str"/>
-      <x:c r="Q172" s="20" t="str"/>
+      <x:c r="A172"/>
+      <x:c r="B172"/>
+      <x:c r="C172"/>
+      <x:c r="D172"/>
+      <x:c r="E172"/>
+      <x:c r="F172"/>
+      <x:c r="G172"/>
+      <x:c r="H172"/>
+      <x:c r="I172"/>
+      <x:c r="J172"/>
+      <x:c r="K172"/>
+      <x:c r="L172"/>
+      <x:c r="M172"/>
+      <x:c r="N172"/>
+      <x:c r="O172"/>
+      <x:c r="P172"/>
+      <x:c r="Q172"/>
     </x:row>
     <x:row r="173" ht="46" customHeight="1">
-      <x:c r="A173" s="25" t="str">
-        <x:v>P161</x:v>
-      </x:c>
-      <x:c r="B173" s="34" t="str">
-        <x:v>综述与研究议程</x:v>
-      </x:c>
-      <x:c r="C173" s="27" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="D173" s="28" t="d">
-        <x:v>2023-11-01T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="E173" s="29" t="str">
-        <x:v>Management Science</x:v>
-      </x:c>
-      <x:c r="F173" s="30" t="str">
-        <x:v>Advances in Blockchain and Crypto Economics</x:v>
-      </x:c>
-      <x:c r="G173" s="30" t="str">
-        <x:v>Bruno Biais; Agostino Capponi; Lin William Cong; Vishal Gaur; Kay Giesecke</x:v>
-      </x:c>
-      <x:c r="H173" s="31" t="str">
-        <x:v>卷期发表</x:v>
-      </x:c>
-      <x:c r="I173" s="30" t="str">
-        <x:v>区块链与加密经济学专辑导论及研究议程</x:v>
-      </x:c>
-      <x:c r="J173" s="30" t="str">
-        <x:v>综述导论</x:v>
-      </x:c>
-      <x:c r="K173" s="30" t="str">
-        <x:v>69(11): 6417-6426</x:v>
-      </x:c>
-      <x:c r="L173" s="32"/>
-      <x:c r="M173" s="30" t="str">
-        <x:v>10.1287/mnsc.2023.intro.v69.n11</x:v>
-      </x:c>
-      <x:c r="N173" s="30" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2023.intro.v69.n11</x:v>
-      </x:c>
-      <x:c r="O173" s="33" t="str">
-        <x:v>打开来源</x:v>
-      </x:c>
-      <x:c r="P173" s="30" t="str"/>
-      <x:c r="Q173" s="30" t="str"/>
+      <x:c r="A173"/>
+      <x:c r="B173"/>
+      <x:c r="C173"/>
+      <x:c r="D173"/>
+      <x:c r="E173"/>
+      <x:c r="F173"/>
+      <x:c r="G173"/>
+      <x:c r="H173"/>
+      <x:c r="I173"/>
+      <x:c r="J173"/>
+      <x:c r="K173"/>
+      <x:c r="L173"/>
+      <x:c r="M173"/>
+      <x:c r="N173"/>
+      <x:c r="O173"/>
+      <x:c r="P173"/>
+      <x:c r="Q173"/>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="H6:H173">
-    <x:cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="已接收"/>
+  <x:conditionalFormatting sqref="H6:H164">
+    <x:cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="已接收"/>
   </x:conditionalFormatting>
   <x:hyperlinks>
-    <x:hyperlink ref="O6" r:id="Hyperlink6" display="打开来源"/>
-    <x:hyperlink ref="O7" r:id="Hyperlink7" display="打开来源"/>
-    <x:hyperlink ref="O8" r:id="Hyperlink8" display="打开来源"/>
-    <x:hyperlink ref="O9" r:id="Hyperlink9" display="打开来源"/>
-    <x:hyperlink ref="O10" r:id="Hyperlink10" display="打开来源"/>
-    <x:hyperlink ref="O11" r:id="Hyperlink11" display="打开来源"/>
-    <x:hyperlink ref="O12" r:id="Hyperlink12" display="打开来源"/>
-    <x:hyperlink ref="O13" r:id="Hyperlink13" display="打开来源"/>
-    <x:hyperlink ref="O14" r:id="Hyperlink14" display="打开来源"/>
-    <x:hyperlink ref="O15" r:id="Hyperlink15" display="打开来源"/>
-    <x:hyperlink ref="O16" r:id="Hyperlink16" display="打开来源"/>
-    <x:hyperlink ref="O17" r:id="Hyperlink17" display="打开来源"/>
-    <x:hyperlink ref="O18" r:id="Hyperlink18" display="打开来源"/>
-    <x:hyperlink ref="O19" r:id="Hyperlink19" display="打开来源"/>
-    <x:hyperlink ref="O20" r:id="Hyperlink20" display="打开来源"/>
-    <x:hyperlink ref="O21" r:id="Hyperlink21" display="打开来源"/>
-    <x:hyperlink ref="O22" r:id="Hyperlink22" display="打开来源"/>
-    <x:hyperlink ref="O23" r:id="Hyperlink23" display="打开来源"/>
-    <x:hyperlink ref="O24" r:id="Hyperlink24" display="打开来源"/>
-    <x:hyperlink ref="O25" r:id="Hyperlink25" display="打开来源"/>
-    <x:hyperlink ref="O26" r:id="Hyperlink26" display="打开来源"/>
-    <x:hyperlink ref="O27" r:id="Hyperlink27" display="打开来源"/>
-    <x:hyperlink ref="O28" r:id="Hyperlink28" display="打开来源"/>
-    <x:hyperlink ref="O29" r:id="Hyperlink29" display="打开来源"/>
-    <x:hyperlink ref="O30" r:id="Hyperlink30" display="打开来源"/>
-    <x:hyperlink ref="O31" r:id="Hyperlink31" display="打开来源"/>
-    <x:hyperlink ref="O32" r:id="Hyperlink32" display="打开来源"/>
-    <x:hyperlink ref="O33" r:id="Hyperlink33" display="打开来源"/>
-    <x:hyperlink ref="O34" r:id="Hyperlink34" display="打开来源"/>
-    <x:hyperlink ref="O35" r:id="Hyperlink35" display="打开来源"/>
-    <x:hyperlink ref="O36" r:id="Hyperlink36" display="打开来源"/>
-    <x:hyperlink ref="O37" r:id="Hyperlink37" display="打开来源"/>
-    <x:hyperlink ref="O38" r:id="Hyperlink38" display="打开来源"/>
-    <x:hyperlink ref="O39" r:id="Hyperlink39" display="打开来源"/>
-    <x:hyperlink ref="O40" r:id="Hyperlink40" display="打开来源"/>
-    <x:hyperlink ref="O41" r:id="Hyperlink41" display="打开来源"/>
-    <x:hyperlink ref="O42" r:id="Hyperlink42" display="打开来源"/>
-    <x:hyperlink ref="O43" r:id="Hyperlink43" display="打开来源"/>
-    <x:hyperlink ref="O44" r:id="Hyperlink44" display="打开来源"/>
-    <x:hyperlink ref="O45" r:id="Hyperlink45" display="打开来源"/>
-    <x:hyperlink ref="O46" r:id="Hyperlink46" display="打开来源"/>
-    <x:hyperlink ref="O47" r:id="Hyperlink47" display="打开来源"/>
-    <x:hyperlink ref="O48" r:id="Hyperlink48" display="打开来源"/>
-    <x:hyperlink ref="O49" r:id="Hyperlink49" display="打开来源"/>
-    <x:hyperlink ref="O50" r:id="Hyperlink50" display="打开来源"/>
-    <x:hyperlink ref="O51" r:id="Hyperlink51" display="打开来源"/>
-    <x:hyperlink ref="O52" r:id="Hyperlink52" display="打开来源"/>
-    <x:hyperlink ref="O53" r:id="Hyperlink53" display="打开来源"/>
-    <x:hyperlink ref="O54" r:id="Hyperlink54" display="打开来源"/>
-    <x:hyperlink ref="O55" r:id="Hyperlink55" display="打开来源"/>
-    <x:hyperlink ref="O56" r:id="Hyperlink56" display="打开来源"/>
-    <x:hyperlink ref="O57" r:id="Hyperlink57" display="打开来源"/>
-    <x:hyperlink ref="O58" r:id="Hyperlink58" display="打开来源"/>
-    <x:hyperlink ref="O59" r:id="Hyperlink59" display="打开来源"/>
-    <x:hyperlink ref="O60" r:id="Hyperlink60" display="打开来源"/>
-    <x:hyperlink ref="O61" r:id="Hyperlink61" display="打开来源"/>
-    <x:hyperlink ref="O62" r:id="Hyperlink62" display="打开来源"/>
-    <x:hyperlink ref="O63" r:id="Hyperlink63" display="打开来源"/>
-    <x:hyperlink ref="O64" r:id="Hyperlink64" display="打开来源"/>
-    <x:hyperlink ref="O65" r:id="Hyperlink65" display="打开来源"/>
-    <x:hyperlink ref="O66" r:id="Hyperlink66" display="打开来源"/>
-    <x:hyperlink ref="O67" r:id="Hyperlink67" display="打开来源"/>
-    <x:hyperlink ref="O68" r:id="Hyperlink68" display="打开来源"/>
-    <x:hyperlink ref="O69" r:id="Hyperlink69" display="打开来源"/>
-    <x:hyperlink ref="O70" r:id="Hyperlink70" display="打开来源"/>
-    <x:hyperlink ref="O71" r:id="Hyperlink71" display="打开来源"/>
-    <x:hyperlink ref="O72" r:id="Hyperlink72" display="打开来源"/>
-    <x:hyperlink ref="O73" r:id="Hyperlink73" display="打开来源"/>
-    <x:hyperlink ref="O74" r:id="Hyperlink74" display="打开来源"/>
-    <x:hyperlink ref="O75" r:id="Hyperlink75" display="打开来源"/>
-    <x:hyperlink ref="O76" r:id="Hyperlink76" display="打开来源"/>
-    <x:hyperlink ref="O77" r:id="Hyperlink77" display="打开来源"/>
-    <x:hyperlink ref="O78" r:id="Hyperlink78" display="打开来源"/>
-    <x:hyperlink ref="O79" r:id="Hyperlink79" display="打开来源"/>
-    <x:hyperlink ref="O80" r:id="Hyperlink80" display="打开来源"/>
-    <x:hyperlink ref="O81" r:id="Hyperlink81" display="打开来源"/>
-    <x:hyperlink ref="O82" r:id="Hyperlink82" display="打开来源"/>
-    <x:hyperlink ref="O83" r:id="Hyperlink83" display="打开来源"/>
-    <x:hyperlink ref="O84" r:id="Hyperlink84" display="打开来源"/>
-    <x:hyperlink ref="O85" r:id="Hyperlink85" display="打开来源"/>
-    <x:hyperlink ref="O86" r:id="Hyperlink86" display="打开来源"/>
-    <x:hyperlink ref="O87" r:id="Hyperlink87" display="打开来源"/>
-    <x:hyperlink ref="O88" r:id="Hyperlink88" display="打开来源"/>
-    <x:hyperlink ref="O89" r:id="Hyperlink89" display="打开来源"/>
-    <x:hyperlink ref="O90" r:id="Hyperlink90" display="打开来源"/>
-    <x:hyperlink ref="O91" r:id="Hyperlink91" display="打开来源"/>
-    <x:hyperlink ref="O92" r:id="Hyperlink92" display="打开来源"/>
-    <x:hyperlink ref="O93" r:id="Hyperlink93" display="打开来源"/>
-    <x:hyperlink ref="O94" r:id="Hyperlink94" display="打开来源"/>
-    <x:hyperlink ref="O95" r:id="Hyperlink95" display="打开来源"/>
-    <x:hyperlink ref="O96" r:id="Hyperlink96" display="打开来源"/>
-    <x:hyperlink ref="O97" r:id="Hyperlink97" display="打开来源"/>
-    <x:hyperlink ref="O98" r:id="Hyperlink98" display="打开来源"/>
-    <x:hyperlink ref="O99" r:id="Hyperlink99" display="打开来源"/>
-    <x:hyperlink ref="O100" r:id="Hyperlink100" display="打开来源"/>
-    <x:hyperlink ref="O101" r:id="Hyperlink101" display="打开来源"/>
-    <x:hyperlink ref="O102" r:id="Hyperlink102" display="打开来源"/>
-    <x:hyperlink ref="O103" r:id="Hyperlink103" display="打开来源"/>
-    <x:hyperlink ref="O104" r:id="Hyperlink104" display="打开来源"/>
-    <x:hyperlink ref="O105" r:id="Hyperlink105" display="打开来源"/>
-    <x:hyperlink ref="O106" r:id="Hyperlink106" display="打开来源"/>
-    <x:hyperlink ref="O107" r:id="Hyperlink107" display="打开来源"/>
-    <x:hyperlink ref="O108" r:id="Hyperlink108" display="打开来源"/>
-    <x:hyperlink ref="O109" r:id="Hyperlink109" display="打开来源"/>
-    <x:hyperlink ref="O110" r:id="Hyperlink110" display="打开来源"/>
-    <x:hyperlink ref="O111" r:id="Hyperlink111" display="打开来源"/>
-    <x:hyperlink ref="O112" r:id="Hyperlink112" display="打开来源"/>
-    <x:hyperlink ref="O113" r:id="Hyperlink113" display="打开来源"/>
-    <x:hyperlink ref="O114" r:id="Hyperlink114" display="打开来源"/>
-    <x:hyperlink ref="O115" r:id="Hyperlink115" display="打开来源"/>
-    <x:hyperlink ref="O116" r:id="Hyperlink116" display="打开来源"/>
-    <x:hyperlink ref="O117" r:id="Hyperlink117" display="打开来源"/>
-    <x:hyperlink ref="O118" r:id="Hyperlink118" display="打开来源"/>
-    <x:hyperlink ref="O119" r:id="Hyperlink119" display="打开来源"/>
-    <x:hyperlink ref="O120" r:id="Hyperlink120" display="打开来源"/>
-    <x:hyperlink ref="O121" r:id="Hyperlink121" display="打开来源"/>
-    <x:hyperlink ref="O122" r:id="Hyperlink122" display="打开来源"/>
-    <x:hyperlink ref="O123" r:id="Hyperlink123" display="打开来源"/>
-    <x:hyperlink ref="O124" r:id="Hyperlink124" display="打开来源"/>
-    <x:hyperlink ref="O125" r:id="Hyperlink125" display="打开来源"/>
-    <x:hyperlink ref="O126" r:id="Hyperlink126" display="打开来源"/>
-    <x:hyperlink ref="O127" r:id="Hyperlink127" display="打开来源"/>
-    <x:hyperlink ref="O128" r:id="Hyperlink128" display="打开来源"/>
-    <x:hyperlink ref="O129" r:id="Hyperlink129" display="打开来源"/>
-    <x:hyperlink ref="O130" r:id="Hyperlink130" display="打开来源"/>
-    <x:hyperlink ref="O131" r:id="Hyperlink131" display="打开来源"/>
-    <x:hyperlink ref="O132" r:id="Hyperlink132" display="打开来源"/>
-    <x:hyperlink ref="O133" r:id="Hyperlink133" display="打开来源"/>
-    <x:hyperlink ref="O134" r:id="Hyperlink134" display="打开来源"/>
-    <x:hyperlink ref="O135" r:id="Hyperlink135" display="打开来源"/>
-    <x:hyperlink ref="O136" r:id="Hyperlink136" display="打开来源"/>
-    <x:hyperlink ref="O137" r:id="Hyperlink137" display="打开来源"/>
-    <x:hyperlink ref="O138" r:id="Hyperlink138" display="打开来源"/>
-    <x:hyperlink ref="O139" r:id="Hyperlink139" display="打开来源"/>
-    <x:hyperlink ref="O140" r:id="Hyperlink140" display="打开来源"/>
-    <x:hyperlink ref="O141" r:id="Hyperlink141" display="打开来源"/>
-    <x:hyperlink ref="O142" r:id="Hyperlink142" display="打开来源"/>
-    <x:hyperlink ref="O143" r:id="Hyperlink143" display="打开来源"/>
-    <x:hyperlink ref="O144" r:id="Hyperlink144" display="打开来源"/>
-    <x:hyperlink ref="O145" r:id="Hyperlink145" display="打开来源"/>
-    <x:hyperlink ref="O146" r:id="Hyperlink146" display="打开来源"/>
-    <x:hyperlink ref="O147" r:id="Hyperlink147" display="打开来源"/>
-    <x:hyperlink ref="O148" r:id="Hyperlink148" display="打开来源"/>
-    <x:hyperlink ref="O149" r:id="Hyperlink149" display="打开来源"/>
-    <x:hyperlink ref="O150" r:id="Hyperlink150" display="打开来源"/>
-    <x:hyperlink ref="O151" r:id="Hyperlink151" display="打开来源"/>
-    <x:hyperlink ref="O152" r:id="Hyperlink152" display="打开来源"/>
-    <x:hyperlink ref="O153" r:id="Hyperlink153" display="打开来源"/>
-    <x:hyperlink ref="O154" r:id="Hyperlink154" display="打开来源"/>
-    <x:hyperlink ref="O155" r:id="Hyperlink155" display="打开来源"/>
-    <x:hyperlink ref="O156" r:id="Hyperlink156" display="打开来源"/>
-    <x:hyperlink ref="O157" r:id="Hyperlink157" display="打开来源"/>
-    <x:hyperlink ref="O158" r:id="Hyperlink158" display="打开来源"/>
-    <x:hyperlink ref="O159" r:id="Hyperlink159" display="打开来源"/>
-    <x:hyperlink ref="O160" r:id="Hyperlink160" display="打开来源"/>
-    <x:hyperlink ref="O161" r:id="Hyperlink161" display="打开来源"/>
-    <x:hyperlink ref="O162" r:id="Hyperlink162" display="打开来源"/>
-    <x:hyperlink ref="O163" r:id="Hyperlink163" display="打开来源"/>
-    <x:hyperlink ref="O164" r:id="Hyperlink164" display="打开来源"/>
-    <x:hyperlink ref="O165" r:id="Hyperlink165" display="打开来源"/>
-    <x:hyperlink ref="O166" r:id="Hyperlink166" display="打开来源"/>
-    <x:hyperlink ref="O167" r:id="Hyperlink167" display="打开来源"/>
-    <x:hyperlink ref="O168" r:id="Hyperlink168" display="打开来源"/>
-    <x:hyperlink ref="O169" r:id="Hyperlink169" display="打开来源"/>
-    <x:hyperlink ref="O170" r:id="Hyperlink170" display="打开来源"/>
-    <x:hyperlink ref="O171" r:id="Hyperlink171" display="打开来源"/>
-    <x:hyperlink ref="O172" r:id="Hyperlink172" display="打开来源"/>
-    <x:hyperlink ref="O173" r:id="Hyperlink173" display="打开来源"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="R0032502370de4844"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="Rfcf79657202d477c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="R759ac2de33ef426f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="R19d01ef0905746be"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="Rc7e1456b8c3c4cf2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="R5bd1fdb310174ece"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="R4dce7b3f41f34dea"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="Rc38d96a2439b464c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="Rc9765b31d3374d31"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="Rec10f92286b34c78"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="R7e11644c8a72456a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="Rafb6b3b0f0ea4161"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="R6657c75014fe4de4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="Rbe5a6a42c649426d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="Rc1f96cea6f8a422d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="R0fdc3fce5aca4aa9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="R6599b273bfce4cf2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="R4ad76894b6314abd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="R02e9e1e41f004fdd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="R02b586b9398946e0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="R26ac68f8590b43c1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="Rae9709d217c749cf"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="Re33277d3385a43b5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="R4a0ad48282a6464b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="R42c416e7811a4a5a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="Rdbfb778ee0444892"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="Rf90c63f4965c406d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="R08554ba32a3c4c53"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="R9b06dd44daab4b0a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="Rca41c1bb3df0463e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="R0887c76c2d684c08"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R270f5975a5f74aa2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="R9aab54b28483498a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="R6b6136d677814cda"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="Rb1c78125cf0d4e9d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="R802895422c67447f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="R3a88b805313e4a17"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="R1ad2826d130646d6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="Re0c3d0e0c5d14936"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="Rda064c320ac64ec8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="Rc1e9f3fb79354dbb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="Rff8a3a60a89c4a1e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="R4bc2cbc8e2114cae"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="R11d9e88e3ba040ed"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="R838aca71617a4d0f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="R4627359cf6e74691"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="R2c539f56da6f42fe"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="R6e1fdbf7a4fb4d17"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="R8ec9016bb2214c1a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="Rdf5c8cc2342f4d0b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="R5e6dcabb7c1c431e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="R74df36cfa4b14617"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="R13580e779b3c416e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="R43b752da7cf7412d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="R36220586031245d0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="Rb5d626ed5c0d4f4f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="R1753757c3bd145da"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="Rfb763df51e5340c6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="R4446855b8a2740c9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="Rb980621eb52740cc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="R1545057608134f07"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="R4d23c08b2a694a48"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="R7269bbeb60a34819"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="R74a758836ee84c38"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="R4193bfc855144fc5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="R4dd8f23f7cc94946"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="Rfd16d30f05374584"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="Rbe35f205929b4a99"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="R902ba9f911a7420c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="Rdc811dcd3bf74d2e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R4b829876ba8449c7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="Rbbdc2534bfb94228"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="R9772d372f20c4fcc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="R3b330a5df3ae4712"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="R20348866e1194d1c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="R351ff9de5fcf468c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="Red584546007f4018"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="R083bea7a3a914a93"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O84" r:id="R6e80aa1e3dc3432a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="R622307ca733d466c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O86" r:id="R40fc79cae90f4b88"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O87" r:id="Rdc31e81ea443409a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="R5cf47363e3864d7f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="Rd1a8c617ab034dcd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="R063b7899d33c4d55"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O91" r:id="R058705042c024252"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="R5335b1e007e4464f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O93" r:id="R81f56300cf284b99"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="R39c25b17f6774b19"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="R95c50bbfa8b54f1c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="R29b91fb29fde47a4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="R7771ded0937c4f4a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O98" r:id="R04e5608fe6214795"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O99" r:id="Rcc6478524c2d4029"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O100" r:id="R21bcf51842854273"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O101" r:id="R098279b453f94a0f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O102" r:id="R8ab01b644a4248f7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="Re7a25f3321d64e47"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O104" r:id="R1edc244a0e974f26"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O105" r:id="Rba9c397808bb408f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O106" r:id="R0d6bb21457b44dc3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="Rade44c94306c4b2c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="Re55ee6d369624729"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="Rf48a4215165640a7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="R5c32cf4dd90a4807"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O111" r:id="R472d0c5e04294c8f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="Rc9b03af1bfa9402a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O113" r:id="R647d22c6f58c49af"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O114" r:id="R4054b7f5d96048d4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O115" r:id="R1587ec727c5e4d22"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O116" r:id="Rf186ca06fe0640eb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O117" r:id="R10700acfdc724150"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O118" r:id="Rce1bc01bfaad4b2f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O119" r:id="R50097ff9b06c46a0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O120" r:id="Rfce60c5d107e4b1d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O121" r:id="Rd568b4e72eb44398"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O122" r:id="R426772c757da41b6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O123" r:id="R12598c77fe2b4ba0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O124" r:id="R06466a318a1f4398"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O125" r:id="Rf6f3a9d304e84b87"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O126" r:id="R01332a9916ef4323"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O127" r:id="Rb6ef7c2296c84e00"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O128" r:id="R170aaf849f1242a7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O129" r:id="Re3daff041aa24091"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O130" r:id="R80f3d4dd616a4d73"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O131" r:id="Rfaec359dec674b01"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O132" r:id="Ra945998a00fe48b9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O133" r:id="Rd6f53c8acd8246a9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O134" r:id="Re322468675204d37"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O135" r:id="R83659a5341ff4687"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O136" r:id="R7d3ff662df024489"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O137" r:id="R9a685661f58344e6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O138" r:id="Rca409d10c755470a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O139" r:id="R5c037aed18b4496a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O140" r:id="R9adc8aec95d449a1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O141" r:id="R8d36d99343f841ed"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O142" r:id="R58de40c2935446c9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O143" r:id="R9ea1a5e55e014337"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O144" r:id="R06f9311490b54a67"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O145" r:id="R72e0510fc1804d83"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O146" r:id="R3c7f4359ea9c4c9f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O147" r:id="R2562c6eeb7f744a4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O148" r:id="Rd0bc32363baf4d46"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O149" r:id="R1e9adc4ba1e64b0e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O150" r:id="Rfbabb838209445d1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O151" r:id="R73ebe3ed76b149e7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O152" r:id="R89ec6ac0341f41da"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O153" r:id="R8958259c340946b0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O154" r:id="R8df21850d0614e91"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O155" r:id="R9a95a678498f4ce7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O156" r:id="R42a91f6adc214813"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O157" r:id="R07ca6c2a69a14e6a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O158" r:id="Rbd661bd102314f11"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O159" r:id="R916b727d48d7469a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O160" r:id="R81e43bcda2aa442c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O161" r:id="Rad349442393745ed"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O162" r:id="R1de1f4e1e1d3414a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O163" r:id="Rb9de5d0f1c4a4d98"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O164" r:id="R31bbf6803d3f4795"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O165" r:id="R21d204e5f7674b91"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O166" r:id="Rf947e37218be4f70"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O167" r:id="R7cd0952ae21c489d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O168" r:id="Rbbe691148c0c4b42"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O169" r:id="R452dbd695d0a4ff2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O170" r:id="R693a465ed1844c3f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O171" r:id="R4a7b88400662409f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O172" r:id="R0d4806aa8cff41c9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O173" r:id="Rc396b978209148a8"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart r:id="R5288ea5c385540f8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0c388c11ac743e1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr>
     <x:tabColor rgb="FF8494A5"/>
   </x:sheetPr>
@@ -10551,7 +10281,7 @@
     </x:row>
     <x:row r="15" ht="46" customHeight="1">
       <x:c r="A15" s="12" t="str">
-        <x:v>R06</x:v>
+        <x:v>R07</x:v>
       </x:c>
       <x:c r="B15" s="18" t="str">
         <x:v>综述与研究议程</x:v>
@@ -10563,34 +10293,32 @@
         <x:v>2025-11-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E15" s="14" t="str">
-        <x:v>TAR</x:v>
+        <x:v>JME</x:v>
       </x:c>
       <x:c r="F15" s="20" t="str">
-        <x:v>Innovative Capital Markets Research and Accounting Practitioners</x:v>
+        <x:v>“Information frictions in macroeconomics: The legacy of Robert E. Lucas, Jr.”</x:v>
       </x:c>
       <x:c r="G15" s="20" t="str">
-        <x:v>Carolyn M. Callahan</x:v>
+        <x:v>Robert M. Townsend</x:v>
       </x:c>
       <x:c r="H15" s="21" t="str">
         <x:v>卷期发表</x:v>
       </x:c>
       <x:c r="I15" s="20" t="str">
-        <x:v>面向实务的会计研究议程，其中包括加密和数字资产</x:v>
+        <x:v>宏观信息摩擦综述，专门讨论分布式账本与可编程数字资产</x:v>
       </x:c>
       <x:c r="J15" s="20" t="str">
         <x:v>相关综述</x:v>
       </x:c>
       <x:c r="K15" s="20" t="str">
-        <x:v>100(6): 419-430</x:v>
-      </x:c>
-      <x:c r="L15" s="22" t="d">
-        <x:v>2025-10-17T00:00:00.000Z</x:v>
-      </x:c>
+        <x:v>155: 103842</x:v>
+      </x:c>
+      <x:c r="L15" s="22"/>
       <x:c r="M15" s="20" t="str">
-        <x:v>10.2308/tar-2025-0273</x:v>
+        <x:v>10.1016/j.jmoneco.2025.103842</x:v>
       </x:c>
       <x:c r="N15" s="20" t="str">
-        <x:v>https://doi.org/10.2308/tar-2025-0273</x:v>
+        <x:v>https://doi.org/10.1016/j.jmoneco.2025.103842</x:v>
       </x:c>
       <x:c r="O15" s="23" t="str">
         <x:v>打开来源</x:v>
@@ -10599,72 +10327,44 @@
       <x:c r="Q15" s="20" t="str"/>
     </x:row>
     <x:row r="16" ht="46" customHeight="1">
-      <x:c r="A16" s="12" t="str">
-        <x:v>R07</x:v>
-      </x:c>
-      <x:c r="B16" s="18" t="str">
-        <x:v>综述与研究议程</x:v>
-      </x:c>
-      <x:c r="C16" s="15" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="D16" s="24" t="d">
-        <x:v>2025-11-01T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="E16" s="14" t="str">
-        <x:v>JME</x:v>
-      </x:c>
-      <x:c r="F16" s="20" t="str">
-        <x:v>“Information frictions in macroeconomics: The legacy of Robert E. Lucas, Jr.”</x:v>
-      </x:c>
-      <x:c r="G16" s="20" t="str">
-        <x:v>Robert M. Townsend</x:v>
-      </x:c>
-      <x:c r="H16" s="21" t="str">
-        <x:v>卷期发表</x:v>
-      </x:c>
-      <x:c r="I16" s="20" t="str">
-        <x:v>宏观信息摩擦综述，专门讨论分布式账本与可编程数字资产</x:v>
-      </x:c>
-      <x:c r="J16" s="20" t="str">
-        <x:v>相关综述</x:v>
-      </x:c>
-      <x:c r="K16" s="20" t="str">
-        <x:v>155: 103842</x:v>
-      </x:c>
-      <x:c r="L16" s="22"/>
-      <x:c r="M16" s="20" t="str">
-        <x:v>10.1016/j.jmoneco.2025.103842</x:v>
-      </x:c>
-      <x:c r="N16" s="20" t="str">
-        <x:v>https://doi.org/10.1016/j.jmoneco.2025.103842</x:v>
-      </x:c>
-      <x:c r="O16" s="23" t="str">
-        <x:v>打开来源</x:v>
-      </x:c>
-      <x:c r="P16" s="20" t="str"/>
-      <x:c r="Q16" s="20" t="str"/>
+      <x:c r="A16"/>
+      <x:c r="B16"/>
+      <x:c r="C16"/>
+      <x:c r="D16"/>
+      <x:c r="E16"/>
+      <x:c r="F16"/>
+      <x:c r="G16"/>
+      <x:c r="H16"/>
+      <x:c r="I16"/>
+      <x:c r="J16"/>
+      <x:c r="K16"/>
+      <x:c r="L16"/>
+      <x:c r="M16"/>
+      <x:c r="N16"/>
+      <x:c r="O16"/>
+      <x:c r="P16"/>
+      <x:c r="Q16"/>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="H6:H16">
-    <x:cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="已接收"/>
+  <x:conditionalFormatting sqref="H6:H15">
+    <x:cfRule type="containsText" dxfId="7" priority="1" operator="containsText" text="已接收"/>
   </x:conditionalFormatting>
   <x:hyperlinks>
-    <x:hyperlink ref="O6" r:id="Hyperlink6" display="打开来源"/>
-    <x:hyperlink ref="O7" r:id="Hyperlink7" display="打开来源"/>
-    <x:hyperlink ref="O8" r:id="Hyperlink8" display="打开来源"/>
-    <x:hyperlink ref="O9" r:id="Hyperlink9" display="打开来源"/>
-    <x:hyperlink ref="O10" r:id="Hyperlink10" display="打开来源"/>
-    <x:hyperlink ref="O11" r:id="Hyperlink11" display="打开来源"/>
-    <x:hyperlink ref="O12" r:id="Hyperlink12" display="打开来源"/>
-    <x:hyperlink ref="O13" r:id="Hyperlink13" display="打开来源"/>
-    <x:hyperlink ref="O14" r:id="Hyperlink14" display="打开来源"/>
-    <x:hyperlink ref="O15" r:id="Hyperlink15" display="打开来源"/>
-    <x:hyperlink ref="O16" r:id="Hyperlink16" display="打开来源"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="R5fe69c1abb9d4996"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="Re4b020b889ef42e4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="R7417be96c7d946d6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="R9ea4febbca5f41f3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="R2d16cbc49d684335"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="R5a5041bb12364b25"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="R4db56dc8e40b40db"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="R2af387d0c0494c12"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="R587dbc1689b3493d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="R010be20e92984fef"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="Rc87f3b9fe0f2475f"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart r:id="R625a90e6e01e4a1d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6253f285e9b94858"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>